<commit_message>
[PROGRAMMER] implement weapon part shop and loadout
</commit_message>
<xml_diff>
--- a/Design/Data/ReEchoData.xlsx
+++ b/Design/Data/ReEchoData.xlsx
@@ -510,9 +510,9 @@
 </file>
 
 <file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="12" name="tblParts" displayName="tblParts" ref="A45:N123" headerRowCount="1">
-  <autoFilter ref="A45:N123"/>
-  <tableColumns count="14">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="12" name="tblParts" displayName="tblParts" ref="A45:P123" headerRowCount="1">
+  <autoFilter ref="A45:P123"/>
+  <tableColumns count="16">
     <tableColumn id="1" name="Id"/>
     <tableColumn id="2" name="PartId"/>
     <tableColumn id="3" name="WeaponTypeId"/>
@@ -527,14 +527,16 @@
     <tableColumn id="12" name="DisabledReason"/>
     <tableColumn id="13" name="SourceSheet"/>
     <tableColumn id="14" name="SourceRow"/>
+    <tableColumn id="15" name="ShopEnabled"/>
+    <tableColumn id="16" name="ShopPrice"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table13.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="13" name="tblPartEffects" displayName="tblPartEffects" ref="P45:AI55" headerRowCount="1">
-  <autoFilter ref="P45:AI55"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="13" name="tblPartEffects" displayName="tblPartEffects" ref="R45:AK55" headerRowCount="1">
+  <autoFilter ref="R45:AK55"/>
   <tableColumns count="20">
     <tableColumn id="16" name="Id"/>
     <tableColumn id="17" name="PartId"/>
@@ -16324,12 +16326,12 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AI123"/>
+  <dimension ref="A1:AK123"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="13.81640625" defaultRowHeight="13"/>
   <cols>
     <col width="25" customWidth="1" style="32" min="1" max="1"/>
@@ -16346,26 +16348,28 @@
     <col width="40" customWidth="1" style="32" min="12" max="12"/>
     <col width="18" customWidth="1" style="32" min="13" max="13"/>
     <col width="16" customWidth="1" style="32" min="14" max="14"/>
-    <col width="25" customWidth="1" style="32" min="16" max="16"/>
-    <col width="25" customWidth="1" style="32" min="17" max="17"/>
-    <col width="16" customWidth="1" style="32" min="18" max="18"/>
-    <col width="16" customWidth="1" style="32" min="19" max="19"/>
+    <col width="14" customWidth="1" style="32" min="15" max="15"/>
+    <col width="11" customWidth="1" style="32" min="16" max="16"/>
+    <col width="25" customWidth="1" style="32" min="18" max="18"/>
+    <col width="25" customWidth="1" style="32" min="19" max="19"/>
     <col width="16" customWidth="1" style="32" min="20" max="20"/>
     <col width="16" customWidth="1" style="32" min="21" max="21"/>
     <col width="16" customWidth="1" style="32" min="22" max="22"/>
     <col width="16" customWidth="1" style="32" min="23" max="23"/>
-    <col width="25" customWidth="1" style="32" min="24" max="24"/>
-    <col width="25" customWidth="1" style="32" min="25" max="25"/>
+    <col width="16" customWidth="1" style="32" min="24" max="24"/>
+    <col width="16" customWidth="1" style="32" min="25" max="25"/>
     <col width="25" customWidth="1" style="32" min="26" max="26"/>
-    <col width="16" customWidth="1" style="32" min="27" max="27"/>
-    <col width="16" customWidth="1" style="32" min="28" max="28"/>
+    <col width="25" customWidth="1" style="32" min="27" max="27"/>
+    <col width="25" customWidth="1" style="32" min="28" max="28"/>
     <col width="16" customWidth="1" style="32" min="29" max="29"/>
     <col width="16" customWidth="1" style="32" min="30" max="30"/>
     <col width="16" customWidth="1" style="32" min="31" max="31"/>
     <col width="16" customWidth="1" style="32" min="32" max="32"/>
-    <col width="40" customWidth="1" style="32" min="33" max="33"/>
-    <col width="18" customWidth="1" style="32" min="34" max="34"/>
-    <col width="16" customWidth="1" style="32" min="35" max="35"/>
+    <col width="16" customWidth="1" style="32" min="33" max="33"/>
+    <col width="16" customWidth="1" style="32" min="34" max="34"/>
+    <col width="40" customWidth="1" style="32" min="35" max="35"/>
+    <col width="18" customWidth="1" style="32" min="36" max="36"/>
+    <col width="16" customWidth="1" style="32" min="37" max="37"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1" s="32">
@@ -17713,7 +17717,7 @@
           <t>tblParts → parts.csv</t>
         </is>
       </c>
-      <c r="P44" s="34" t="inlineStr">
+      <c r="R44" s="34" t="inlineStr">
         <is>
           <t>tblPartEffects → part_effects.csv</t>
         </is>
@@ -17790,102 +17794,112 @@
           <t>SourceRow</t>
         </is>
       </c>
-      <c r="P45" s="29" t="inlineStr">
+      <c r="O45" t="inlineStr" s="29">
+        <is>
+          <t xml:space="preserve">ShopEnabled</t>
+        </is>
+      </c>
+      <c r="P45" t="inlineStr" s="29">
+        <is>
+          <t xml:space="preserve">ShopPrice</t>
+        </is>
+      </c>
+      <c r="R45" s="29" t="inlineStr">
         <is>
           <t>Id</t>
         </is>
       </c>
-      <c r="Q45" s="29" t="inlineStr">
+      <c r="S45" s="29" t="inlineStr">
         <is>
           <t>PartId</t>
         </is>
       </c>
-      <c r="R45" s="29" t="inlineStr">
+      <c r="T45" s="29" t="inlineStr">
         <is>
           <t>Order</t>
         </is>
       </c>
-      <c r="S45" s="29" t="inlineStr">
+      <c r="U45" s="29" t="inlineStr">
         <is>
           <t>Trigger</t>
         </is>
       </c>
-      <c r="T45" s="29" t="inlineStr">
+      <c r="V45" s="29" t="inlineStr">
         <is>
           <t>EffectKind</t>
         </is>
       </c>
-      <c r="U45" s="29" t="inlineStr">
+      <c r="W45" s="29" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
       </c>
-      <c r="V45" s="29" t="inlineStr">
+      <c r="X45" s="29" t="inlineStr">
         <is>
           <t>ValueOp</t>
         </is>
       </c>
-      <c r="W45" s="29" t="inlineStr">
+      <c r="Y45" s="29" t="inlineStr">
         <is>
           <t>Value</t>
         </is>
       </c>
-      <c r="X45" s="29" t="inlineStr">
+      <c r="Z45" s="29" t="inlineStr">
         <is>
           <t>BehaviorId</t>
         </is>
       </c>
-      <c r="Y45" s="29" t="inlineStr">
+      <c r="AA45" s="29" t="inlineStr">
         <is>
           <t>FormulaId</t>
         </is>
       </c>
-      <c r="Z45" s="29" t="inlineStr">
+      <c r="AB45" s="29" t="inlineStr">
         <is>
           <t>AttackPatternId</t>
         </is>
       </c>
-      <c r="AA45" s="29" t="inlineStr">
+      <c r="AC45" s="29" t="inlineStr">
         <is>
           <t>ParamName</t>
         </is>
       </c>
-      <c r="AB45" s="29" t="inlineStr">
+      <c r="AD45" s="29" t="inlineStr">
         <is>
           <t>ParamValue</t>
         </is>
       </c>
-      <c r="AC45" s="29" t="inlineStr">
+      <c r="AE45" s="29" t="inlineStr">
         <is>
           <t>DurationSeconds</t>
         </is>
       </c>
-      <c r="AD45" s="29" t="inlineStr">
+      <c r="AF45" s="29" t="inlineStr">
         <is>
           <t>CooldownSeconds</t>
         </is>
       </c>
-      <c r="AE45" s="29" t="inlineStr">
+      <c r="AG45" s="29" t="inlineStr">
         <is>
           <t>StackPolicy</t>
         </is>
       </c>
-      <c r="AF45" s="29" t="inlineStr">
+      <c r="AH45" s="29" t="inlineStr">
         <is>
           <t>Enabled</t>
         </is>
       </c>
-      <c r="AG45" s="29" t="inlineStr">
+      <c r="AI45" s="29" t="inlineStr">
         <is>
           <t>DisabledReason</t>
         </is>
       </c>
-      <c r="AH45" s="29" t="inlineStr">
+      <c r="AJ45" s="29" t="inlineStr">
         <is>
           <t>SourceSheet</t>
         </is>
       </c>
-      <c r="AI45" s="29" t="inlineStr">
+      <c r="AK45" s="29" t="inlineStr">
         <is>
           <t>SourceRow</t>
         </is>
@@ -17959,98 +17973,106 @@
           <t>2</t>
         </is>
       </c>
-      <c r="P46" s="31" t="inlineStr">
+      <c r="O46" t="inlineStr" s="31">
+        <is>
+          <t xml:space="preserve">true</t>
+        </is>
+      </c>
+      <c r="P46" t="n" s="31">
+        <v>10</v>
+      </c>
+      <c r="R46" s="31" t="inlineStr">
         <is>
           <t>PE_CORE_PRIMORDIAL_CHANNEL</t>
         </is>
       </c>
-      <c r="Q46" s="31" t="inlineStr">
+      <c r="S46" s="31" t="inlineStr">
         <is>
           <t>P_CORE_PRIMORDIAL</t>
         </is>
       </c>
-      <c r="R46" s="31" t="inlineStr">
+      <c r="T46" s="31" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="S46" s="31" t="inlineStr">
+      <c r="U46" s="31" t="inlineStr">
         <is>
           <t>OnEquip</t>
         </is>
       </c>
-      <c r="T46" s="31" t="inlineStr">
+      <c r="V46" s="31" t="inlineStr">
         <is>
           <t>WeaponDamageChannel</t>
         </is>
       </c>
-      <c r="U46" s="31" t="inlineStr">
+      <c r="W46" s="31" t="inlineStr">
         <is>
           <t>DamageChannel</t>
         </is>
       </c>
-      <c r="V46" s="31" t="inlineStr">
+      <c r="X46" s="31" t="inlineStr">
         <is>
           <t>Override</t>
         </is>
       </c>
-      <c r="W46" s="31" t="inlineStr">
+      <c r="Y46" s="31" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="X46" s="31" t="inlineStr">
+      <c r="Z46" s="31" t="inlineStr">
         <is>
           <t>Part.CoreDamageChannel</t>
         </is>
       </c>
-      <c r="Y46" s="31" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="Z46" s="31" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
       <c r="AA46" s="31" t="inlineStr">
         <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="AB46" s="31" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="AC46" s="31" t="inlineStr">
+        <is>
           <t>Physical</t>
         </is>
       </c>
-      <c r="AB46" s="31" t="inlineStr">
+      <c r="AD46" s="31" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="AC46" s="31" t="inlineStr">
+      <c r="AE46" s="31" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="AD46" s="31" t="inlineStr">
+      <c r="AF46" s="31" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="AE46" s="31" t="inlineStr">
+      <c r="AG46" s="31" t="inlineStr">
         <is>
           <t>Unique</t>
         </is>
       </c>
-      <c r="AF46" s="31" t="inlineStr">
+      <c r="AH46" s="31" t="inlineStr">
         <is>
           <t>true</t>
         </is>
       </c>
-      <c r="AG46" s="31" t="n"/>
-      <c r="AH46" s="31" t="inlineStr">
+      <c r="AI46" s="31" t="n"/>
+      <c r="AJ46" s="31" t="inlineStr">
         <is>
           <t>武器插槽C</t>
         </is>
       </c>
-      <c r="AI46" s="31" t="inlineStr">
+      <c r="AK46" s="31" t="inlineStr">
         <is>
           <t>2</t>
         </is>
@@ -18124,98 +18146,106 @@
           <t>3</t>
         </is>
       </c>
-      <c r="P47" s="31" t="inlineStr">
+      <c r="O47" t="inlineStr" s="31">
+        <is>
+          <t xml:space="preserve">true</t>
+        </is>
+      </c>
+      <c r="P47" t="n" s="31">
+        <v>10</v>
+      </c>
+      <c r="R47" s="31" t="inlineStr">
         <is>
           <t>PE_CORE_TIDE_CHANNEL</t>
         </is>
       </c>
-      <c r="Q47" s="31" t="inlineStr">
+      <c r="S47" s="31" t="inlineStr">
         <is>
           <t>P_CORE_TIDE</t>
         </is>
       </c>
-      <c r="R47" s="31" t="inlineStr">
+      <c r="T47" s="31" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="S47" s="31" t="inlineStr">
+      <c r="U47" s="31" t="inlineStr">
         <is>
           <t>OnEquip</t>
         </is>
       </c>
-      <c r="T47" s="31" t="inlineStr">
+      <c r="V47" s="31" t="inlineStr">
         <is>
           <t>WeaponDamageChannel</t>
         </is>
       </c>
-      <c r="U47" s="31" t="inlineStr">
+      <c r="W47" s="31" t="inlineStr">
         <is>
           <t>DamageChannel</t>
         </is>
       </c>
-      <c r="V47" s="31" t="inlineStr">
+      <c r="X47" s="31" t="inlineStr">
         <is>
           <t>Override</t>
         </is>
       </c>
-      <c r="W47" s="31" t="inlineStr">
+      <c r="Y47" s="31" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="X47" s="31" t="inlineStr">
+      <c r="Z47" s="31" t="inlineStr">
         <is>
           <t>Part.CoreDamageChannel</t>
         </is>
       </c>
-      <c r="Y47" s="31" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="Z47" s="31" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
       <c r="AA47" s="31" t="inlineStr">
         <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="AB47" s="31" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="AC47" s="31" t="inlineStr">
+        <is>
           <t>Water</t>
         </is>
       </c>
-      <c r="AB47" s="31" t="inlineStr">
+      <c r="AD47" s="31" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="AC47" s="31" t="inlineStr">
+      <c r="AE47" s="31" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="AD47" s="31" t="inlineStr">
+      <c r="AF47" s="31" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="AE47" s="31" t="inlineStr">
+      <c r="AG47" s="31" t="inlineStr">
         <is>
           <t>Unique</t>
         </is>
       </c>
-      <c r="AF47" s="31" t="inlineStr">
+      <c r="AH47" s="31" t="inlineStr">
         <is>
           <t>true</t>
         </is>
       </c>
-      <c r="AG47" s="31" t="n"/>
-      <c r="AH47" s="31" t="inlineStr">
+      <c r="AI47" s="31" t="n"/>
+      <c r="AJ47" s="31" t="inlineStr">
         <is>
           <t>武器插槽C</t>
         </is>
       </c>
-      <c r="AI47" s="31" t="inlineStr">
+      <c r="AK47" s="31" t="inlineStr">
         <is>
           <t>3</t>
         </is>
@@ -18289,98 +18319,106 @@
           <t>4</t>
         </is>
       </c>
-      <c r="P48" s="31" t="inlineStr">
+      <c r="O48" t="inlineStr" s="31">
+        <is>
+          <t xml:space="preserve">true</t>
+        </is>
+      </c>
+      <c r="P48" t="n" s="31">
+        <v>10</v>
+      </c>
+      <c r="R48" s="31" t="inlineStr">
         <is>
           <t>PE_CORE_FOREST_CHANNEL</t>
         </is>
       </c>
-      <c r="Q48" s="31" t="inlineStr">
+      <c r="S48" s="31" t="inlineStr">
         <is>
           <t>P_CORE_FOREST</t>
         </is>
       </c>
-      <c r="R48" s="31" t="inlineStr">
+      <c r="T48" s="31" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="S48" s="31" t="inlineStr">
+      <c r="U48" s="31" t="inlineStr">
         <is>
           <t>OnEquip</t>
         </is>
       </c>
-      <c r="T48" s="31" t="inlineStr">
+      <c r="V48" s="31" t="inlineStr">
         <is>
           <t>WeaponDamageChannel</t>
         </is>
       </c>
-      <c r="U48" s="31" t="inlineStr">
+      <c r="W48" s="31" t="inlineStr">
         <is>
           <t>DamageChannel</t>
         </is>
       </c>
-      <c r="V48" s="31" t="inlineStr">
+      <c r="X48" s="31" t="inlineStr">
         <is>
           <t>Override</t>
         </is>
       </c>
-      <c r="W48" s="31" t="inlineStr">
+      <c r="Y48" s="31" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="X48" s="31" t="inlineStr">
+      <c r="Z48" s="31" t="inlineStr">
         <is>
           <t>Part.CoreDamageChannel</t>
         </is>
       </c>
-      <c r="Y48" s="31" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="Z48" s="31" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
       <c r="AA48" s="31" t="inlineStr">
         <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="AB48" s="31" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="AC48" s="31" t="inlineStr">
+        <is>
           <t>Grass</t>
         </is>
       </c>
-      <c r="AB48" s="31" t="inlineStr">
+      <c r="AD48" s="31" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="AC48" s="31" t="inlineStr">
+      <c r="AE48" s="31" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="AD48" s="31" t="inlineStr">
+      <c r="AF48" s="31" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="AE48" s="31" t="inlineStr">
+      <c r="AG48" s="31" t="inlineStr">
         <is>
           <t>Unique</t>
         </is>
       </c>
-      <c r="AF48" s="31" t="inlineStr">
+      <c r="AH48" s="31" t="inlineStr">
         <is>
           <t>true</t>
         </is>
       </c>
-      <c r="AG48" s="31" t="n"/>
-      <c r="AH48" s="31" t="inlineStr">
+      <c r="AI48" s="31" t="n"/>
+      <c r="AJ48" s="31" t="inlineStr">
         <is>
           <t>武器插槽C</t>
         </is>
       </c>
-      <c r="AI48" s="31" t="inlineStr">
+      <c r="AK48" s="31" t="inlineStr">
         <is>
           <t>4</t>
         </is>
@@ -18454,98 +18492,106 @@
           <t>5</t>
         </is>
       </c>
-      <c r="P49" s="31" t="inlineStr">
+      <c r="O49" t="inlineStr" s="31">
+        <is>
+          <t xml:space="preserve">true</t>
+        </is>
+      </c>
+      <c r="P49" t="n" s="31">
+        <v>10</v>
+      </c>
+      <c r="R49" s="31" t="inlineStr">
         <is>
           <t>PE_CORE_FLAME_CHANNEL</t>
         </is>
       </c>
-      <c r="Q49" s="31" t="inlineStr">
+      <c r="S49" s="31" t="inlineStr">
         <is>
           <t>P_CORE_FLAME</t>
         </is>
       </c>
-      <c r="R49" s="31" t="inlineStr">
+      <c r="T49" s="31" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="S49" s="31" t="inlineStr">
+      <c r="U49" s="31" t="inlineStr">
         <is>
           <t>OnEquip</t>
         </is>
       </c>
-      <c r="T49" s="31" t="inlineStr">
+      <c r="V49" s="31" t="inlineStr">
         <is>
           <t>WeaponDamageChannel</t>
         </is>
       </c>
-      <c r="U49" s="31" t="inlineStr">
+      <c r="W49" s="31" t="inlineStr">
         <is>
           <t>DamageChannel</t>
         </is>
       </c>
-      <c r="V49" s="31" t="inlineStr">
+      <c r="X49" s="31" t="inlineStr">
         <is>
           <t>Override</t>
         </is>
       </c>
-      <c r="W49" s="31" t="inlineStr">
+      <c r="Y49" s="31" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="X49" s="31" t="inlineStr">
+      <c r="Z49" s="31" t="inlineStr">
         <is>
           <t>Part.CoreDamageChannel</t>
         </is>
       </c>
-      <c r="Y49" s="31" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="Z49" s="31" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
       <c r="AA49" s="31" t="inlineStr">
         <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="AB49" s="31" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="AC49" s="31" t="inlineStr">
+        <is>
           <t>Flame</t>
         </is>
       </c>
-      <c r="AB49" s="31" t="inlineStr">
+      <c r="AD49" s="31" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="AC49" s="31" t="inlineStr">
+      <c r="AE49" s="31" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="AD49" s="31" t="inlineStr">
+      <c r="AF49" s="31" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="AE49" s="31" t="inlineStr">
+      <c r="AG49" s="31" t="inlineStr">
         <is>
           <t>Unique</t>
         </is>
       </c>
-      <c r="AF49" s="31" t="inlineStr">
+      <c r="AH49" s="31" t="inlineStr">
         <is>
           <t>true</t>
         </is>
       </c>
-      <c r="AG49" s="31" t="n"/>
-      <c r="AH49" s="31" t="inlineStr">
+      <c r="AI49" s="31" t="n"/>
+      <c r="AJ49" s="31" t="inlineStr">
         <is>
           <t>武器插槽C</t>
         </is>
       </c>
-      <c r="AI49" s="31" t="inlineStr">
+      <c r="AK49" s="31" t="inlineStr">
         <is>
           <t>5</t>
         </is>
@@ -18619,98 +18665,106 @@
           <t>6</t>
         </is>
       </c>
-      <c r="P50" s="31" t="inlineStr">
+      <c r="O50" t="inlineStr" s="31">
+        <is>
+          <t xml:space="preserve">true</t>
+        </is>
+      </c>
+      <c r="P50" t="n" s="31">
+        <v>10</v>
+      </c>
+      <c r="R50" s="31" t="inlineStr">
         <is>
           <t>PE_CORE_THUNDER_CHANNEL</t>
         </is>
       </c>
-      <c r="Q50" s="31" t="inlineStr">
+      <c r="S50" s="31" t="inlineStr">
         <is>
           <t>P_CORE_THUNDER</t>
         </is>
       </c>
-      <c r="R50" s="31" t="inlineStr">
+      <c r="T50" s="31" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="S50" s="31" t="inlineStr">
+      <c r="U50" s="31" t="inlineStr">
         <is>
           <t>OnEquip</t>
         </is>
       </c>
-      <c r="T50" s="31" t="inlineStr">
+      <c r="V50" s="31" t="inlineStr">
         <is>
           <t>WeaponDamageChannel</t>
         </is>
       </c>
-      <c r="U50" s="31" t="inlineStr">
+      <c r="W50" s="31" t="inlineStr">
         <is>
           <t>DamageChannel</t>
         </is>
       </c>
-      <c r="V50" s="31" t="inlineStr">
+      <c r="X50" s="31" t="inlineStr">
         <is>
           <t>Override</t>
         </is>
       </c>
-      <c r="W50" s="31" t="inlineStr">
+      <c r="Y50" s="31" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="X50" s="31" t="inlineStr">
+      <c r="Z50" s="31" t="inlineStr">
         <is>
           <t>Part.CoreDamageChannel</t>
         </is>
       </c>
-      <c r="Y50" s="31" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="Z50" s="31" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
       <c r="AA50" s="31" t="inlineStr">
         <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="AB50" s="31" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="AC50" s="31" t="inlineStr">
+        <is>
           <t>Lightning</t>
         </is>
       </c>
-      <c r="AB50" s="31" t="inlineStr">
+      <c r="AD50" s="31" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="AC50" s="31" t="inlineStr">
+      <c r="AE50" s="31" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="AD50" s="31" t="inlineStr">
+      <c r="AF50" s="31" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="AE50" s="31" t="inlineStr">
+      <c r="AG50" s="31" t="inlineStr">
         <is>
           <t>Unique</t>
         </is>
       </c>
-      <c r="AF50" s="31" t="inlineStr">
+      <c r="AH50" s="31" t="inlineStr">
         <is>
           <t>true</t>
         </is>
       </c>
-      <c r="AG50" s="31" t="n"/>
-      <c r="AH50" s="31" t="inlineStr">
+      <c r="AI50" s="31" t="n"/>
+      <c r="AJ50" s="31" t="inlineStr">
         <is>
           <t>武器插槽C</t>
         </is>
       </c>
-      <c r="AI50" s="31" t="inlineStr">
+      <c r="AK50" s="31" t="inlineStr">
         <is>
           <t>6</t>
         </is>
@@ -18783,98 +18837,106 @@
           <t>7</t>
         </is>
       </c>
-      <c r="P51" s="31" t="inlineStr">
+      <c r="O51" t="inlineStr" s="31">
+        <is>
+          <t xml:space="preserve">true</t>
+        </is>
+      </c>
+      <c r="P51" t="n" s="31">
+        <v>10</v>
+      </c>
+      <c r="R51" s="31" t="inlineStr">
         <is>
           <t>PE_CORE_PRISM_CHANNEL</t>
         </is>
       </c>
-      <c r="Q51" s="31" t="inlineStr">
+      <c r="S51" s="31" t="inlineStr">
         <is>
           <t>P_CORE_PRISM</t>
         </is>
       </c>
-      <c r="R51" s="31" t="inlineStr">
+      <c r="T51" s="31" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="S51" s="31" t="inlineStr">
+      <c r="U51" s="31" t="inlineStr">
         <is>
           <t>OnEquip</t>
         </is>
       </c>
-      <c r="T51" s="31" t="inlineStr">
+      <c r="V51" s="31" t="inlineStr">
         <is>
           <t>WeaponDamageChannel</t>
         </is>
       </c>
-      <c r="U51" s="31" t="inlineStr">
+      <c r="W51" s="31" t="inlineStr">
         <is>
           <t>DamageChannel</t>
         </is>
       </c>
-      <c r="V51" s="31" t="inlineStr">
+      <c r="X51" s="31" t="inlineStr">
         <is>
           <t>Override</t>
         </is>
       </c>
-      <c r="W51" s="31" t="inlineStr">
+      <c r="Y51" s="31" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="X51" s="31" t="inlineStr">
+      <c r="Z51" s="31" t="inlineStr">
         <is>
           <t>Part.CoreDamageChannel</t>
         </is>
       </c>
-      <c r="Y51" s="31" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="Z51" s="31" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
       <c r="AA51" s="31" t="inlineStr">
         <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="AB51" s="31" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="AC51" s="31" t="inlineStr">
+        <is>
           <t>RandomElement</t>
         </is>
       </c>
-      <c r="AB51" s="31" t="inlineStr">
+      <c r="AD51" s="31" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="AC51" s="31" t="inlineStr">
+      <c r="AE51" s="31" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="AD51" s="31" t="inlineStr">
+      <c r="AF51" s="31" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="AE51" s="31" t="inlineStr">
+      <c r="AG51" s="31" t="inlineStr">
         <is>
           <t>Unique</t>
         </is>
       </c>
-      <c r="AF51" s="31" t="inlineStr">
+      <c r="AH51" s="31" t="inlineStr">
         <is>
           <t>true</t>
         </is>
       </c>
-      <c r="AG51" s="31" t="n"/>
-      <c r="AH51" s="31" t="inlineStr">
+      <c r="AI51" s="31" t="n"/>
+      <c r="AJ51" s="31" t="inlineStr">
         <is>
           <t>武器插槽C</t>
         </is>
       </c>
-      <c r="AI51" s="31" t="inlineStr">
+      <c r="AK51" s="31" t="inlineStr">
         <is>
           <t>7</t>
         </is>
@@ -18947,98 +19009,106 @@
           <t>8</t>
         </is>
       </c>
-      <c r="P52" s="31" t="inlineStr">
+      <c r="O52" t="inlineStr" s="31">
+        <is>
+          <t xml:space="preserve">true</t>
+        </is>
+      </c>
+      <c r="P52" t="n" s="31">
+        <v>10</v>
+      </c>
+      <c r="R52" s="31" t="inlineStr">
         <is>
           <t>PE_DAGGER_THRUST_PATTERN</t>
         </is>
       </c>
-      <c r="Q52" s="31" t="inlineStr">
+      <c r="S52" s="31" t="inlineStr">
         <is>
           <t>P_DAGGER_THRUST_GRIP</t>
         </is>
       </c>
-      <c r="R52" s="31" t="inlineStr">
+      <c r="T52" s="31" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="S52" s="31" t="inlineStr">
+      <c r="U52" s="31" t="inlineStr">
         <is>
           <t>OnEquip</t>
         </is>
       </c>
-      <c r="T52" s="31" t="inlineStr">
+      <c r="V52" s="31" t="inlineStr">
         <is>
           <t>AttackPatternReplacement</t>
         </is>
       </c>
-      <c r="U52" s="31" t="inlineStr">
+      <c r="W52" s="31" t="inlineStr">
         <is>
           <t>AttackPattern</t>
         </is>
       </c>
-      <c r="V52" s="31" t="inlineStr">
+      <c r="X52" s="31" t="inlineStr">
         <is>
           <t>Override</t>
         </is>
       </c>
-      <c r="W52" s="31" t="inlineStr">
+      <c r="Y52" s="31" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="X52" s="31" t="inlineStr">
+      <c r="Z52" s="31" t="inlineStr">
         <is>
           <t>Part.AttackPatternReplacement</t>
         </is>
       </c>
-      <c r="Y52" s="31" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="Z52" s="31" t="inlineStr">
+      <c r="AA52" s="31" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="AB52" s="31" t="inlineStr">
         <is>
           <t>Pattern.DaggerDashOnly</t>
         </is>
       </c>
-      <c r="AA52" s="31" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="AB52" s="31" t="inlineStr">
+      <c r="AC52" s="31" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="AD52" s="31" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="AC52" s="31" t="inlineStr">
+      <c r="AE52" s="31" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="AD52" s="31" t="inlineStr">
+      <c r="AF52" s="31" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="AE52" s="31" t="inlineStr">
+      <c r="AG52" s="31" t="inlineStr">
         <is>
           <t>Unique</t>
         </is>
       </c>
-      <c r="AF52" s="31" t="inlineStr">
+      <c r="AH52" s="31" t="inlineStr">
         <is>
           <t>true</t>
         </is>
       </c>
-      <c r="AG52" s="31" t="n"/>
-      <c r="AH52" s="31" t="inlineStr">
+      <c r="AI52" s="31" t="n"/>
+      <c r="AJ52" s="31" t="inlineStr">
         <is>
           <t>武器插槽C</t>
         </is>
       </c>
-      <c r="AI52" s="31" t="inlineStr">
+      <c r="AK52" s="31" t="inlineStr">
         <is>
           <t>8</t>
         </is>
@@ -19111,61 +19181,59 @@
           <t>9</t>
         </is>
       </c>
-      <c r="P53" s="31" t="inlineStr">
+      <c r="O53" t="inlineStr" s="31">
+        <is>
+          <t xml:space="preserve">true</t>
+        </is>
+      </c>
+      <c r="P53" t="n" s="31">
+        <v>10</v>
+      </c>
+      <c r="R53" s="31" t="inlineStr">
         <is>
           <t>PE_DAGGER_THRUST_COOLDOWN</t>
         </is>
       </c>
-      <c r="Q53" s="31" t="inlineStr">
+      <c r="S53" s="31" t="inlineStr">
         <is>
           <t>P_DAGGER_THRUST_GRIP</t>
         </is>
       </c>
-      <c r="R53" s="31" t="inlineStr">
+      <c r="T53" s="31" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="S53" s="31" t="inlineStr">
+      <c r="U53" s="31" t="inlineStr">
         <is>
           <t>OnEquip</t>
         </is>
       </c>
-      <c r="T53" s="31" t="inlineStr">
+      <c r="V53" s="31" t="inlineStr">
         <is>
           <t>StatModifier</t>
         </is>
       </c>
-      <c r="U53" s="31" t="inlineStr">
+      <c r="W53" s="31" t="inlineStr">
         <is>
           <t>AttackIntervalSeconds</t>
         </is>
       </c>
-      <c r="V53" s="31" t="inlineStr">
+      <c r="X53" s="31" t="inlineStr">
         <is>
           <t>Override</t>
         </is>
       </c>
-      <c r="W53" s="31" t="inlineStr">
+      <c r="Y53" s="31" t="inlineStr">
         <is>
           <t>0.4</t>
         </is>
       </c>
-      <c r="X53" s="31" t="inlineStr">
+      <c r="Z53" s="31" t="inlineStr">
         <is>
           <t>Part.StatModifier</t>
         </is>
       </c>
-      <c r="Y53" s="31" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="Z53" s="31" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
       <c r="AA53" s="31" t="inlineStr">
         <is>
           <t>None</t>
@@ -19173,36 +19241,46 @@
       </c>
       <c r="AB53" s="31" t="inlineStr">
         <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="AC53" s="31" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="AD53" s="31" t="inlineStr">
+        <is>
           <t>0</t>
         </is>
       </c>
-      <c r="AC53" s="31" t="inlineStr">
+      <c r="AE53" s="31" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="AD53" s="31" t="inlineStr">
+      <c r="AF53" s="31" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="AE53" s="31" t="inlineStr">
+      <c r="AG53" s="31" t="inlineStr">
         <is>
           <t>Unique</t>
         </is>
       </c>
-      <c r="AF53" s="31" t="inlineStr">
+      <c r="AH53" s="31" t="inlineStr">
         <is>
           <t>true</t>
         </is>
       </c>
-      <c r="AG53" s="31" t="n"/>
-      <c r="AH53" s="31" t="inlineStr">
+      <c r="AI53" s="31" t="n"/>
+      <c r="AJ53" s="31" t="inlineStr">
         <is>
           <t>武器插槽C</t>
         </is>
       </c>
-      <c r="AI53" s="31" t="inlineStr">
+      <c r="AK53" s="31" t="inlineStr">
         <is>
           <t>8</t>
         </is>
@@ -19275,61 +19353,59 @@
           <t>10</t>
         </is>
       </c>
-      <c r="P54" s="31" t="inlineStr">
+      <c r="O54" t="inlineStr" s="31">
+        <is>
+          <t xml:space="preserve">false</t>
+        </is>
+      </c>
+      <c r="P54" t="n" s="31">
+        <v>0</v>
+      </c>
+      <c r="R54" s="31" t="inlineStr">
         <is>
           <t>PE_DAGGER_STRENGTH_SPEED</t>
         </is>
       </c>
-      <c r="Q54" s="31" t="inlineStr">
+      <c r="S54" s="31" t="inlineStr">
         <is>
           <t>P_DAGGER_STRENGTH_GRIP</t>
         </is>
       </c>
-      <c r="R54" s="31" t="inlineStr">
+      <c r="T54" s="31" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="S54" s="31" t="inlineStr">
+      <c r="U54" s="31" t="inlineStr">
         <is>
           <t>OnEquip</t>
         </is>
       </c>
-      <c r="T54" s="31" t="inlineStr">
+      <c r="V54" s="31" t="inlineStr">
         <is>
           <t>StatModifier</t>
         </is>
       </c>
-      <c r="U54" s="31" t="inlineStr">
+      <c r="W54" s="31" t="inlineStr">
         <is>
           <t>AttackSpeed</t>
         </is>
       </c>
-      <c r="V54" s="31" t="inlineStr">
+      <c r="X54" s="31" t="inlineStr">
         <is>
           <t>Multiply</t>
         </is>
       </c>
-      <c r="W54" s="31" t="inlineStr">
+      <c r="Y54" s="31" t="inlineStr">
         <is>
           <t>1.2</t>
         </is>
       </c>
-      <c r="X54" s="31" t="inlineStr">
+      <c r="Z54" s="31" t="inlineStr">
         <is>
           <t>Part.StatModifier</t>
         </is>
       </c>
-      <c r="Y54" s="31" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="Z54" s="31" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
       <c r="AA54" s="31" t="inlineStr">
         <is>
           <t>None</t>
@@ -19337,36 +19413,46 @@
       </c>
       <c r="AB54" s="31" t="inlineStr">
         <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="AC54" s="31" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="AD54" s="31" t="inlineStr">
+        <is>
           <t>0</t>
         </is>
       </c>
-      <c r="AC54" s="31" t="inlineStr">
+      <c r="AE54" s="31" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="AD54" s="31" t="inlineStr">
+      <c r="AF54" s="31" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="AE54" s="31" t="inlineStr">
+      <c r="AG54" s="31" t="inlineStr">
         <is>
           <t>Stackable</t>
         </is>
       </c>
-      <c r="AF54" s="31" t="inlineStr">
+      <c r="AH54" s="31" t="inlineStr">
         <is>
           <t>true</t>
         </is>
       </c>
-      <c r="AG54" s="31" t="n"/>
-      <c r="AH54" s="31" t="inlineStr">
+      <c r="AI54" s="31" t="n"/>
+      <c r="AJ54" s="31" t="inlineStr">
         <is>
           <t>武器插槽C</t>
         </is>
       </c>
-      <c r="AI54" s="31" t="inlineStr">
+      <c r="AK54" s="31" t="inlineStr">
         <is>
           <t>9</t>
         </is>
@@ -19439,98 +19525,106 @@
           <t>11</t>
         </is>
       </c>
-      <c r="P55" s="31" t="inlineStr">
+      <c r="O55" t="inlineStr" s="31">
+        <is>
+          <t xml:space="preserve">false</t>
+        </is>
+      </c>
+      <c r="P55" t="n" s="31">
+        <v>0</v>
+      </c>
+      <c r="R55" s="31" t="inlineStr">
         <is>
           <t>PE_DAGGER_HOLY_KILL_HEAL</t>
         </is>
       </c>
-      <c r="Q55" s="31" t="inlineStr">
+      <c r="S55" s="31" t="inlineStr">
         <is>
           <t>P_DAGGER_HOLY_BLADE</t>
         </is>
       </c>
-      <c r="R55" s="31" t="inlineStr">
+      <c r="T55" s="31" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="S55" s="31" t="inlineStr">
+      <c r="U55" s="31" t="inlineStr">
         <is>
           <t>OnKill</t>
         </is>
       </c>
-      <c r="T55" s="31" t="inlineStr">
+      <c r="V55" s="31" t="inlineStr">
         <is>
           <t>UniqueBehavior</t>
         </is>
       </c>
-      <c r="U55" s="31" t="inlineStr">
+      <c r="W55" s="31" t="inlineStr">
         <is>
           <t>OnKill</t>
         </is>
       </c>
-      <c r="V55" s="31" t="inlineStr">
+      <c r="X55" s="31" t="inlineStr">
         <is>
           <t>Add</t>
         </is>
       </c>
-      <c r="W55" s="31" t="inlineStr">
+      <c r="Y55" s="31" t="inlineStr">
         <is>
           <t>0.05</t>
         </is>
       </c>
-      <c r="X55" s="31" t="inlineStr">
+      <c r="Z55" s="31" t="inlineStr">
         <is>
           <t>Part.OnKillHealPercent</t>
         </is>
       </c>
-      <c r="Y55" s="31" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="Z55" s="31" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
       <c r="AA55" s="31" t="inlineStr">
         <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="AB55" s="31" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="AC55" s="31" t="inlineStr">
+        <is>
           <t>HealMaxHpPercent</t>
         </is>
       </c>
-      <c r="AB55" s="31" t="inlineStr">
+      <c r="AD55" s="31" t="inlineStr">
         <is>
           <t>0.05</t>
         </is>
       </c>
-      <c r="AC55" s="31" t="inlineStr">
+      <c r="AE55" s="31" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="AD55" s="31" t="inlineStr">
+      <c r="AF55" s="31" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="AE55" s="31" t="inlineStr">
+      <c r="AG55" s="31" t="inlineStr">
         <is>
           <t>Stackable</t>
         </is>
       </c>
-      <c r="AF55" s="31" t="inlineStr">
+      <c r="AH55" s="31" t="inlineStr">
         <is>
           <t>true</t>
         </is>
       </c>
-      <c r="AG55" s="31" t="n"/>
-      <c r="AH55" s="31" t="inlineStr">
+      <c r="AI55" s="31" t="n"/>
+      <c r="AJ55" s="31" t="inlineStr">
         <is>
           <t>武器插槽C</t>
         </is>
       </c>
-      <c r="AI55" s="31" t="inlineStr">
+      <c r="AK55" s="31" t="inlineStr">
         <is>
           <t>14</t>
         </is>
@@ -19607,6 +19701,14 @@
           <t>12</t>
         </is>
       </c>
+      <c r="O56" t="inlineStr" s="31">
+        <is>
+          <t xml:space="preserve">false</t>
+        </is>
+      </c>
+      <c r="P56" t="n" s="31">
+        <v>0</v>
+      </c>
     </row>
     <row r="57" ht="22" customHeight="1" s="32">
       <c r="A57" s="31" t="inlineStr">
@@ -19679,6 +19781,14 @@
           <t>13</t>
         </is>
       </c>
+      <c r="O57" t="inlineStr" s="31">
+        <is>
+          <t xml:space="preserve">false</t>
+        </is>
+      </c>
+      <c r="P57" t="n" s="31">
+        <v>0</v>
+      </c>
     </row>
     <row r="58" ht="22" customHeight="1" s="32">
       <c r="A58" s="31" t="inlineStr">
@@ -19747,6 +19857,14 @@
           <t>14</t>
         </is>
       </c>
+      <c r="O58" t="inlineStr" s="31">
+        <is>
+          <t xml:space="preserve">true</t>
+        </is>
+      </c>
+      <c r="P58" t="n" s="31">
+        <v>10</v>
+      </c>
     </row>
     <row r="59" ht="22" customHeight="1" s="32">
       <c r="A59" s="31" t="inlineStr">
@@ -19819,6 +19937,14 @@
           <t>15</t>
         </is>
       </c>
+      <c r="O59" t="inlineStr" s="31">
+        <is>
+          <t xml:space="preserve">false</t>
+        </is>
+      </c>
+      <c r="P59" t="n" s="31">
+        <v>0</v>
+      </c>
     </row>
     <row r="60" ht="30" customHeight="1" s="32">
       <c r="A60" s="31" t="inlineStr">
@@ -19892,6 +20018,14 @@
           <t>16</t>
         </is>
       </c>
+      <c r="O60" t="inlineStr" s="31">
+        <is>
+          <t xml:space="preserve">false</t>
+        </is>
+      </c>
+      <c r="P60" t="n" s="31">
+        <v>0</v>
+      </c>
     </row>
     <row r="61" ht="22" customHeight="1" s="32">
       <c r="A61" s="31" t="inlineStr">
@@ -19964,6 +20098,14 @@
           <t>17</t>
         </is>
       </c>
+      <c r="O61" t="inlineStr" s="31">
+        <is>
+          <t xml:space="preserve">false</t>
+        </is>
+      </c>
+      <c r="P61" t="n" s="31">
+        <v>0</v>
+      </c>
     </row>
     <row r="62" ht="22" customHeight="1" s="32">
       <c r="A62" s="31" t="inlineStr">
@@ -20036,6 +20178,14 @@
           <t>18</t>
         </is>
       </c>
+      <c r="O62" t="inlineStr" s="31">
+        <is>
+          <t xml:space="preserve">false</t>
+        </is>
+      </c>
+      <c r="P62" t="n" s="31">
+        <v>0</v>
+      </c>
     </row>
     <row r="63" ht="22" customHeight="1" s="32">
       <c r="A63" s="31" t="inlineStr">
@@ -20104,6 +20254,14 @@
           <t>19</t>
         </is>
       </c>
+      <c r="O63" t="inlineStr" s="31">
+        <is>
+          <t xml:space="preserve">false</t>
+        </is>
+      </c>
+      <c r="P63" t="n" s="31">
+        <v>0</v>
+      </c>
     </row>
     <row r="64" ht="22" customHeight="1" s="32">
       <c r="A64" s="31" t="inlineStr">
@@ -20176,6 +20334,14 @@
           <t>20</t>
         </is>
       </c>
+      <c r="O64" t="inlineStr" s="31">
+        <is>
+          <t xml:space="preserve">false</t>
+        </is>
+      </c>
+      <c r="P64" t="n" s="31">
+        <v>0</v>
+      </c>
     </row>
     <row r="65" ht="22" customHeight="1" s="32">
       <c r="A65" s="31" t="inlineStr">
@@ -20244,6 +20410,14 @@
           <t>21</t>
         </is>
       </c>
+      <c r="O65" t="inlineStr" s="31">
+        <is>
+          <t xml:space="preserve">false</t>
+        </is>
+      </c>
+      <c r="P65" t="n" s="31">
+        <v>0</v>
+      </c>
     </row>
     <row r="66" ht="22" customHeight="1" s="32">
       <c r="A66" s="31" t="inlineStr">
@@ -20312,6 +20486,14 @@
           <t>22</t>
         </is>
       </c>
+      <c r="O66" t="inlineStr" s="31">
+        <is>
+          <t xml:space="preserve">false</t>
+        </is>
+      </c>
+      <c r="P66" t="n" s="31">
+        <v>0</v>
+      </c>
     </row>
     <row r="67" ht="22" customHeight="1" s="32">
       <c r="A67" s="31" t="inlineStr">
@@ -20380,6 +20562,14 @@
           <t>23</t>
         </is>
       </c>
+      <c r="O67" t="inlineStr" s="31">
+        <is>
+          <t xml:space="preserve">false</t>
+        </is>
+      </c>
+      <c r="P67" t="n" s="31">
+        <v>0</v>
+      </c>
     </row>
     <row r="68" ht="22" customHeight="1" s="32">
       <c r="A68" s="31" t="inlineStr">
@@ -20448,6 +20638,14 @@
           <t>24</t>
         </is>
       </c>
+      <c r="O68" t="inlineStr" s="31">
+        <is>
+          <t xml:space="preserve">false</t>
+        </is>
+      </c>
+      <c r="P68" t="n" s="31">
+        <v>0</v>
+      </c>
     </row>
     <row r="69" ht="22" customHeight="1" s="32">
       <c r="A69" s="31" t="inlineStr">
@@ -20516,6 +20714,14 @@
           <t>25</t>
         </is>
       </c>
+      <c r="O69" t="inlineStr" s="31">
+        <is>
+          <t xml:space="preserve">false</t>
+        </is>
+      </c>
+      <c r="P69" t="n" s="31">
+        <v>0</v>
+      </c>
     </row>
     <row r="70" ht="22" customHeight="1" s="32">
       <c r="A70" s="31" t="inlineStr">
@@ -20584,6 +20790,14 @@
           <t>26</t>
         </is>
       </c>
+      <c r="O70" t="inlineStr" s="31">
+        <is>
+          <t xml:space="preserve">false</t>
+        </is>
+      </c>
+      <c r="P70" t="n" s="31">
+        <v>0</v>
+      </c>
     </row>
     <row r="71" ht="22" customHeight="1" s="32">
       <c r="A71" s="31" t="inlineStr">
@@ -20652,6 +20866,14 @@
           <t>27</t>
         </is>
       </c>
+      <c r="O71" t="inlineStr" s="31">
+        <is>
+          <t xml:space="preserve">false</t>
+        </is>
+      </c>
+      <c r="P71" t="n" s="31">
+        <v>0</v>
+      </c>
     </row>
     <row r="72" ht="22" customHeight="1" s="32">
       <c r="A72" s="31" t="inlineStr">
@@ -20720,6 +20942,14 @@
           <t>28</t>
         </is>
       </c>
+      <c r="O72" t="inlineStr" s="31">
+        <is>
+          <t xml:space="preserve">false</t>
+        </is>
+      </c>
+      <c r="P72" t="n" s="31">
+        <v>0</v>
+      </c>
     </row>
     <row r="73" ht="22" customHeight="1" s="32">
       <c r="A73" s="31" t="inlineStr">
@@ -20788,6 +21018,14 @@
           <t>29</t>
         </is>
       </c>
+      <c r="O73" t="inlineStr" s="31">
+        <is>
+          <t xml:space="preserve">false</t>
+        </is>
+      </c>
+      <c r="P73" t="n" s="31">
+        <v>0</v>
+      </c>
     </row>
     <row r="74" ht="22" customHeight="1" s="32">
       <c r="A74" s="31" t="inlineStr">
@@ -20856,6 +21094,14 @@
           <t>30</t>
         </is>
       </c>
+      <c r="O74" t="inlineStr" s="31">
+        <is>
+          <t xml:space="preserve">false</t>
+        </is>
+      </c>
+      <c r="P74" t="n" s="31">
+        <v>0</v>
+      </c>
     </row>
     <row r="75" ht="22" customHeight="1" s="32">
       <c r="A75" s="31" t="inlineStr">
@@ -20924,6 +21170,14 @@
           <t>31</t>
         </is>
       </c>
+      <c r="O75" t="inlineStr" s="31">
+        <is>
+          <t xml:space="preserve">false</t>
+        </is>
+      </c>
+      <c r="P75" t="n" s="31">
+        <v>0</v>
+      </c>
     </row>
     <row r="76" ht="22" customHeight="1" s="32">
       <c r="A76" s="31" t="inlineStr">
@@ -20992,6 +21246,14 @@
           <t>32</t>
         </is>
       </c>
+      <c r="O76" t="inlineStr" s="31">
+        <is>
+          <t xml:space="preserve">false</t>
+        </is>
+      </c>
+      <c r="P76" t="n" s="31">
+        <v>0</v>
+      </c>
     </row>
     <row r="77" ht="22" customHeight="1" s="32">
       <c r="A77" s="31" t="inlineStr">
@@ -21060,6 +21322,14 @@
           <t>33</t>
         </is>
       </c>
+      <c r="O77" t="inlineStr" s="31">
+        <is>
+          <t xml:space="preserve">false</t>
+        </is>
+      </c>
+      <c r="P77" t="n" s="31">
+        <v>0</v>
+      </c>
     </row>
     <row r="78" ht="22" customHeight="1" s="32">
       <c r="A78" s="31" t="inlineStr">
@@ -21127,6 +21397,14 @@
         <is>
           <t>34</t>
         </is>
+      </c>
+      <c r="O78" t="inlineStr" s="31">
+        <is>
+          <t xml:space="preserve">false</t>
+        </is>
+      </c>
+      <c r="P78" t="n" s="31">
+        <v>0</v>
       </c>
     </row>
     <row r="79" ht="75" customHeight="1" s="32">
@@ -21200,6 +21478,14 @@
           <t>35</t>
         </is>
       </c>
+      <c r="O79" t="inlineStr" s="31">
+        <is>
+          <t xml:space="preserve">false</t>
+        </is>
+      </c>
+      <c r="P79" t="n" s="31">
+        <v>0</v>
+      </c>
     </row>
     <row r="80" ht="22" customHeight="1" s="32">
       <c r="A80" s="31" t="inlineStr">
@@ -21268,6 +21554,14 @@
           <t>36</t>
         </is>
       </c>
+      <c r="O80" t="inlineStr" s="31">
+        <is>
+          <t xml:space="preserve">false</t>
+        </is>
+      </c>
+      <c r="P80" t="n" s="31">
+        <v>0</v>
+      </c>
     </row>
     <row r="81" ht="22" customHeight="1" s="32">
       <c r="A81" s="31" t="inlineStr">
@@ -21336,6 +21630,14 @@
           <t>37</t>
         </is>
       </c>
+      <c r="O81" t="inlineStr" s="31">
+        <is>
+          <t xml:space="preserve">false</t>
+        </is>
+      </c>
+      <c r="P81" t="n" s="31">
+        <v>0</v>
+      </c>
     </row>
     <row r="82" ht="22" customHeight="1" s="32">
       <c r="A82" s="31" t="inlineStr">
@@ -21404,6 +21706,14 @@
           <t>38</t>
         </is>
       </c>
+      <c r="O82" t="inlineStr" s="31">
+        <is>
+          <t xml:space="preserve">false</t>
+        </is>
+      </c>
+      <c r="P82" t="n" s="31">
+        <v>0</v>
+      </c>
     </row>
     <row r="83" ht="22" customHeight="1" s="32">
       <c r="A83" s="31" t="inlineStr">
@@ -21472,6 +21782,14 @@
           <t>39</t>
         </is>
       </c>
+      <c r="O83" t="inlineStr" s="31">
+        <is>
+          <t xml:space="preserve">false</t>
+        </is>
+      </c>
+      <c r="P83" t="n" s="31">
+        <v>0</v>
+      </c>
     </row>
     <row r="84" ht="22" customHeight="1" s="32">
       <c r="A84" s="31" t="inlineStr">
@@ -21540,6 +21858,14 @@
           <t>40</t>
         </is>
       </c>
+      <c r="O84" t="inlineStr" s="31">
+        <is>
+          <t xml:space="preserve">false</t>
+        </is>
+      </c>
+      <c r="P84" t="n" s="31">
+        <v>0</v>
+      </c>
     </row>
     <row r="85" ht="22" customHeight="1" s="32">
       <c r="A85" s="31" t="inlineStr">
@@ -21607,6 +21933,14 @@
         <is>
           <t>41</t>
         </is>
+      </c>
+      <c r="O85" t="inlineStr" s="31">
+        <is>
+          <t xml:space="preserve">false</t>
+        </is>
+      </c>
+      <c r="P85" t="n" s="31">
+        <v>0</v>
       </c>
     </row>
     <row r="86" ht="45" customHeight="1" s="32">
@@ -21678,6 +22012,14 @@
           <t>42</t>
         </is>
       </c>
+      <c r="O86" t="inlineStr" s="31">
+        <is>
+          <t xml:space="preserve">false</t>
+        </is>
+      </c>
+      <c r="P86" t="n" s="31">
+        <v>0</v>
+      </c>
     </row>
     <row r="87" ht="22" customHeight="1" s="32">
       <c r="A87" s="31" t="inlineStr">
@@ -21746,6 +22088,14 @@
           <t>43</t>
         </is>
       </c>
+      <c r="O87" t="inlineStr" s="31">
+        <is>
+          <t xml:space="preserve">false</t>
+        </is>
+      </c>
+      <c r="P87" t="n" s="31">
+        <v>0</v>
+      </c>
     </row>
     <row r="88" ht="22" customHeight="1" s="32">
       <c r="A88" s="31" t="inlineStr">
@@ -21814,6 +22164,14 @@
           <t>44</t>
         </is>
       </c>
+      <c r="O88" t="inlineStr" s="31">
+        <is>
+          <t xml:space="preserve">false</t>
+        </is>
+      </c>
+      <c r="P88" t="n" s="31">
+        <v>0</v>
+      </c>
     </row>
     <row r="89" ht="22" customHeight="1" s="32">
       <c r="A89" s="31" t="inlineStr">
@@ -21882,6 +22240,14 @@
           <t>45</t>
         </is>
       </c>
+      <c r="O89" t="inlineStr" s="31">
+        <is>
+          <t xml:space="preserve">false</t>
+        </is>
+      </c>
+      <c r="P89" t="n" s="31">
+        <v>0</v>
+      </c>
     </row>
     <row r="90" ht="22" customHeight="1" s="32">
       <c r="A90" s="31" t="inlineStr">
@@ -21950,6 +22316,14 @@
           <t>46</t>
         </is>
       </c>
+      <c r="O90" t="inlineStr" s="31">
+        <is>
+          <t xml:space="preserve">false</t>
+        </is>
+      </c>
+      <c r="P90" t="n" s="31">
+        <v>0</v>
+      </c>
     </row>
     <row r="91" ht="22" customHeight="1" s="32">
       <c r="A91" s="31" t="inlineStr">
@@ -22018,6 +22392,14 @@
           <t>47</t>
         </is>
       </c>
+      <c r="O91" t="inlineStr" s="31">
+        <is>
+          <t xml:space="preserve">false</t>
+        </is>
+      </c>
+      <c r="P91" t="n" s="31">
+        <v>0</v>
+      </c>
     </row>
     <row r="92" ht="22" customHeight="1" s="32">
       <c r="A92" s="31" t="inlineStr">
@@ -22086,6 +22468,14 @@
           <t>48</t>
         </is>
       </c>
+      <c r="O92" t="inlineStr" s="31">
+        <is>
+          <t xml:space="preserve">false</t>
+        </is>
+      </c>
+      <c r="P92" t="n" s="31">
+        <v>0</v>
+      </c>
     </row>
     <row r="93" ht="22" customHeight="1" s="32">
       <c r="A93" s="31" t="inlineStr">
@@ -22154,6 +22544,14 @@
           <t>49</t>
         </is>
       </c>
+      <c r="O93" t="inlineStr" s="31">
+        <is>
+          <t xml:space="preserve">false</t>
+        </is>
+      </c>
+      <c r="P93" t="n" s="31">
+        <v>0</v>
+      </c>
     </row>
     <row r="94" ht="22" customHeight="1" s="32">
       <c r="A94" s="31" t="inlineStr">
@@ -22222,6 +22620,14 @@
           <t>50</t>
         </is>
       </c>
+      <c r="O94" t="inlineStr" s="31">
+        <is>
+          <t xml:space="preserve">false</t>
+        </is>
+      </c>
+      <c r="P94" t="n" s="31">
+        <v>0</v>
+      </c>
     </row>
     <row r="95" ht="22" customHeight="1" s="32">
       <c r="A95" s="31" t="inlineStr">
@@ -22290,6 +22696,14 @@
           <t>51</t>
         </is>
       </c>
+      <c r="O95" t="inlineStr" s="31">
+        <is>
+          <t xml:space="preserve">false</t>
+        </is>
+      </c>
+      <c r="P95" t="n" s="31">
+        <v>0</v>
+      </c>
     </row>
     <row r="96" ht="22" customHeight="1" s="32">
       <c r="A96" s="31" t="inlineStr">
@@ -22358,6 +22772,14 @@
           <t>52</t>
         </is>
       </c>
+      <c r="O96" t="inlineStr" s="31">
+        <is>
+          <t xml:space="preserve">false</t>
+        </is>
+      </c>
+      <c r="P96" t="n" s="31">
+        <v>0</v>
+      </c>
     </row>
     <row r="97" ht="22" customHeight="1" s="32">
       <c r="A97" s="31" t="inlineStr">
@@ -22426,6 +22848,14 @@
           <t>53</t>
         </is>
       </c>
+      <c r="O97" t="inlineStr" s="31">
+        <is>
+          <t xml:space="preserve">false</t>
+        </is>
+      </c>
+      <c r="P97" t="n" s="31">
+        <v>0</v>
+      </c>
     </row>
     <row r="98" ht="22" customHeight="1" s="32">
       <c r="A98" s="31" t="inlineStr">
@@ -22494,6 +22924,14 @@
           <t>54</t>
         </is>
       </c>
+      <c r="O98" t="inlineStr" s="31">
+        <is>
+          <t xml:space="preserve">false</t>
+        </is>
+      </c>
+      <c r="P98" t="n" s="31">
+        <v>0</v>
+      </c>
     </row>
     <row r="99" ht="22" customHeight="1" s="32">
       <c r="A99" s="31" t="inlineStr">
@@ -22562,6 +23000,14 @@
           <t>55</t>
         </is>
       </c>
+      <c r="O99" t="inlineStr" s="31">
+        <is>
+          <t xml:space="preserve">false</t>
+        </is>
+      </c>
+      <c r="P99" t="n" s="31">
+        <v>0</v>
+      </c>
     </row>
     <row r="100" ht="22" customHeight="1" s="32">
       <c r="A100" s="31" t="inlineStr">
@@ -22630,6 +23076,14 @@
           <t>56</t>
         </is>
       </c>
+      <c r="O100" t="inlineStr" s="31">
+        <is>
+          <t xml:space="preserve">false</t>
+        </is>
+      </c>
+      <c r="P100" t="n" s="31">
+        <v>0</v>
+      </c>
     </row>
     <row r="101" ht="22" customHeight="1" s="32">
       <c r="A101" s="31" t="inlineStr">
@@ -22698,6 +23152,14 @@
           <t>57</t>
         </is>
       </c>
+      <c r="O101" t="inlineStr" s="31">
+        <is>
+          <t xml:space="preserve">false</t>
+        </is>
+      </c>
+      <c r="P101" t="n" s="31">
+        <v>0</v>
+      </c>
     </row>
     <row r="102" ht="22" customHeight="1" s="32">
       <c r="A102" s="31" t="inlineStr">
@@ -22766,6 +23228,14 @@
           <t>58</t>
         </is>
       </c>
+      <c r="O102" t="inlineStr" s="31">
+        <is>
+          <t xml:space="preserve">false</t>
+        </is>
+      </c>
+      <c r="P102" t="n" s="31">
+        <v>0</v>
+      </c>
     </row>
     <row r="103" ht="22" customHeight="1" s="32">
       <c r="A103" s="31" t="inlineStr">
@@ -22834,6 +23304,14 @@
           <t>59</t>
         </is>
       </c>
+      <c r="O103" t="inlineStr" s="31">
+        <is>
+          <t xml:space="preserve">false</t>
+        </is>
+      </c>
+      <c r="P103" t="n" s="31">
+        <v>0</v>
+      </c>
     </row>
     <row r="104" ht="22" customHeight="1" s="32">
       <c r="A104" s="31" t="inlineStr">
@@ -22902,6 +23380,14 @@
           <t>60</t>
         </is>
       </c>
+      <c r="O104" t="inlineStr" s="31">
+        <is>
+          <t xml:space="preserve">false</t>
+        </is>
+      </c>
+      <c r="P104" t="n" s="31">
+        <v>0</v>
+      </c>
     </row>
     <row r="105" ht="22" customHeight="1" s="32">
       <c r="A105" s="31" t="inlineStr">
@@ -22970,6 +23456,14 @@
           <t>61</t>
         </is>
       </c>
+      <c r="O105" t="inlineStr" s="31">
+        <is>
+          <t xml:space="preserve">false</t>
+        </is>
+      </c>
+      <c r="P105" t="n" s="31">
+        <v>0</v>
+      </c>
     </row>
     <row r="106" ht="22" customHeight="1" s="32">
       <c r="A106" s="31" t="inlineStr">
@@ -23037,6 +23531,14 @@
         <is>
           <t>62</t>
         </is>
+      </c>
+      <c r="O106" t="inlineStr" s="31">
+        <is>
+          <t xml:space="preserve">false</t>
+        </is>
+      </c>
+      <c r="P106" t="n" s="31">
+        <v>0</v>
       </c>
     </row>
     <row r="107" ht="75" customHeight="1" s="32">
@@ -23110,6 +23612,14 @@
           <t>63</t>
         </is>
       </c>
+      <c r="O107" t="inlineStr" s="31">
+        <is>
+          <t xml:space="preserve">false</t>
+        </is>
+      </c>
+      <c r="P107" t="n" s="31">
+        <v>0</v>
+      </c>
     </row>
     <row r="108" ht="22" customHeight="1" s="32">
       <c r="A108" s="31" t="inlineStr">
@@ -23178,6 +23688,14 @@
           <t>64</t>
         </is>
       </c>
+      <c r="O108" t="inlineStr" s="31">
+        <is>
+          <t xml:space="preserve">false</t>
+        </is>
+      </c>
+      <c r="P108" t="n" s="31">
+        <v>0</v>
+      </c>
     </row>
     <row r="109" ht="22" customHeight="1" s="32">
       <c r="A109" s="31" t="inlineStr">
@@ -23246,6 +23764,14 @@
           <t>65</t>
         </is>
       </c>
+      <c r="O109" t="inlineStr" s="31">
+        <is>
+          <t xml:space="preserve">false</t>
+        </is>
+      </c>
+      <c r="P109" t="n" s="31">
+        <v>0</v>
+      </c>
     </row>
     <row r="110" ht="22" customHeight="1" s="32">
       <c r="A110" s="31" t="inlineStr">
@@ -23314,6 +23840,14 @@
           <t>66</t>
         </is>
       </c>
+      <c r="O110" t="inlineStr" s="31">
+        <is>
+          <t xml:space="preserve">false</t>
+        </is>
+      </c>
+      <c r="P110" t="n" s="31">
+        <v>0</v>
+      </c>
     </row>
     <row r="111" ht="22" customHeight="1" s="32">
       <c r="A111" s="31" t="inlineStr">
@@ -23382,6 +23916,14 @@
           <t>67</t>
         </is>
       </c>
+      <c r="O111" t="inlineStr" s="31">
+        <is>
+          <t xml:space="preserve">false</t>
+        </is>
+      </c>
+      <c r="P111" t="n" s="31">
+        <v>0</v>
+      </c>
     </row>
     <row r="112" ht="22" customHeight="1" s="32">
       <c r="A112" s="31" t="inlineStr">
@@ -23450,6 +23992,14 @@
           <t>68</t>
         </is>
       </c>
+      <c r="O112" t="inlineStr" s="31">
+        <is>
+          <t xml:space="preserve">false</t>
+        </is>
+      </c>
+      <c r="P112" t="n" s="31">
+        <v>0</v>
+      </c>
     </row>
     <row r="113" ht="22" customHeight="1" s="32">
       <c r="A113" s="31" t="inlineStr">
@@ -23518,6 +24068,14 @@
           <t>69</t>
         </is>
       </c>
+      <c r="O113" t="inlineStr" s="31">
+        <is>
+          <t xml:space="preserve">false</t>
+        </is>
+      </c>
+      <c r="P113" t="n" s="31">
+        <v>0</v>
+      </c>
     </row>
     <row r="114" ht="22" customHeight="1" s="32">
       <c r="A114" s="31" t="inlineStr">
@@ -23586,6 +24144,14 @@
           <t>70</t>
         </is>
       </c>
+      <c r="O114" t="inlineStr" s="31">
+        <is>
+          <t xml:space="preserve">false</t>
+        </is>
+      </c>
+      <c r="P114" t="n" s="31">
+        <v>0</v>
+      </c>
     </row>
     <row r="115" ht="22" customHeight="1" s="32">
       <c r="A115" s="31" t="inlineStr">
@@ -23654,6 +24220,14 @@
           <t>71</t>
         </is>
       </c>
+      <c r="O115" t="inlineStr" s="31">
+        <is>
+          <t xml:space="preserve">false</t>
+        </is>
+      </c>
+      <c r="P115" t="n" s="31">
+        <v>0</v>
+      </c>
     </row>
     <row r="116" ht="22" customHeight="1" s="32">
       <c r="A116" s="31" t="inlineStr">
@@ -23722,6 +24296,14 @@
           <t>72</t>
         </is>
       </c>
+      <c r="O116" t="inlineStr" s="31">
+        <is>
+          <t xml:space="preserve">false</t>
+        </is>
+      </c>
+      <c r="P116" t="n" s="31">
+        <v>0</v>
+      </c>
     </row>
     <row r="117" ht="22" customHeight="1" s="32">
       <c r="A117" s="31" t="inlineStr">
@@ -23790,6 +24372,14 @@
           <t>73</t>
         </is>
       </c>
+      <c r="O117" t="inlineStr" s="31">
+        <is>
+          <t xml:space="preserve">false</t>
+        </is>
+      </c>
+      <c r="P117" t="n" s="31">
+        <v>0</v>
+      </c>
     </row>
     <row r="118" ht="22" customHeight="1" s="32">
       <c r="A118" s="31" t="inlineStr">
@@ -23858,6 +24448,14 @@
           <t>74</t>
         </is>
       </c>
+      <c r="O118" t="inlineStr" s="31">
+        <is>
+          <t xml:space="preserve">false</t>
+        </is>
+      </c>
+      <c r="P118" t="n" s="31">
+        <v>0</v>
+      </c>
     </row>
     <row r="119" ht="22" customHeight="1" s="32">
       <c r="A119" s="31" t="inlineStr">
@@ -23926,6 +24524,14 @@
           <t>75</t>
         </is>
       </c>
+      <c r="O119" t="inlineStr" s="31">
+        <is>
+          <t xml:space="preserve">false</t>
+        </is>
+      </c>
+      <c r="P119" t="n" s="31">
+        <v>0</v>
+      </c>
     </row>
     <row r="120" ht="22" customHeight="1" s="32">
       <c r="A120" s="31" t="inlineStr">
@@ -23994,6 +24600,14 @@
           <t>76</t>
         </is>
       </c>
+      <c r="O120" t="inlineStr" s="31">
+        <is>
+          <t xml:space="preserve">false</t>
+        </is>
+      </c>
+      <c r="P120" t="n" s="31">
+        <v>0</v>
+      </c>
     </row>
     <row r="121" ht="22" customHeight="1" s="32">
       <c r="A121" s="31" t="inlineStr">
@@ -24062,6 +24676,14 @@
           <t>77</t>
         </is>
       </c>
+      <c r="O121" t="inlineStr" s="31">
+        <is>
+          <t xml:space="preserve">false</t>
+        </is>
+      </c>
+      <c r="P121" t="n" s="31">
+        <v>0</v>
+      </c>
     </row>
     <row r="122" ht="22" customHeight="1" s="32">
       <c r="A122" s="31" t="inlineStr">
@@ -24130,6 +24752,14 @@
           <t>78</t>
         </is>
       </c>
+      <c r="O122" t="inlineStr" s="31">
+        <is>
+          <t xml:space="preserve">false</t>
+        </is>
+      </c>
+      <c r="P122" t="n" s="31">
+        <v>0</v>
+      </c>
     </row>
     <row r="123" ht="22" customHeight="1" s="32">
       <c r="A123" s="31" t="inlineStr">
@@ -24197,6 +24827,14 @@
         <is>
           <t>79</t>
         </is>
+      </c>
+      <c r="O123" t="inlineStr" s="31">
+        <is>
+          <t xml:space="preserve">false</t>
+        </is>
+      </c>
+      <c r="P123" t="n" s="31">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -24208,7 +24846,7 @@
     <mergeCell ref="A2:D2"/>
     <mergeCell ref="A44:D44"/>
   </mergeCells>
-  <dataValidations count="23">
+  <dataValidations count="25">
     <dataValidation sqref="C4:C15" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" errorTitle="无效选项" error="只能从下拉列表中选择有效值。" promptTitle="请选择" prompt="请从下拉列表选择，不能输入列表外的值。" type="list" errorStyle="stop">
       <formula1>=DV_Logic_SlotTypes_Enabled</formula1>
     </dataValidation>
@@ -24245,46 +24883,53 @@
     <dataValidation sqref="K46:K123" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" errorTitle="无效选项" error="只能从下拉列表中选择有效值。" promptTitle="请选择" prompt="请从下拉列表选择，不能输入列表外的值。" type="list" errorStyle="stop">
       <formula1>=DV_Logic_Parts_ImplementationStatus</formula1>
     </dataValidation>
-    <dataValidation sqref="Q46:Q55" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" errorTitle="无效选项" error="只能从下拉列表中选择有效值。" promptTitle="请选择" prompt="请从下拉列表选择，不能输入列表外的值。" type="list" errorStyle="stop">
+    <dataValidation sqref="S46:S55" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" errorTitle="无效选项" error="只能从下拉列表中选择有效值。" promptTitle="请选择" prompt="请从下拉列表选择，不能输入列表外的值。" type="list" errorStyle="stop">
       <formula1>INDIRECT("tblParts[PartId]")</formula1>
     </dataValidation>
-    <dataValidation sqref="S46:S55" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" errorTitle="无效选项" error="只能从下拉列表中选择有效值。" promptTitle="请选择" prompt="请从下拉列表选择，不能输入列表外的值。" type="list" errorStyle="stop">
+    <dataValidation sqref="U46:U55" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" errorTitle="无效选项" error="只能从下拉列表中选择有效值。" promptTitle="请选择" prompt="请从下拉列表选择，不能输入列表外的值。" type="list" errorStyle="stop">
       <formula1>=DV_Logic_PartEffects_Trigger</formula1>
     </dataValidation>
-    <dataValidation sqref="T46:T55" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" errorTitle="无效选项" error="只能从下拉列表中选择有效值。" promptTitle="请选择" prompt="请从下拉列表选择，不能输入列表外的值。" type="list" errorStyle="stop">
+    <dataValidation sqref="V46:V55" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" errorTitle="无效选项" error="只能从下拉列表中选择有效值。" promptTitle="请选择" prompt="请从下拉列表选择，不能输入列表外的值。" type="list" errorStyle="stop">
       <formula1>=DV_Logic_PartEffects_EffectKind</formula1>
     </dataValidation>
-    <dataValidation sqref="U46:U55" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" errorTitle="无效选项" error="只能从下拉列表中选择有效值。" promptTitle="请选择" prompt="请从下拉列表选择，不能输入列表外的值。" type="list" errorStyle="stop">
+    <dataValidation sqref="W46:W55" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" errorTitle="无效选项" error="只能从下拉列表中选择有效值。" promptTitle="请选择" prompt="请从下拉列表选择，不能输入列表外的值。" type="list" errorStyle="stop">
       <formula1>=DV_Logic_PartEffects_Target</formula1>
     </dataValidation>
-    <dataValidation sqref="V46:V55" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" errorTitle="无效选项" error="只能从下拉列表中选择有效值。" promptTitle="请选择" prompt="请从下拉列表选择，不能输入列表外的值。" type="list" errorStyle="stop">
+    <dataValidation sqref="X46:X55" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" errorTitle="无效选项" error="只能从下拉列表中选择有效值。" promptTitle="请选择" prompt="请从下拉列表选择，不能输入列表外的值。" type="list" errorStyle="stop">
       <formula1>=DV_Logic_PartEffects_ValueOp</formula1>
     </dataValidation>
-    <dataValidation sqref="X46:X55" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" errorTitle="无效选项" error="只能从下拉列表中选择有效值。" promptTitle="请选择" prompt="请从下拉列表选择，不能输入列表外的值。" type="list" errorStyle="stop">
+    <dataValidation sqref="Z46:Z55" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" errorTitle="无效选项" error="只能从下拉列表中选择有效值。" promptTitle="请选择" prompt="请从下拉列表选择，不能输入列表外的值。" type="list" errorStyle="stop">
       <formula1>=DV_Logic_PartEffects_BehaviorId</formula1>
     </dataValidation>
-    <dataValidation sqref="Y46:Y55" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" errorTitle="无效选项" error="只能从下拉列表中选择有效值。" promptTitle="请选择" prompt="请从下拉列表选择，不能输入列表外的值。" type="list" errorStyle="stop">
+    <dataValidation sqref="AA46:AA55" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" errorTitle="无效选项" error="只能从下拉列表中选择有效值。" promptTitle="请选择" prompt="请从下拉列表选择，不能输入列表外的值。" type="list" errorStyle="stop">
       <formula1>=DV_Logic_PartEffects_FormulaId</formula1>
     </dataValidation>
-    <dataValidation sqref="Z46:Z55" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" errorTitle="无效选项" error="只能从下拉列表中选择有效值。" promptTitle="请选择" prompt="请从下拉列表选择，不能输入列表外的值。" type="list" errorStyle="stop">
+    <dataValidation sqref="AB46:AB55" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" errorTitle="无效选项" error="只能从下拉列表中选择有效值。" promptTitle="请选择" prompt="请从下拉列表选择，不能输入列表外的值。" type="list" errorStyle="stop">
       <formula1>=DV_Logic_PartEffects_AttackPatternId</formula1>
     </dataValidation>
-    <dataValidation sqref="AA46:AA55" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" errorTitle="无效选项" error="只能从下拉列表中选择有效值。" promptTitle="请选择" prompt="请从下拉列表选择，不能输入列表外的值。" type="list" errorStyle="stop">
+    <dataValidation sqref="AC46:AC55" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" errorTitle="无效选项" error="只能从下拉列表中选择有效值。" promptTitle="请选择" prompt="请从下拉列表选择，不能输入列表外的值。" type="list" errorStyle="stop">
       <formula1>=DV_Logic_PartEffects_ParamName</formula1>
     </dataValidation>
-    <dataValidation sqref="AE46:AE55" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" errorTitle="无效选项" error="只能从下拉列表中选择有效值。" promptTitle="请选择" prompt="请从下拉列表选择，不能输入列表外的值。" type="list" errorStyle="stop">
+    <dataValidation sqref="AG46:AG55" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" errorTitle="无效选项" error="只能从下拉列表中选择有效值。" promptTitle="请选择" prompt="请从下拉列表选择，不能输入列表外的值。" type="list" errorStyle="stop">
       <formula1>=DV_Logic_PartEffects_StackPolicy</formula1>
     </dataValidation>
-    <dataValidation sqref="AF46:AF55" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" errorTitle="无效选项" error="只能从下拉列表中选择有效值。" promptTitle="请选择" prompt="请从下拉列表选择，不能输入列表外的值。" type="list" errorStyle="stop">
+    <dataValidation sqref="AH46:AH55" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" errorTitle="无效选项" error="只能从下拉列表中选择有效值。" promptTitle="请选择" prompt="请从下拉列表选择，不能输入列表外的值。" type="list" errorStyle="stop">
       <formula1>=DV_Logic_PartEffects_Enabled</formula1>
+    </dataValidation>
+    <dataValidation sqref="O46:O123" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" errorTitle="无效选项" error="只能从下拉列表中选择有效值。" promptTitle="请选择" prompt="请从下拉列表选择，不能输入列表外的值。" type="list" errorStyle="stop">
+      <formula1>=DV_Logic_Parts_Enabled</formula1>
+    </dataValidation>
+    <dataValidation sqref="P46:P123" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" type="whole" operator="between" errorStyle="stop" errorTitle="无效数值" error="请输入 0 到 100000 之间的整数。" promptTitle="商店价格" prompt="未上架填 0；上架符文必须填写正整数价格。">
+      <formula1>0</formula1>
+      <formula2>100000</formula2>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="4">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
+    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
+    <tablePart r:id="rId3"/>
+    <tablePart r:id="rId4"/>
   </tableParts>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
[PROGRAMMER] Plan56: attribute panel on shop clock hover (data-driven Attributes domain)
</commit_message>
<xml_diff>
--- a/Design/Data/ReEchoData.xlsx
+++ b/Design/Data/ReEchoData.xlsx
@@ -15,6 +15,7 @@
     <sheet name="_WorkbookMeta" sheetId="10" state="visible" r:id="rId10"/>
     <sheet name="_ExportMap" sheetId="11" state="visible" r:id="rId11"/>
     <sheet name="_SystemData" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="AttributeCatalog" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames>
     <definedName name="DV_Logic_Elements_Id">'_SystemData'!$R$2:$R$5</definedName>
@@ -97,7 +98,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode=";;;"/>
   </numFmts>
-  <fonts count="15">
+  <fonts count="16">
     <font>
       <name val="等线"/>
       <color theme="1"/>
@@ -169,6 +170,9 @@
     </font>
     <font>
       <color rgb="FFFFFFFF"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="11">
@@ -247,7 +251,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -361,6 +365,10 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <protection locked="0" hidden="0"/>
     </xf>
   </cellXfs>
@@ -576,7 +584,7 @@
 </file>
 
 <file path=xl/tables/table16.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="16" name="tblExportMap" displayName="tblExportMap" ref="A1:E17" headerRowCount="1" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="16" name="tblExportMap" displayName="tblExportMap" ref="A1:E18" headerRowCount="1" totalsRowShown="0">
   <tableColumns count="5">
     <tableColumn id="1" name="SheetName"/>
     <tableColumn id="2" name="TableName"/>
@@ -616,6 +624,22 @@
     <tableColumn id="5" name="Value"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table19.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="19" name="tblAttributes" displayName="tblAttributes" ref="A1:G9" headerRowCount="1">
+  <autoFilter ref="A1:G9"/>
+  <tableColumns count="7">
+    <tableColumn id="1" name="Id"/>
+    <tableColumn id="2" name="DisplayName"/>
+    <tableColumn id="3" name="Tier"/>
+    <tableColumn id="4" name="IconName"/>
+    <tableColumn id="5" name="ValueKind"/>
+    <tableColumn id="6" name="DisplayOrder"/>
+    <tableColumn id="7" name="Explanation"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
 </table>
 </file>
 
@@ -2620,7 +2644,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:E18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13"/>
   <cols>
     <col width="13" customWidth="1" style="28" min="1" max="1"/>
@@ -3086,6 +3110,33 @@
       <c r="E17" s="31" t="inlineStr">
         <is>
           <t>16</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>AttributeCatalog</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>tblAttributes</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>attributes.csv</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>100</t>
         </is>
       </c>
     </row>
@@ -5591,6 +5642,327 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00FFC000"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="39" t="inlineStr">
+        <is>
+          <t>Id</t>
+        </is>
+      </c>
+      <c r="B1" s="39" t="inlineStr">
+        <is>
+          <t>DisplayName</t>
+        </is>
+      </c>
+      <c r="C1" s="39" t="inlineStr">
+        <is>
+          <t>Tier</t>
+        </is>
+      </c>
+      <c r="D1" s="39" t="inlineStr">
+        <is>
+          <t>IconName</t>
+        </is>
+      </c>
+      <c r="E1" s="39" t="inlineStr">
+        <is>
+          <t>ValueKind</t>
+        </is>
+      </c>
+      <c r="F1" s="39" t="inlineStr">
+        <is>
+          <t>DisplayOrder</t>
+        </is>
+      </c>
+      <c r="G1" s="39" t="inlineStr">
+        <is>
+          <t>Explanation</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="40" t="inlineStr">
+        <is>
+          <t>S_HP</t>
+        </is>
+      </c>
+      <c r="B2" s="40" t="inlineStr">
+        <is>
+          <t>生命值</t>
+        </is>
+      </c>
+      <c r="C2" s="40" t="n">
+        <v>1</v>
+      </c>
+      <c r="D2" s="40" t="inlineStr">
+        <is>
+          <t>生命值</t>
+        </is>
+      </c>
+      <c r="E2" s="40" t="inlineStr">
+        <is>
+          <t>Absolute</t>
+        </is>
+      </c>
+      <c r="F2" s="40" t="n">
+        <v>1</v>
+      </c>
+      <c r="G2" s="40" t="inlineStr">
+        <is>
+          <t>角色受到伤害的承受上限</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="40" t="inlineStr">
+        <is>
+          <t>S_P_Attack_Power</t>
+        </is>
+      </c>
+      <c r="B3" s="40" t="inlineStr">
+        <is>
+          <t>物理攻击力</t>
+        </is>
+      </c>
+      <c r="C3" s="40" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3" s="40" t="inlineStr">
+        <is>
+          <t>物理攻击力</t>
+        </is>
+      </c>
+      <c r="E3" s="40" t="inlineStr">
+        <is>
+          <t>Absolute</t>
+        </is>
+      </c>
+      <c r="F3" s="40" t="n">
+        <v>2</v>
+      </c>
+      <c r="G3" s="40" t="inlineStr">
+        <is>
+          <t>物理系攻击加值</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="40" t="inlineStr">
+        <is>
+          <t>S_E_Attack_Power</t>
+        </is>
+      </c>
+      <c r="B4" s="40" t="inlineStr">
+        <is>
+          <t>元素攻击力</t>
+        </is>
+      </c>
+      <c r="C4" s="40" t="n">
+        <v>1</v>
+      </c>
+      <c r="D4" s="40" t="inlineStr">
+        <is>
+          <t>元素攻击力</t>
+        </is>
+      </c>
+      <c r="E4" s="40" t="inlineStr">
+        <is>
+          <t>Absolute</t>
+        </is>
+      </c>
+      <c r="F4" s="40" t="n">
+        <v>3</v>
+      </c>
+      <c r="G4" s="40" t="inlineStr">
+        <is>
+          <t>元素系攻击加值</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="40" t="inlineStr">
+        <is>
+          <t>S_Movement_Speed</t>
+        </is>
+      </c>
+      <c r="B5" s="40" t="inlineStr">
+        <is>
+          <t>移动速度</t>
+        </is>
+      </c>
+      <c r="C5" s="40" t="n">
+        <v>2</v>
+      </c>
+      <c r="D5" s="40" t="inlineStr">
+        <is>
+          <t>移动速度</t>
+        </is>
+      </c>
+      <c r="E5" s="40" t="inlineStr">
+        <is>
+          <t>Percent</t>
+        </is>
+      </c>
+      <c r="F5" s="40" t="n">
+        <v>4</v>
+      </c>
+      <c r="G5" s="40" t="inlineStr">
+        <is>
+          <t>角色移动速度（以百分比表示）</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="40" t="inlineStr">
+        <is>
+          <t>S_Critical_Hit_Rate</t>
+        </is>
+      </c>
+      <c r="B6" s="40" t="inlineStr">
+        <is>
+          <t>暴击率</t>
+        </is>
+      </c>
+      <c r="C6" s="40" t="n">
+        <v>2</v>
+      </c>
+      <c r="D6" s="40" t="inlineStr">
+        <is>
+          <t>暴击率</t>
+        </is>
+      </c>
+      <c r="E6" s="40" t="inlineStr">
+        <is>
+          <t>Percent</t>
+        </is>
+      </c>
+      <c r="F6" s="40" t="n">
+        <v>5</v>
+      </c>
+      <c r="G6" s="40" t="inlineStr">
+        <is>
+          <t>触发暴击的概率</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="40" t="inlineStr">
+        <is>
+          <t>S_Critical_Hit_Effect</t>
+        </is>
+      </c>
+      <c r="B7" s="40" t="inlineStr">
+        <is>
+          <t>暴击效果</t>
+        </is>
+      </c>
+      <c r="C7" s="40" t="n">
+        <v>2</v>
+      </c>
+      <c r="D7" s="40" t="inlineStr">
+        <is>
+          <t>暴击效果</t>
+        </is>
+      </c>
+      <c r="E7" s="40" t="inlineStr">
+        <is>
+          <t>Percent</t>
+        </is>
+      </c>
+      <c r="F7" s="40" t="n">
+        <v>6</v>
+      </c>
+      <c r="G7" s="40" t="inlineStr">
+        <is>
+          <t>暴击造成的额外伤害比例</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="40" t="inlineStr">
+        <is>
+          <t>S_Echo_Efficiency</t>
+        </is>
+      </c>
+      <c r="B8" s="40" t="inlineStr">
+        <is>
+          <t>回响效能</t>
+        </is>
+      </c>
+      <c r="C8" s="40" t="n">
+        <v>2</v>
+      </c>
+      <c r="D8" s="40" t="inlineStr">
+        <is>
+          <t>回响效能</t>
+        </is>
+      </c>
+      <c r="E8" s="40" t="inlineStr">
+        <is>
+          <t>Percent</t>
+        </is>
+      </c>
+      <c r="F8" s="40" t="n">
+        <v>7</v>
+      </c>
+      <c r="G8" s="40" t="inlineStr">
+        <is>
+          <t>回响造成的伤害效率</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="40" t="inlineStr">
+        <is>
+          <t>S_Elemental_Reaction_Efficiency</t>
+        </is>
+      </c>
+      <c r="B9" s="40" t="inlineStr">
+        <is>
+          <t>元素反应效能</t>
+        </is>
+      </c>
+      <c r="C9" s="40" t="n">
+        <v>2</v>
+      </c>
+      <c r="D9" s="40" t="inlineStr">
+        <is>
+          <t>元素反应效能</t>
+        </is>
+      </c>
+      <c r="E9" s="40" t="inlineStr">
+        <is>
+          <t>Percent</t>
+        </is>
+      </c>
+      <c r="F9" s="40" t="n">
+        <v>8</v>
+      </c>
+      <c r="G9" s="40" t="inlineStr">
+        <is>
+          <t>元素反应造成的效率</t>
+        </is>
+      </c>
+    </row>
+    <row r="10"/>
+  </sheetData>
+  <sheetProtection selectLockedCells="1" selectUnlockedCells="1" sheet="1" objects="0" insertRows="0" insertHyperlinks="1" autoFilter="0" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="0" formatCells="0" formatRows="1" sort="0"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -5878,9 +6250,6 @@
       </c>
       <c r="J7" s="37" t="n"/>
     </row>
-    <row r="8"/>
-    <row r="9"/>
-    <row r="10"/>
     <row r="11" ht="25" customHeight="1" s="32">
       <c r="A11" s="34" t="inlineStr">
         <is>
@@ -9471,7 +9840,6 @@
       </c>
       <c r="N45" s="37" t="n"/>
     </row>
-    <row r="46"/>
     <row r="47" ht="25" customHeight="1" s="32">
       <c r="A47" s="34" t="inlineStr">
         <is>
@@ -13013,8 +13381,6 @@
       <c r="V8" s="31" t="n"/>
       <c r="W8" s="31" t="n"/>
     </row>
-    <row r="9"/>
-    <row r="10"/>
     <row r="11" ht="25" customHeight="1" s="32">
       <c r="A11" s="34" t="inlineStr">
         <is>
@@ -13912,8 +14278,6 @@
       </c>
       <c r="P10" s="37" t="n"/>
     </row>
-    <row r="11"/>
-    <row r="12"/>
     <row r="13" ht="25" customHeight="1" s="32">
       <c r="A13" s="34" t="inlineStr">
         <is>
@@ -14646,8 +15010,6 @@
       </c>
       <c r="U20" s="37" t="n"/>
     </row>
-    <row r="21"/>
-    <row r="22"/>
     <row r="23" ht="25" customHeight="1" s="32">
       <c r="A23" s="34" t="inlineStr">
         <is>
@@ -16625,7 +16987,6 @@
       </c>
       <c r="F15" s="37" t="n"/>
     </row>
-    <row r="16"/>
     <row r="17" ht="25" customHeight="1" s="32">
       <c r="A17" s="34" t="inlineStr">
         <is>
@@ -17583,10 +17944,6 @@
       </c>
       <c r="I39" s="37" t="n"/>
     </row>
-    <row r="40"/>
-    <row r="41"/>
-    <row r="42"/>
-    <row r="43"/>
     <row r="44" ht="25" customHeight="1" s="32">
       <c r="A44" s="34" t="inlineStr">
         <is>
@@ -24852,8 +25209,6 @@
         </is>
       </c>
     </row>
-    <row r="5"/>
-    <row r="6"/>
     <row r="7">
       <c r="B7" s="1" t="inlineStr">
         <is>
@@ -25452,7 +25807,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1"/>
+  <dimension ref="L1:L1"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="13.81640625" defaultRowHeight="13"/>
   <sheetData>
     <row r="1" ht="39" customHeight="1" s="32">

</xml_diff>

<commit_message>
[PROGRAMMER] Plan67: weapon parameter StatModifier effects + runtime guard alignment
- ReEchoWeaponRuntime: land AttackRange/AttackArc/ProjectileCount/ConcentrationDegrees/
  ExplosionRadius as RuleFlags (StatModifier) and read them back in
  BuildEffectiveWeaponDefinition, with FMath::Max/Clamp guards.
- Runtime CSV loader: align AllowedTargets with validate WEAPON_EFFECT_TARGETS and
  register StatModifier EffectKind; relax the 10-named/60-unnamed audit to the same
  guard as the validator (every row named or inert unnamed placeholder).
- xlsx backfill: 15 named+enabled parts and 31 effects; regenerate CSVs.
- validate_project.py: WEAPON_EFFECT_TARGETS +5, EffectKind one-to-many, audit guard.
</commit_message>
<xml_diff>
--- a/Design/Data/ReEchoData.xlsx
+++ b/Design/Data/ReEchoData.xlsx
@@ -525,7 +525,7 @@
 </file>
 
 <file path=xl/tables/table13.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="13" name="tblPartEffects" displayName="tblPartEffects" ref="R45:AK51" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="13" name="tblPartEffects" displayName="tblPartEffects" ref="R45:AK82" headerRowCount="1">
   <autoFilter ref="R45:AK55"/>
   <tableColumns count="20">
     <tableColumn id="16" name="Id"/>
@@ -18635,26 +18635,90 @@
           <t>0</t>
         </is>
       </c>
-      <c r="R52" s="31" t="n"/>
-      <c r="S52" s="31" t="n"/>
-      <c r="T52" s="31" t="n"/>
-      <c r="U52" s="31" t="n"/>
-      <c r="V52" s="31" t="n"/>
-      <c r="W52" s="31" t="n"/>
-      <c r="X52" s="31" t="n"/>
-      <c r="Y52" s="31" t="n"/>
-      <c r="Z52" s="31" t="n"/>
-      <c r="AA52" s="31" t="n"/>
-      <c r="AB52" s="31" t="n"/>
-      <c r="AC52" s="31" t="n"/>
-      <c r="AD52" s="31" t="n"/>
-      <c r="AE52" s="31" t="n"/>
-      <c r="AF52" s="31" t="n"/>
-      <c r="AG52" s="31" t="n"/>
-      <c r="AH52" s="31" t="n"/>
-      <c r="AI52" s="31" t="n"/>
-      <c r="AJ52" s="31" t="n"/>
-      <c r="AK52" s="31" t="n"/>
+      <c r="R52" s="37" t="inlineStr">
+        <is>
+          <t>PE_BOW_HASTE_BOWSTRING_1</t>
+        </is>
+      </c>
+      <c r="S52" s="37" t="inlineStr">
+        <is>
+          <t>P_BOW_HASTE_BOWSTRING</t>
+        </is>
+      </c>
+      <c r="T52" s="37" t="n">
+        <v>1</v>
+      </c>
+      <c r="U52" s="37" t="inlineStr">
+        <is>
+          <t>OnEquip</t>
+        </is>
+      </c>
+      <c r="V52" s="37" t="inlineStr">
+        <is>
+          <t>StatModifier</t>
+        </is>
+      </c>
+      <c r="W52" s="37" t="inlineStr">
+        <is>
+          <t>AttackSpeed</t>
+        </is>
+      </c>
+      <c r="X52" s="37" t="inlineStr">
+        <is>
+          <t>Multiply</t>
+        </is>
+      </c>
+      <c r="Y52" s="37" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="Z52" s="37" t="inlineStr">
+        <is>
+          <t>Part.StatModifier</t>
+        </is>
+      </c>
+      <c r="AA52" s="37" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="AB52" s="37" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="AC52" s="37" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="AD52" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE52" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF52" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG52" s="37" t="inlineStr">
+        <is>
+          <t>Unique</t>
+        </is>
+      </c>
+      <c r="AH52" s="37" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="AI52" s="37" t="n"/>
+      <c r="AJ52" s="37" t="inlineStr">
+        <is>
+          <t>武器插槽C</t>
+        </is>
+      </c>
+      <c r="AK52" s="37" t="n">
+        <v>22</v>
+      </c>
     </row>
     <row r="53" ht="22" customHeight="1" s="32">
       <c r="A53" s="37" t="inlineStr">
@@ -18737,26 +18801,90 @@
           <t>0</t>
         </is>
       </c>
-      <c r="R53" s="31" t="n"/>
-      <c r="S53" s="31" t="n"/>
-      <c r="T53" s="31" t="n"/>
-      <c r="U53" s="31" t="n"/>
-      <c r="V53" s="31" t="n"/>
-      <c r="W53" s="31" t="n"/>
-      <c r="X53" s="31" t="n"/>
-      <c r="Y53" s="31" t="n"/>
-      <c r="Z53" s="31" t="n"/>
-      <c r="AA53" s="31" t="n"/>
-      <c r="AB53" s="31" t="n"/>
-      <c r="AC53" s="31" t="n"/>
-      <c r="AD53" s="31" t="n"/>
-      <c r="AE53" s="31" t="n"/>
-      <c r="AF53" s="31" t="n"/>
-      <c r="AG53" s="31" t="n"/>
-      <c r="AH53" s="31" t="n"/>
-      <c r="AI53" s="31" t="n"/>
-      <c r="AJ53" s="31" t="n"/>
-      <c r="AK53" s="31" t="n"/>
+      <c r="R53" s="37" t="inlineStr">
+        <is>
+          <t>PE_BOW_HASTE_BOWSTRING_2</t>
+        </is>
+      </c>
+      <c r="S53" s="37" t="inlineStr">
+        <is>
+          <t>P_BOW_HASTE_BOWSTRING</t>
+        </is>
+      </c>
+      <c r="T53" s="37" t="n">
+        <v>2</v>
+      </c>
+      <c r="U53" s="37" t="inlineStr">
+        <is>
+          <t>OnEquip</t>
+        </is>
+      </c>
+      <c r="V53" s="37" t="inlineStr">
+        <is>
+          <t>StatModifier</t>
+        </is>
+      </c>
+      <c r="W53" s="37" t="inlineStr">
+        <is>
+          <t>PhysicalCoefficient</t>
+        </is>
+      </c>
+      <c r="X53" s="37" t="inlineStr">
+        <is>
+          <t>Multiply</t>
+        </is>
+      </c>
+      <c r="Y53" s="37" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="Z53" s="37" t="inlineStr">
+        <is>
+          <t>Part.StatModifier</t>
+        </is>
+      </c>
+      <c r="AA53" s="37" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="AB53" s="37" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="AC53" s="37" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="AD53" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE53" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF53" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG53" s="37" t="inlineStr">
+        <is>
+          <t>Unique</t>
+        </is>
+      </c>
+      <c r="AH53" s="37" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="AI53" s="37" t="n"/>
+      <c r="AJ53" s="37" t="inlineStr">
+        <is>
+          <t>武器插槽C</t>
+        </is>
+      </c>
+      <c r="AK53" s="37" t="n">
+        <v>22</v>
+      </c>
     </row>
     <row r="54" ht="22" customHeight="1" s="32">
       <c r="A54" s="37" t="inlineStr">
@@ -18839,26 +18967,90 @@
           <t>0</t>
         </is>
       </c>
-      <c r="R54" s="31" t="n"/>
-      <c r="S54" s="31" t="n"/>
-      <c r="T54" s="31" t="n"/>
-      <c r="U54" s="31" t="n"/>
-      <c r="V54" s="31" t="n"/>
-      <c r="W54" s="31" t="n"/>
-      <c r="X54" s="31" t="n"/>
-      <c r="Y54" s="31" t="n"/>
-      <c r="Z54" s="31" t="n"/>
-      <c r="AA54" s="31" t="n"/>
-      <c r="AB54" s="31" t="n"/>
-      <c r="AC54" s="31" t="n"/>
-      <c r="AD54" s="31" t="n"/>
-      <c r="AE54" s="31" t="n"/>
-      <c r="AF54" s="31" t="n"/>
-      <c r="AG54" s="31" t="n"/>
-      <c r="AH54" s="31" t="n"/>
-      <c r="AI54" s="31" t="n"/>
-      <c r="AJ54" s="31" t="n"/>
-      <c r="AK54" s="31" t="n"/>
+      <c r="R54" s="37" t="inlineStr">
+        <is>
+          <t>PE_BOW_HASTE_BOWSTRING_3</t>
+        </is>
+      </c>
+      <c r="S54" s="37" t="inlineStr">
+        <is>
+          <t>P_BOW_HASTE_BOWSTRING</t>
+        </is>
+      </c>
+      <c r="T54" s="37" t="n">
+        <v>3</v>
+      </c>
+      <c r="U54" s="37" t="inlineStr">
+        <is>
+          <t>OnEquip</t>
+        </is>
+      </c>
+      <c r="V54" s="37" t="inlineStr">
+        <is>
+          <t>StatModifier</t>
+        </is>
+      </c>
+      <c r="W54" s="37" t="inlineStr">
+        <is>
+          <t>ElementalCoefficient</t>
+        </is>
+      </c>
+      <c r="X54" s="37" t="inlineStr">
+        <is>
+          <t>Multiply</t>
+        </is>
+      </c>
+      <c r="Y54" s="37" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="Z54" s="37" t="inlineStr">
+        <is>
+          <t>Part.StatModifier</t>
+        </is>
+      </c>
+      <c r="AA54" s="37" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="AB54" s="37" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="AC54" s="37" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="AD54" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE54" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF54" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG54" s="37" t="inlineStr">
+        <is>
+          <t>Unique</t>
+        </is>
+      </c>
+      <c r="AH54" s="37" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="AI54" s="37" t="n"/>
+      <c r="AJ54" s="37" t="inlineStr">
+        <is>
+          <t>武器插槽C</t>
+        </is>
+      </c>
+      <c r="AK54" s="37" t="n">
+        <v>22</v>
+      </c>
     </row>
     <row r="55" ht="22" customHeight="1" s="32">
       <c r="A55" s="37" t="inlineStr">
@@ -18937,26 +19129,90 @@
           <t>0</t>
         </is>
       </c>
-      <c r="R55" s="31" t="n"/>
-      <c r="S55" s="31" t="n"/>
-      <c r="T55" s="31" t="n"/>
-      <c r="U55" s="31" t="n"/>
-      <c r="V55" s="31" t="n"/>
-      <c r="W55" s="31" t="n"/>
-      <c r="X55" s="31" t="n"/>
-      <c r="Y55" s="31" t="n"/>
-      <c r="Z55" s="31" t="n"/>
-      <c r="AA55" s="31" t="n"/>
-      <c r="AB55" s="31" t="n"/>
-      <c r="AC55" s="31" t="n"/>
-      <c r="AD55" s="31" t="n"/>
-      <c r="AE55" s="31" t="n"/>
-      <c r="AF55" s="31" t="n"/>
-      <c r="AG55" s="31" t="n"/>
-      <c r="AH55" s="31" t="n"/>
-      <c r="AI55" s="31" t="n"/>
-      <c r="AJ55" s="31" t="n"/>
-      <c r="AK55" s="31" t="n"/>
+      <c r="R55" s="37" t="inlineStr">
+        <is>
+          <t>PE_BOW_HEAVY_BOWSTRING_1</t>
+        </is>
+      </c>
+      <c r="S55" s="37" t="inlineStr">
+        <is>
+          <t>P_BOW_HEAVY_BOWSTRING</t>
+        </is>
+      </c>
+      <c r="T55" s="37" t="n">
+        <v>1</v>
+      </c>
+      <c r="U55" s="37" t="inlineStr">
+        <is>
+          <t>OnEquip</t>
+        </is>
+      </c>
+      <c r="V55" s="37" t="inlineStr">
+        <is>
+          <t>StatModifier</t>
+        </is>
+      </c>
+      <c r="W55" s="37" t="inlineStr">
+        <is>
+          <t>AttackSpeed</t>
+        </is>
+      </c>
+      <c r="X55" s="37" t="inlineStr">
+        <is>
+          <t>Multiply</t>
+        </is>
+      </c>
+      <c r="Y55" s="37" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="Z55" s="37" t="inlineStr">
+        <is>
+          <t>Part.StatModifier</t>
+        </is>
+      </c>
+      <c r="AA55" s="37" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="AB55" s="37" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="AC55" s="37" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="AD55" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE55" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF55" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG55" s="37" t="inlineStr">
+        <is>
+          <t>Unique</t>
+        </is>
+      </c>
+      <c r="AH55" s="37" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="AI55" s="37" t="n"/>
+      <c r="AJ55" s="37" t="inlineStr">
+        <is>
+          <t>武器插槽C</t>
+        </is>
+      </c>
+      <c r="AK55" s="37" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="56" ht="22" customHeight="1" s="32">
       <c r="A56" s="37" t="inlineStr">
@@ -19039,6 +19295,90 @@
           <t>0</t>
         </is>
       </c>
+      <c r="R56" s="37" t="inlineStr">
+        <is>
+          <t>PE_BOW_HEAVY_BOWSTRING_2</t>
+        </is>
+      </c>
+      <c r="S56" s="37" t="inlineStr">
+        <is>
+          <t>P_BOW_HEAVY_BOWSTRING</t>
+        </is>
+      </c>
+      <c r="T56" s="37" t="n">
+        <v>2</v>
+      </c>
+      <c r="U56" s="37" t="inlineStr">
+        <is>
+          <t>OnEquip</t>
+        </is>
+      </c>
+      <c r="V56" s="37" t="inlineStr">
+        <is>
+          <t>StatModifier</t>
+        </is>
+      </c>
+      <c r="W56" s="37" t="inlineStr">
+        <is>
+          <t>PhysicalCoefficient</t>
+        </is>
+      </c>
+      <c r="X56" s="37" t="inlineStr">
+        <is>
+          <t>Multiply</t>
+        </is>
+      </c>
+      <c r="Y56" s="37" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="Z56" s="37" t="inlineStr">
+        <is>
+          <t>Part.StatModifier</t>
+        </is>
+      </c>
+      <c r="AA56" s="37" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="AB56" s="37" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="AC56" s="37" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="AD56" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE56" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF56" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG56" s="37" t="inlineStr">
+        <is>
+          <t>Unique</t>
+        </is>
+      </c>
+      <c r="AH56" s="37" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="AI56" s="37" t="n"/>
+      <c r="AJ56" s="37" t="inlineStr">
+        <is>
+          <t>武器插槽C</t>
+        </is>
+      </c>
+      <c r="AK56" s="37" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="57" ht="22" customHeight="1" s="32">
       <c r="A57" s="37" t="inlineStr">
@@ -19117,16 +19457,100 @@
           <t>0</t>
         </is>
       </c>
+      <c r="R57" s="37" t="inlineStr">
+        <is>
+          <t>PE_BOW_HEAVY_BOWSTRING_3</t>
+        </is>
+      </c>
+      <c r="S57" s="37" t="inlineStr">
+        <is>
+          <t>P_BOW_HEAVY_BOWSTRING</t>
+        </is>
+      </c>
+      <c r="T57" s="37" t="n">
+        <v>3</v>
+      </c>
+      <c r="U57" s="37" t="inlineStr">
+        <is>
+          <t>OnEquip</t>
+        </is>
+      </c>
+      <c r="V57" s="37" t="inlineStr">
+        <is>
+          <t>StatModifier</t>
+        </is>
+      </c>
+      <c r="W57" s="37" t="inlineStr">
+        <is>
+          <t>ElementalCoefficient</t>
+        </is>
+      </c>
+      <c r="X57" s="37" t="inlineStr">
+        <is>
+          <t>Multiply</t>
+        </is>
+      </c>
+      <c r="Y57" s="37" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="Z57" s="37" t="inlineStr">
+        <is>
+          <t>Part.StatModifier</t>
+        </is>
+      </c>
+      <c r="AA57" s="37" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="AB57" s="37" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="AC57" s="37" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="AD57" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE57" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF57" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG57" s="37" t="inlineStr">
+        <is>
+          <t>Unique</t>
+        </is>
+      </c>
+      <c r="AH57" s="37" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="AI57" s="37" t="n"/>
+      <c r="AJ57" s="37" t="inlineStr">
+        <is>
+          <t>武器插槽C</t>
+        </is>
+      </c>
+      <c r="AK57" s="37" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="58" ht="22" customHeight="1" s="32">
       <c r="A58" s="37" t="inlineStr">
         <is>
-          <t>AUDIT_WEAPON_SLOTS_C_22</t>
+          <t>P_BOW_HASTE_BOWSTRING</t>
         </is>
       </c>
       <c r="B58" s="37" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>P_BOW_HASTE_BOWSTRING</t>
         </is>
       </c>
       <c r="C58" s="37" t="inlineStr">
@@ -19139,7 +19563,11 @@
           <t>Bowstring</t>
         </is>
       </c>
-      <c r="E58" s="37" t="n"/>
+      <c r="E58" s="37" t="inlineStr">
+        <is>
+          <t>攻速弓弦</t>
+        </is>
+      </c>
       <c r="F58" s="37" t="inlineStr">
         <is>
           <t>效果：攻击速度+60%，伤害倍率-40%</t>
@@ -19147,34 +19575,30 @@
       </c>
       <c r="G58" s="37" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Common</t>
         </is>
       </c>
       <c r="H58" s="37" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Bowstring|Numeric</t>
         </is>
       </c>
       <c r="I58" s="37" t="inlineStr">
         <is>
-          <t>false</t>
+          <t>true</t>
         </is>
       </c>
       <c r="J58" s="37" t="inlineStr">
         <is>
-          <t>Unimplemented</t>
+          <t>Approved</t>
         </is>
       </c>
       <c r="K58" s="37" t="inlineStr">
         <is>
-          <t>Disabled</t>
-        </is>
-      </c>
-      <c r="L58" s="37" t="inlineStr">
-        <is>
-          <t>Unnamed workbook row; no stable PartId assigned.</t>
-        </is>
-      </c>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="L58" s="37" t="n"/>
       <c r="M58" s="37" t="inlineStr">
         <is>
           <t>武器插槽C</t>
@@ -19187,24 +19611,106 @@
       </c>
       <c r="O58" s="37" t="inlineStr">
         <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="P58" s="37" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="P58" s="37" t="n">
+        <v>30</v>
+      </c>
+      <c r="R58" s="37" t="inlineStr">
+        <is>
+          <t>PE_SCYTHE_HASTE_ROTARYBLADE_1</t>
+        </is>
+      </c>
+      <c r="S58" s="37" t="inlineStr">
+        <is>
+          <t>P_SCYTHE_HASTE_ROTARYBLADE</t>
+        </is>
+      </c>
+      <c r="T58" s="37" t="n">
+        <v>1</v>
+      </c>
+      <c r="U58" s="37" t="inlineStr">
+        <is>
+          <t>OnEquip</t>
+        </is>
+      </c>
+      <c r="V58" s="37" t="inlineStr">
+        <is>
+          <t>StatModifier</t>
+        </is>
+      </c>
+      <c r="W58" s="37" t="inlineStr">
+        <is>
+          <t>AttackSpeed</t>
+        </is>
+      </c>
+      <c r="X58" s="37" t="inlineStr">
+        <is>
+          <t>Multiply</t>
+        </is>
+      </c>
+      <c r="Y58" s="37" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="Z58" s="37" t="inlineStr">
+        <is>
+          <t>Part.StatModifier</t>
+        </is>
+      </c>
+      <c r="AA58" s="37" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="AB58" s="37" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="AC58" s="37" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="AD58" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE58" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF58" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG58" s="37" t="inlineStr">
+        <is>
+          <t>Unique</t>
+        </is>
+      </c>
+      <c r="AH58" s="37" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="AI58" s="37" t="n"/>
+      <c r="AJ58" s="37" t="inlineStr">
+        <is>
+          <t>武器插槽C</t>
+        </is>
+      </c>
+      <c r="AK58" s="37" t="n">
+        <v>28</v>
       </c>
     </row>
     <row r="59" ht="22" customHeight="1" s="32">
       <c r="A59" s="37" t="inlineStr">
         <is>
-          <t>AUDIT_WEAPON_SLOTS_C_23</t>
+          <t>P_BOW_HEAVY_BOWSTRING</t>
         </is>
       </c>
       <c r="B59" s="37" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>P_BOW_HEAVY_BOWSTRING</t>
         </is>
       </c>
       <c r="C59" s="37" t="inlineStr">
@@ -19217,7 +19723,11 @@
           <t>Bowstring</t>
         </is>
       </c>
-      <c r="E59" s="37" t="n"/>
+      <c r="E59" s="37" t="inlineStr">
+        <is>
+          <t>重击弓弦</t>
+        </is>
+      </c>
       <c r="F59" s="37" t="inlineStr">
         <is>
           <t>效果：攻击速度-30%，伤害倍率+50%</t>
@@ -19225,34 +19735,30 @@
       </c>
       <c r="G59" s="37" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Common</t>
         </is>
       </c>
       <c r="H59" s="37" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Bowstring|Numeric</t>
         </is>
       </c>
       <c r="I59" s="37" t="inlineStr">
         <is>
-          <t>false</t>
+          <t>true</t>
         </is>
       </c>
       <c r="J59" s="37" t="inlineStr">
         <is>
-          <t>Unimplemented</t>
+          <t>Approved</t>
         </is>
       </c>
       <c r="K59" s="37" t="inlineStr">
         <is>
-          <t>Disabled</t>
-        </is>
-      </c>
-      <c r="L59" s="37" t="inlineStr">
-        <is>
-          <t>Unnamed workbook row; no stable PartId assigned.</t>
-        </is>
-      </c>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="L59" s="37" t="n"/>
       <c r="M59" s="37" t="inlineStr">
         <is>
           <t>武器插槽C</t>
@@ -19265,13 +19771,95 @@
       </c>
       <c r="O59" s="37" t="inlineStr">
         <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="P59" s="37" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="P59" s="37" t="n">
+        <v>30</v>
+      </c>
+      <c r="R59" s="37" t="inlineStr">
+        <is>
+          <t>PE_SCYTHE_HASTE_ROTARYBLADE_2</t>
+        </is>
+      </c>
+      <c r="S59" s="37" t="inlineStr">
+        <is>
+          <t>P_SCYTHE_HASTE_ROTARYBLADE</t>
+        </is>
+      </c>
+      <c r="T59" s="37" t="n">
+        <v>2</v>
+      </c>
+      <c r="U59" s="37" t="inlineStr">
+        <is>
+          <t>OnEquip</t>
+        </is>
+      </c>
+      <c r="V59" s="37" t="inlineStr">
+        <is>
+          <t>StatModifier</t>
+        </is>
+      </c>
+      <c r="W59" s="37" t="inlineStr">
+        <is>
+          <t>AttackRange</t>
+        </is>
+      </c>
+      <c r="X59" s="37" t="inlineStr">
+        <is>
+          <t>Multiply</t>
+        </is>
+      </c>
+      <c r="Y59" s="37" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="Z59" s="37" t="inlineStr">
+        <is>
+          <t>Part.StatModifier</t>
+        </is>
+      </c>
+      <c r="AA59" s="37" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="AB59" s="37" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="AC59" s="37" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="AD59" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE59" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF59" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG59" s="37" t="inlineStr">
+        <is>
+          <t>Unique</t>
+        </is>
+      </c>
+      <c r="AH59" s="37" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="AI59" s="37" t="n"/>
+      <c r="AJ59" s="37" t="inlineStr">
+        <is>
+          <t>武器插槽C</t>
+        </is>
+      </c>
+      <c r="AK59" s="37" t="n">
+        <v>28</v>
       </c>
     </row>
     <row r="60" ht="30" customHeight="1" s="32">
@@ -19351,6 +19939,90 @@
           <t>0</t>
         </is>
       </c>
+      <c r="R60" s="37" t="inlineStr">
+        <is>
+          <t>PE_LONGSWORD_NARROWWIDE_SWORDBLADE_1</t>
+        </is>
+      </c>
+      <c r="S60" s="37" t="inlineStr">
+        <is>
+          <t>P_LONGSWORD_NARROWWIDE_SWORDBLADE</t>
+        </is>
+      </c>
+      <c r="T60" s="37" t="n">
+        <v>1</v>
+      </c>
+      <c r="U60" s="37" t="inlineStr">
+        <is>
+          <t>OnEquip</t>
+        </is>
+      </c>
+      <c r="V60" s="37" t="inlineStr">
+        <is>
+          <t>StatModifier</t>
+        </is>
+      </c>
+      <c r="W60" s="37" t="inlineStr">
+        <is>
+          <t>AttackArc</t>
+        </is>
+      </c>
+      <c r="X60" s="37" t="inlineStr">
+        <is>
+          <t>Override</t>
+        </is>
+      </c>
+      <c r="Y60" s="37" t="n">
+        <v>120</v>
+      </c>
+      <c r="Z60" s="37" t="inlineStr">
+        <is>
+          <t>Part.StatModifier</t>
+        </is>
+      </c>
+      <c r="AA60" s="37" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="AB60" s="37" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="AC60" s="37" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="AD60" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE60" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF60" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG60" s="37" t="inlineStr">
+        <is>
+          <t>Unique</t>
+        </is>
+      </c>
+      <c r="AH60" s="37" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="AI60" s="37" t="n"/>
+      <c r="AJ60" s="37" t="inlineStr">
+        <is>
+          <t>武器插槽C</t>
+        </is>
+      </c>
+      <c r="AK60" s="37" t="n">
+        <v>36</v>
+      </c>
     </row>
     <row r="61" ht="22" customHeight="1" s="32">
       <c r="A61" s="37" t="inlineStr">
@@ -19429,6 +20101,90 @@
           <t>0</t>
         </is>
       </c>
+      <c r="R61" s="37" t="inlineStr">
+        <is>
+          <t>PE_LONGSWORD_NARROWWIDE_SWORDBLADE_2</t>
+        </is>
+      </c>
+      <c r="S61" s="37" t="inlineStr">
+        <is>
+          <t>P_LONGSWORD_NARROWWIDE_SWORDBLADE</t>
+        </is>
+      </c>
+      <c r="T61" s="37" t="n">
+        <v>2</v>
+      </c>
+      <c r="U61" s="37" t="inlineStr">
+        <is>
+          <t>OnEquip</t>
+        </is>
+      </c>
+      <c r="V61" s="37" t="inlineStr">
+        <is>
+          <t>StatModifier</t>
+        </is>
+      </c>
+      <c r="W61" s="37" t="inlineStr">
+        <is>
+          <t>AttackRange</t>
+        </is>
+      </c>
+      <c r="X61" s="37" t="inlineStr">
+        <is>
+          <t>Multiply</t>
+        </is>
+      </c>
+      <c r="Y61" s="37" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="Z61" s="37" t="inlineStr">
+        <is>
+          <t>Part.StatModifier</t>
+        </is>
+      </c>
+      <c r="AA61" s="37" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="AB61" s="37" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="AC61" s="37" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="AD61" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE61" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF61" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG61" s="37" t="inlineStr">
+        <is>
+          <t>Unique</t>
+        </is>
+      </c>
+      <c r="AH61" s="37" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="AI61" s="37" t="n"/>
+      <c r="AJ61" s="37" t="inlineStr">
+        <is>
+          <t>武器插槽C</t>
+        </is>
+      </c>
+      <c r="AK61" s="37" t="n">
+        <v>36</v>
+      </c>
     </row>
     <row r="62" ht="22" customHeight="1" s="32">
       <c r="A62" s="37" t="inlineStr">
@@ -19507,6 +20263,90 @@
           <t>0</t>
         </is>
       </c>
+      <c r="R62" s="37" t="inlineStr">
+        <is>
+          <t>PE_LONGSWORD_SLOWWIDE_SWORDBLADE_1</t>
+        </is>
+      </c>
+      <c r="S62" s="37" t="inlineStr">
+        <is>
+          <t>P_LONGSWORD_SLOWWIDE_SWORDBLADE</t>
+        </is>
+      </c>
+      <c r="T62" s="37" t="n">
+        <v>1</v>
+      </c>
+      <c r="U62" s="37" t="inlineStr">
+        <is>
+          <t>OnEquip</t>
+        </is>
+      </c>
+      <c r="V62" s="37" t="inlineStr">
+        <is>
+          <t>StatModifier</t>
+        </is>
+      </c>
+      <c r="W62" s="37" t="inlineStr">
+        <is>
+          <t>AttackSpeed</t>
+        </is>
+      </c>
+      <c r="X62" s="37" t="inlineStr">
+        <is>
+          <t>Multiply</t>
+        </is>
+      </c>
+      <c r="Y62" s="37" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="Z62" s="37" t="inlineStr">
+        <is>
+          <t>Part.StatModifier</t>
+        </is>
+      </c>
+      <c r="AA62" s="37" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="AB62" s="37" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="AC62" s="37" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="AD62" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE62" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF62" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG62" s="37" t="inlineStr">
+        <is>
+          <t>Unique</t>
+        </is>
+      </c>
+      <c r="AH62" s="37" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="AI62" s="37" t="n"/>
+      <c r="AJ62" s="37" t="inlineStr">
+        <is>
+          <t>武器插槽C</t>
+        </is>
+      </c>
+      <c r="AK62" s="37" t="n">
+        <v>37</v>
+      </c>
     </row>
     <row r="63" ht="22" customHeight="1" s="32">
       <c r="A63" s="37" t="inlineStr">
@@ -19585,16 +20425,100 @@
           <t>0</t>
         </is>
       </c>
+      <c r="R63" s="37" t="inlineStr">
+        <is>
+          <t>PE_LONGSWORD_SLOWWIDE_SWORDBLADE_2</t>
+        </is>
+      </c>
+      <c r="S63" s="37" t="inlineStr">
+        <is>
+          <t>P_LONGSWORD_SLOWWIDE_SWORDBLADE</t>
+        </is>
+      </c>
+      <c r="T63" s="37" t="n">
+        <v>2</v>
+      </c>
+      <c r="U63" s="37" t="inlineStr">
+        <is>
+          <t>OnEquip</t>
+        </is>
+      </c>
+      <c r="V63" s="37" t="inlineStr">
+        <is>
+          <t>StatModifier</t>
+        </is>
+      </c>
+      <c r="W63" s="37" t="inlineStr">
+        <is>
+          <t>AttackRange</t>
+        </is>
+      </c>
+      <c r="X63" s="37" t="inlineStr">
+        <is>
+          <t>Multiply</t>
+        </is>
+      </c>
+      <c r="Y63" s="37" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="Z63" s="37" t="inlineStr">
+        <is>
+          <t>Part.StatModifier</t>
+        </is>
+      </c>
+      <c r="AA63" s="37" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="AB63" s="37" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="AC63" s="37" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="AD63" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE63" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF63" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG63" s="37" t="inlineStr">
+        <is>
+          <t>Unique</t>
+        </is>
+      </c>
+      <c r="AH63" s="37" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="AI63" s="37" t="n"/>
+      <c r="AJ63" s="37" t="inlineStr">
+        <is>
+          <t>武器插槽C</t>
+        </is>
+      </c>
+      <c r="AK63" s="37" t="n">
+        <v>37</v>
+      </c>
     </row>
     <row r="64" ht="22" customHeight="1" s="32">
       <c r="A64" s="37" t="inlineStr">
         <is>
-          <t>AUDIT_WEAPON_SLOTS_C_28</t>
+          <t>P_SCYTHE_HASTE_ROTARYBLADE</t>
         </is>
       </c>
       <c r="B64" s="37" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>P_SCYTHE_HASTE_ROTARYBLADE</t>
         </is>
       </c>
       <c r="C64" s="37" t="inlineStr">
@@ -19607,7 +20531,11 @@
           <t>RotaryBlade</t>
         </is>
       </c>
-      <c r="E64" s="37" t="n"/>
+      <c r="E64" s="37" t="inlineStr">
+        <is>
+          <t>攻速减范围旋刃</t>
+        </is>
+      </c>
       <c r="F64" s="37" t="inlineStr">
         <is>
           <t>效果：攻击速度+40%，攻击范围-20%</t>
@@ -19615,34 +20543,30 @@
       </c>
       <c r="G64" s="37" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Common</t>
         </is>
       </c>
       <c r="H64" s="37" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>RotaryBlade|Numeric</t>
         </is>
       </c>
       <c r="I64" s="37" t="inlineStr">
         <is>
-          <t>false</t>
+          <t>true</t>
         </is>
       </c>
       <c r="J64" s="37" t="inlineStr">
         <is>
-          <t>Unimplemented</t>
+          <t>Approved</t>
         </is>
       </c>
       <c r="K64" s="37" t="inlineStr">
         <is>
-          <t>Disabled</t>
-        </is>
-      </c>
-      <c r="L64" s="37" t="inlineStr">
-        <is>
-          <t>Unnamed workbook row; no stable PartId assigned.</t>
-        </is>
-      </c>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="L64" s="37" t="n"/>
       <c r="M64" s="37" t="inlineStr">
         <is>
           <t>武器插槽C</t>
@@ -19655,13 +20579,95 @@
       </c>
       <c r="O64" s="37" t="inlineStr">
         <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="P64" s="37" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="P64" s="37" t="n">
+        <v>30</v>
+      </c>
+      <c r="R64" s="37" t="inlineStr">
+        <is>
+          <t>PE_LONGSWORD_KILLHEAL_SWORDBLADE_1</t>
+        </is>
+      </c>
+      <c r="S64" s="37" t="inlineStr">
+        <is>
+          <t>P_LONGSWORD_KILLHEAL_SWORDBLADE</t>
+        </is>
+      </c>
+      <c r="T64" s="37" t="n">
+        <v>1</v>
+      </c>
+      <c r="U64" s="37" t="inlineStr">
+        <is>
+          <t>OnKill</t>
+        </is>
+      </c>
+      <c r="V64" s="37" t="inlineStr">
+        <is>
+          <t>UniqueBehavior</t>
+        </is>
+      </c>
+      <c r="W64" s="37" t="inlineStr">
+        <is>
+          <t>OnKill</t>
+        </is>
+      </c>
+      <c r="X64" s="37" t="inlineStr">
+        <is>
+          <t>Add</t>
+        </is>
+      </c>
+      <c r="Y64" s="37" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="Z64" s="37" t="inlineStr">
+        <is>
+          <t>Part.OnKillHealPercent</t>
+        </is>
+      </c>
+      <c r="AA64" s="37" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="AB64" s="37" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="AC64" s="37" t="inlineStr">
+        <is>
+          <t>HealMaxHpPercent</t>
+        </is>
+      </c>
+      <c r="AD64" s="37" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="AE64" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF64" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG64" s="37" t="inlineStr">
+        <is>
+          <t>Unique</t>
+        </is>
+      </c>
+      <c r="AH64" s="37" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="AI64" s="37" t="n"/>
+      <c r="AJ64" s="37" t="inlineStr">
+        <is>
+          <t>武器插槽C</t>
+        </is>
+      </c>
+      <c r="AK64" s="37" t="n">
+        <v>39</v>
       </c>
     </row>
     <row r="65" ht="22" customHeight="1" s="32">
@@ -19741,6 +20747,90 @@
           <t>0</t>
         </is>
       </c>
+      <c r="R65" s="37" t="inlineStr">
+        <is>
+          <t>PE_LONGSWORD_HASTE_GRIP_1</t>
+        </is>
+      </c>
+      <c r="S65" s="37" t="inlineStr">
+        <is>
+          <t>P_LONGSWORD_HASTE_GRIP</t>
+        </is>
+      </c>
+      <c r="T65" s="37" t="n">
+        <v>1</v>
+      </c>
+      <c r="U65" s="37" t="inlineStr">
+        <is>
+          <t>OnEquip</t>
+        </is>
+      </c>
+      <c r="V65" s="37" t="inlineStr">
+        <is>
+          <t>StatModifier</t>
+        </is>
+      </c>
+      <c r="W65" s="37" t="inlineStr">
+        <is>
+          <t>AttackSpeed</t>
+        </is>
+      </c>
+      <c r="X65" s="37" t="inlineStr">
+        <is>
+          <t>Multiply</t>
+        </is>
+      </c>
+      <c r="Y65" s="37" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="Z65" s="37" t="inlineStr">
+        <is>
+          <t>Part.StatModifier</t>
+        </is>
+      </c>
+      <c r="AA65" s="37" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="AB65" s="37" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="AC65" s="37" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="AD65" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE65" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF65" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG65" s="37" t="inlineStr">
+        <is>
+          <t>Unique</t>
+        </is>
+      </c>
+      <c r="AH65" s="37" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="AI65" s="37" t="n"/>
+      <c r="AJ65" s="37" t="inlineStr">
+        <is>
+          <t>武器插槽C</t>
+        </is>
+      </c>
+      <c r="AK65" s="37" t="n">
+        <v>43</v>
+      </c>
     </row>
     <row r="66" ht="22" customHeight="1" s="32">
       <c r="A66" s="37" t="inlineStr">
@@ -19819,6 +20909,90 @@
           <t>0</t>
         </is>
       </c>
+      <c r="R66" s="37" t="inlineStr">
+        <is>
+          <t>PE_LONGSWORD_HEAVY_GRIP_1</t>
+        </is>
+      </c>
+      <c r="S66" s="37" t="inlineStr">
+        <is>
+          <t>P_LONGSWORD_HEAVY_GRIP</t>
+        </is>
+      </c>
+      <c r="T66" s="37" t="n">
+        <v>1</v>
+      </c>
+      <c r="U66" s="37" t="inlineStr">
+        <is>
+          <t>OnEquip</t>
+        </is>
+      </c>
+      <c r="V66" s="37" t="inlineStr">
+        <is>
+          <t>StatModifier</t>
+        </is>
+      </c>
+      <c r="W66" s="37" t="inlineStr">
+        <is>
+          <t>AttackSpeed</t>
+        </is>
+      </c>
+      <c r="X66" s="37" t="inlineStr">
+        <is>
+          <t>Multiply</t>
+        </is>
+      </c>
+      <c r="Y66" s="37" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="Z66" s="37" t="inlineStr">
+        <is>
+          <t>Part.StatModifier</t>
+        </is>
+      </c>
+      <c r="AA66" s="37" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="AB66" s="37" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="AC66" s="37" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="AD66" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE66" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF66" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG66" s="37" t="inlineStr">
+        <is>
+          <t>Unique</t>
+        </is>
+      </c>
+      <c r="AH66" s="37" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="AI66" s="37" t="n"/>
+      <c r="AJ66" s="37" t="inlineStr">
+        <is>
+          <t>武器插槽C</t>
+        </is>
+      </c>
+      <c r="AK66" s="37" t="n">
+        <v>47</v>
+      </c>
     </row>
     <row r="67" ht="22" customHeight="1" s="32">
       <c r="A67" s="37" t="inlineStr">
@@ -19897,6 +21071,90 @@
           <t>0</t>
         </is>
       </c>
+      <c r="R67" s="37" t="inlineStr">
+        <is>
+          <t>PE_LONGSWORD_HEAVY_GRIP_2</t>
+        </is>
+      </c>
+      <c r="S67" s="37" t="inlineStr">
+        <is>
+          <t>P_LONGSWORD_HEAVY_GRIP</t>
+        </is>
+      </c>
+      <c r="T67" s="37" t="n">
+        <v>2</v>
+      </c>
+      <c r="U67" s="37" t="inlineStr">
+        <is>
+          <t>OnEquip</t>
+        </is>
+      </c>
+      <c r="V67" s="37" t="inlineStr">
+        <is>
+          <t>StatModifier</t>
+        </is>
+      </c>
+      <c r="W67" s="37" t="inlineStr">
+        <is>
+          <t>PhysicalCoefficient</t>
+        </is>
+      </c>
+      <c r="X67" s="37" t="inlineStr">
+        <is>
+          <t>Multiply</t>
+        </is>
+      </c>
+      <c r="Y67" s="37" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="Z67" s="37" t="inlineStr">
+        <is>
+          <t>Part.StatModifier</t>
+        </is>
+      </c>
+      <c r="AA67" s="37" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="AB67" s="37" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="AC67" s="37" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="AD67" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE67" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF67" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG67" s="37" t="inlineStr">
+        <is>
+          <t>Unique</t>
+        </is>
+      </c>
+      <c r="AH67" s="37" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="AI67" s="37" t="n"/>
+      <c r="AJ67" s="37" t="inlineStr">
+        <is>
+          <t>武器插槽C</t>
+        </is>
+      </c>
+      <c r="AK67" s="37" t="n">
+        <v>47</v>
+      </c>
     </row>
     <row r="68" ht="22" customHeight="1" s="32">
       <c r="A68" s="37" t="inlineStr">
@@ -19975,6 +21233,90 @@
           <t>0</t>
         </is>
       </c>
+      <c r="R68" s="37" t="inlineStr">
+        <is>
+          <t>PE_LONGSWORD_HEAVY_GRIP_3</t>
+        </is>
+      </c>
+      <c r="S68" s="37" t="inlineStr">
+        <is>
+          <t>P_LONGSWORD_HEAVY_GRIP</t>
+        </is>
+      </c>
+      <c r="T68" s="37" t="n">
+        <v>3</v>
+      </c>
+      <c r="U68" s="37" t="inlineStr">
+        <is>
+          <t>OnEquip</t>
+        </is>
+      </c>
+      <c r="V68" s="37" t="inlineStr">
+        <is>
+          <t>StatModifier</t>
+        </is>
+      </c>
+      <c r="W68" s="37" t="inlineStr">
+        <is>
+          <t>ElementalCoefficient</t>
+        </is>
+      </c>
+      <c r="X68" s="37" t="inlineStr">
+        <is>
+          <t>Multiply</t>
+        </is>
+      </c>
+      <c r="Y68" s="37" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="Z68" s="37" t="inlineStr">
+        <is>
+          <t>Part.StatModifier</t>
+        </is>
+      </c>
+      <c r="AA68" s="37" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="AB68" s="37" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="AC68" s="37" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="AD68" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE68" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF68" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG68" s="37" t="inlineStr">
+        <is>
+          <t>Unique</t>
+        </is>
+      </c>
+      <c r="AH68" s="37" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="AI68" s="37" t="n"/>
+      <c r="AJ68" s="37" t="inlineStr">
+        <is>
+          <t>武器插槽C</t>
+        </is>
+      </c>
+      <c r="AK68" s="37" t="n">
+        <v>47</v>
+      </c>
     </row>
     <row r="69" ht="22" customHeight="1" s="32">
       <c r="A69" s="37" t="inlineStr">
@@ -20053,6 +21395,90 @@
           <t>0</t>
         </is>
       </c>
+      <c r="R69" s="37" t="inlineStr">
+        <is>
+          <t>PE_GUN_TRIPLESPREAD_MUZZLE_1</t>
+        </is>
+      </c>
+      <c r="S69" s="37" t="inlineStr">
+        <is>
+          <t>P_GUN_TRIPLESPREAD_MUZZLE</t>
+        </is>
+      </c>
+      <c r="T69" s="37" t="n">
+        <v>1</v>
+      </c>
+      <c r="U69" s="37" t="inlineStr">
+        <is>
+          <t>OnEquip</t>
+        </is>
+      </c>
+      <c r="V69" s="37" t="inlineStr">
+        <is>
+          <t>StatModifier</t>
+        </is>
+      </c>
+      <c r="W69" s="37" t="inlineStr">
+        <is>
+          <t>ProjectileCount</t>
+        </is>
+      </c>
+      <c r="X69" s="37" t="inlineStr">
+        <is>
+          <t>Override</t>
+        </is>
+      </c>
+      <c r="Y69" s="37" t="n">
+        <v>3</v>
+      </c>
+      <c r="Z69" s="37" t="inlineStr">
+        <is>
+          <t>Part.StatModifier</t>
+        </is>
+      </c>
+      <c r="AA69" s="37" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="AB69" s="37" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="AC69" s="37" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="AD69" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE69" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF69" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG69" s="37" t="inlineStr">
+        <is>
+          <t>Unique</t>
+        </is>
+      </c>
+      <c r="AH69" s="37" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="AI69" s="37" t="n"/>
+      <c r="AJ69" s="37" t="inlineStr">
+        <is>
+          <t>武器插槽C</t>
+        </is>
+      </c>
+      <c r="AK69" s="37" t="n">
+        <v>48</v>
+      </c>
     </row>
     <row r="70" ht="22" customHeight="1" s="32">
       <c r="A70" s="37" t="inlineStr">
@@ -20130,6 +21556,90 @@
         <is>
           <t>0</t>
         </is>
+      </c>
+      <c r="R70" s="37" t="inlineStr">
+        <is>
+          <t>PE_GUN_TRIPLESPREAD_MUZZLE_2</t>
+        </is>
+      </c>
+      <c r="S70" s="37" t="inlineStr">
+        <is>
+          <t>P_GUN_TRIPLESPREAD_MUZZLE</t>
+        </is>
+      </c>
+      <c r="T70" s="37" t="n">
+        <v>2</v>
+      </c>
+      <c r="U70" s="37" t="inlineStr">
+        <is>
+          <t>OnEquip</t>
+        </is>
+      </c>
+      <c r="V70" s="37" t="inlineStr">
+        <is>
+          <t>StatModifier</t>
+        </is>
+      </c>
+      <c r="W70" s="37" t="inlineStr">
+        <is>
+          <t>ConcentrationDegrees</t>
+        </is>
+      </c>
+      <c r="X70" s="37" t="inlineStr">
+        <is>
+          <t>Override</t>
+        </is>
+      </c>
+      <c r="Y70" s="37" t="n">
+        <v>60</v>
+      </c>
+      <c r="Z70" s="37" t="inlineStr">
+        <is>
+          <t>Part.StatModifier</t>
+        </is>
+      </c>
+      <c r="AA70" s="37" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="AB70" s="37" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="AC70" s="37" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="AD70" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE70" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF70" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG70" s="37" t="inlineStr">
+        <is>
+          <t>Unique</t>
+        </is>
+      </c>
+      <c r="AH70" s="37" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="AI70" s="37" t="n"/>
+      <c r="AJ70" s="37" t="inlineStr">
+        <is>
+          <t>武器插槽C</t>
+        </is>
+      </c>
+      <c r="AK70" s="37" t="n">
+        <v>48</v>
       </c>
     </row>
     <row r="71" ht="22" customHeight="1" s="32">
@@ -20213,16 +21723,100 @@
           <t>0</t>
         </is>
       </c>
+      <c r="R71" s="37" t="inlineStr">
+        <is>
+          <t>PE_STAFF_DUALSPREAD_STAFFBODY_1</t>
+        </is>
+      </c>
+      <c r="S71" s="37" t="inlineStr">
+        <is>
+          <t>P_STAFF_DUALSPREAD_STAFFBODY</t>
+        </is>
+      </c>
+      <c r="T71" s="37" t="n">
+        <v>1</v>
+      </c>
+      <c r="U71" s="37" t="inlineStr">
+        <is>
+          <t>OnEquip</t>
+        </is>
+      </c>
+      <c r="V71" s="37" t="inlineStr">
+        <is>
+          <t>StatModifier</t>
+        </is>
+      </c>
+      <c r="W71" s="37" t="inlineStr">
+        <is>
+          <t>ProjectileCount</t>
+        </is>
+      </c>
+      <c r="X71" s="37" t="inlineStr">
+        <is>
+          <t>Override</t>
+        </is>
+      </c>
+      <c r="Y71" s="37" t="n">
+        <v>2</v>
+      </c>
+      <c r="Z71" s="37" t="inlineStr">
+        <is>
+          <t>Part.StatModifier</t>
+        </is>
+      </c>
+      <c r="AA71" s="37" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="AB71" s="37" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="AC71" s="37" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="AD71" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE71" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF71" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG71" s="37" t="inlineStr">
+        <is>
+          <t>Unique</t>
+        </is>
+      </c>
+      <c r="AH71" s="37" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="AI71" s="37" t="n"/>
+      <c r="AJ71" s="37" t="inlineStr">
+        <is>
+          <t>武器插槽C</t>
+        </is>
+      </c>
+      <c r="AK71" s="37" t="n">
+        <v>59</v>
+      </c>
     </row>
     <row r="72" ht="22" customHeight="1" s="32">
       <c r="A72" s="37" t="inlineStr">
         <is>
-          <t>AUDIT_WEAPON_SLOTS_C_36</t>
+          <t>P_LONGSWORD_NARROWWIDE_SWORDBLADE</t>
         </is>
       </c>
       <c r="B72" s="37" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>P_LONGSWORD_NARROWWIDE_SWORDBLADE</t>
         </is>
       </c>
       <c r="C72" s="37" t="inlineStr">
@@ -20235,7 +21829,11 @@
           <t>SwordBlade</t>
         </is>
       </c>
-      <c r="E72" s="37" t="n"/>
+      <c r="E72" s="37" t="inlineStr">
+        <is>
+          <t>窄角广域剑刃</t>
+        </is>
+      </c>
       <c r="F72" s="37" t="inlineStr">
         <is>
           <t>效果：攻击角度降为120°；攻击范围+30%</t>
@@ -20243,34 +21841,30 @@
       </c>
       <c r="G72" s="37" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Common</t>
         </is>
       </c>
       <c r="H72" s="37" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>SwordBlade|Numeric</t>
         </is>
       </c>
       <c r="I72" s="37" t="inlineStr">
         <is>
-          <t>false</t>
+          <t>true</t>
         </is>
       </c>
       <c r="J72" s="37" t="inlineStr">
         <is>
-          <t>Unimplemented</t>
+          <t>Approved</t>
         </is>
       </c>
       <c r="K72" s="37" t="inlineStr">
         <is>
-          <t>Disabled</t>
-        </is>
-      </c>
-      <c r="L72" s="37" t="inlineStr">
-        <is>
-          <t>Unnamed workbook row; no stable PartId assigned.</t>
-        </is>
-      </c>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="L72" s="37" t="n"/>
       <c r="M72" s="37" t="inlineStr">
         <is>
           <t>武器插槽C</t>
@@ -20283,24 +21877,106 @@
       </c>
       <c r="O72" s="37" t="inlineStr">
         <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="P72" s="37" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="P72" s="37" t="n">
+        <v>30</v>
+      </c>
+      <c r="R72" s="37" t="inlineStr">
+        <is>
+          <t>PE_STAFF_DUALSPREAD_STAFFBODY_2</t>
+        </is>
+      </c>
+      <c r="S72" s="37" t="inlineStr">
+        <is>
+          <t>P_STAFF_DUALSPREAD_STAFFBODY</t>
+        </is>
+      </c>
+      <c r="T72" s="37" t="n">
+        <v>2</v>
+      </c>
+      <c r="U72" s="37" t="inlineStr">
+        <is>
+          <t>OnEquip</t>
+        </is>
+      </c>
+      <c r="V72" s="37" t="inlineStr">
+        <is>
+          <t>StatModifier</t>
+        </is>
+      </c>
+      <c r="W72" s="37" t="inlineStr">
+        <is>
+          <t>ConcentrationDegrees</t>
+        </is>
+      </c>
+      <c r="X72" s="37" t="inlineStr">
+        <is>
+          <t>Override</t>
+        </is>
+      </c>
+      <c r="Y72" s="37" t="n">
+        <v>60</v>
+      </c>
+      <c r="Z72" s="37" t="inlineStr">
+        <is>
+          <t>Part.StatModifier</t>
+        </is>
+      </c>
+      <c r="AA72" s="37" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="AB72" s="37" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="AC72" s="37" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="AD72" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE72" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF72" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG72" s="37" t="inlineStr">
+        <is>
+          <t>Unique</t>
+        </is>
+      </c>
+      <c r="AH72" s="37" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="AI72" s="37" t="n"/>
+      <c r="AJ72" s="37" t="inlineStr">
+        <is>
+          <t>武器插槽C</t>
+        </is>
+      </c>
+      <c r="AK72" s="37" t="n">
+        <v>59</v>
       </c>
     </row>
     <row r="73" ht="22" customHeight="1" s="32">
       <c r="A73" s="37" t="inlineStr">
         <is>
-          <t>AUDIT_WEAPON_SLOTS_C_37</t>
+          <t>P_LONGSWORD_SLOWWIDE_SWORDBLADE</t>
         </is>
       </c>
       <c r="B73" s="37" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>P_LONGSWORD_SLOWWIDE_SWORDBLADE</t>
         </is>
       </c>
       <c r="C73" s="37" t="inlineStr">
@@ -20313,7 +21989,11 @@
           <t>SwordBlade</t>
         </is>
       </c>
-      <c r="E73" s="37" t="n"/>
+      <c r="E73" s="37" t="inlineStr">
+        <is>
+          <t>减攻速广域剑刃</t>
+        </is>
+      </c>
       <c r="F73" s="37" t="inlineStr">
         <is>
           <t>效果：攻击速度-20%，攻击范围+30%</t>
@@ -20321,34 +22001,30 @@
       </c>
       <c r="G73" s="37" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Common</t>
         </is>
       </c>
       <c r="H73" s="37" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>SwordBlade|Numeric</t>
         </is>
       </c>
       <c r="I73" s="37" t="inlineStr">
         <is>
-          <t>false</t>
+          <t>true</t>
         </is>
       </c>
       <c r="J73" s="37" t="inlineStr">
         <is>
-          <t>Unimplemented</t>
+          <t>Approved</t>
         </is>
       </c>
       <c r="K73" s="37" t="inlineStr">
         <is>
-          <t>Disabled</t>
-        </is>
-      </c>
-      <c r="L73" s="37" t="inlineStr">
-        <is>
-          <t>Unnamed workbook row; no stable PartId assigned.</t>
-        </is>
-      </c>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="L73" s="37" t="n"/>
       <c r="M73" s="37" t="inlineStr">
         <is>
           <t>武器插槽C</t>
@@ -20361,13 +22037,95 @@
       </c>
       <c r="O73" s="37" t="inlineStr">
         <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="P73" s="37" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="P73" s="37" t="n">
+        <v>30</v>
+      </c>
+      <c r="R73" s="37" t="inlineStr">
+        <is>
+          <t>PE_STAFF_WIDEWEAK_STAFFCRYSTAL_1</t>
+        </is>
+      </c>
+      <c r="S73" s="37" t="inlineStr">
+        <is>
+          <t>P_STAFF_WIDEWEAK_STAFFCRYSTAL</t>
+        </is>
+      </c>
+      <c r="T73" s="37" t="n">
+        <v>1</v>
+      </c>
+      <c r="U73" s="37" t="inlineStr">
+        <is>
+          <t>OnEquip</t>
+        </is>
+      </c>
+      <c r="V73" s="37" t="inlineStr">
+        <is>
+          <t>StatModifier</t>
+        </is>
+      </c>
+      <c r="W73" s="37" t="inlineStr">
+        <is>
+          <t>PhysicalCoefficient</t>
+        </is>
+      </c>
+      <c r="X73" s="37" t="inlineStr">
+        <is>
+          <t>Multiply</t>
+        </is>
+      </c>
+      <c r="Y73" s="37" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="Z73" s="37" t="inlineStr">
+        <is>
+          <t>Part.StatModifier</t>
+        </is>
+      </c>
+      <c r="AA73" s="37" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="AB73" s="37" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="AC73" s="37" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="AD73" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE73" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF73" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG73" s="37" t="inlineStr">
+        <is>
+          <t>Unique</t>
+        </is>
+      </c>
+      <c r="AH73" s="37" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="AI73" s="37" t="n"/>
+      <c r="AJ73" s="37" t="inlineStr">
+        <is>
+          <t>武器插槽C</t>
+        </is>
+      </c>
+      <c r="AK73" s="37" t="n">
+        <v>64</v>
       </c>
     </row>
     <row r="74" ht="22" customHeight="1" s="32">
@@ -20447,16 +22205,100 @@
           <t>0</t>
         </is>
       </c>
+      <c r="R74" s="37" t="inlineStr">
+        <is>
+          <t>PE_STAFF_WIDEWEAK_STAFFCRYSTAL_2</t>
+        </is>
+      </c>
+      <c r="S74" s="37" t="inlineStr">
+        <is>
+          <t>P_STAFF_WIDEWEAK_STAFFCRYSTAL</t>
+        </is>
+      </c>
+      <c r="T74" s="37" t="n">
+        <v>2</v>
+      </c>
+      <c r="U74" s="37" t="inlineStr">
+        <is>
+          <t>OnEquip</t>
+        </is>
+      </c>
+      <c r="V74" s="37" t="inlineStr">
+        <is>
+          <t>StatModifier</t>
+        </is>
+      </c>
+      <c r="W74" s="37" t="inlineStr">
+        <is>
+          <t>ElementalCoefficient</t>
+        </is>
+      </c>
+      <c r="X74" s="37" t="inlineStr">
+        <is>
+          <t>Multiply</t>
+        </is>
+      </c>
+      <c r="Y74" s="37" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="Z74" s="37" t="inlineStr">
+        <is>
+          <t>Part.StatModifier</t>
+        </is>
+      </c>
+      <c r="AA74" s="37" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="AB74" s="37" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="AC74" s="37" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="AD74" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE74" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF74" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG74" s="37" t="inlineStr">
+        <is>
+          <t>Unique</t>
+        </is>
+      </c>
+      <c r="AH74" s="37" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="AI74" s="37" t="n"/>
+      <c r="AJ74" s="37" t="inlineStr">
+        <is>
+          <t>武器插槽C</t>
+        </is>
+      </c>
+      <c r="AK74" s="37" t="n">
+        <v>64</v>
+      </c>
     </row>
     <row r="75" ht="22" customHeight="1" s="32">
       <c r="A75" s="37" t="inlineStr">
         <is>
-          <t>AUDIT_WEAPON_SLOTS_C_39</t>
+          <t>P_LONGSWORD_KILLHEAL_SWORDBLADE</t>
         </is>
       </c>
       <c r="B75" s="37" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>P_LONGSWORD_KILLHEAL_SWORDBLADE</t>
         </is>
       </c>
       <c r="C75" s="37" t="inlineStr">
@@ -20469,7 +22311,11 @@
           <t>SwordBlade</t>
         </is>
       </c>
-      <c r="E75" s="37" t="n"/>
+      <c r="E75" s="37" t="inlineStr">
+        <is>
+          <t>击杀吸血剑刃</t>
+        </is>
+      </c>
       <c r="F75" s="37" t="inlineStr">
         <is>
           <t>效果：每击杀一名敌方单位，回复5%最大生命值</t>
@@ -20477,34 +22323,30 @@
       </c>
       <c r="G75" s="37" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Rare</t>
         </is>
       </c>
       <c r="H75" s="37" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>SwordBlade|UniqueBehavior</t>
         </is>
       </c>
       <c r="I75" s="37" t="inlineStr">
         <is>
-          <t>false</t>
+          <t>true</t>
         </is>
       </c>
       <c r="J75" s="37" t="inlineStr">
         <is>
-          <t>Unimplemented</t>
+          <t>Approved</t>
         </is>
       </c>
       <c r="K75" s="37" t="inlineStr">
         <is>
-          <t>Disabled</t>
-        </is>
-      </c>
-      <c r="L75" s="37" t="inlineStr">
-        <is>
-          <t>Unnamed workbook row; no stable PartId assigned.</t>
-        </is>
-      </c>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="L75" s="37" t="n"/>
       <c r="M75" s="37" t="inlineStr">
         <is>
           <t>武器插槽C</t>
@@ -20517,13 +22359,95 @@
       </c>
       <c r="O75" s="37" t="inlineStr">
         <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="P75" s="37" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="P75" s="37" t="n">
+        <v>45</v>
+      </c>
+      <c r="R75" s="37" t="inlineStr">
+        <is>
+          <t>PE_STAFF_WIDEWEAK_STAFFCRYSTAL_3</t>
+        </is>
+      </c>
+      <c r="S75" s="37" t="inlineStr">
+        <is>
+          <t>P_STAFF_WIDEWEAK_STAFFCRYSTAL</t>
+        </is>
+      </c>
+      <c r="T75" s="37" t="n">
+        <v>3</v>
+      </c>
+      <c r="U75" s="37" t="inlineStr">
+        <is>
+          <t>OnEquip</t>
+        </is>
+      </c>
+      <c r="V75" s="37" t="inlineStr">
+        <is>
+          <t>StatModifier</t>
+        </is>
+      </c>
+      <c r="W75" s="37" t="inlineStr">
+        <is>
+          <t>ExplosionRadius</t>
+        </is>
+      </c>
+      <c r="X75" s="37" t="inlineStr">
+        <is>
+          <t>Multiply</t>
+        </is>
+      </c>
+      <c r="Y75" s="37" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="Z75" s="37" t="inlineStr">
+        <is>
+          <t>Part.StatModifier</t>
+        </is>
+      </c>
+      <c r="AA75" s="37" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="AB75" s="37" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="AC75" s="37" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="AD75" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE75" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF75" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG75" s="37" t="inlineStr">
+        <is>
+          <t>Unique</t>
+        </is>
+      </c>
+      <c r="AH75" s="37" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="AI75" s="37" t="n"/>
+      <c r="AJ75" s="37" t="inlineStr">
+        <is>
+          <t>武器插槽C</t>
+        </is>
+      </c>
+      <c r="AK75" s="37" t="n">
+        <v>64</v>
       </c>
     </row>
     <row r="76" ht="22" customHeight="1" s="32">
@@ -20603,6 +22527,90 @@
           <t>0</t>
         </is>
       </c>
+      <c r="R76" s="37" t="inlineStr">
+        <is>
+          <t>PE_STAFF_NARROWSTRONG_STAFFCRYSTAL_1</t>
+        </is>
+      </c>
+      <c r="S76" s="37" t="inlineStr">
+        <is>
+          <t>P_STAFF_NARROWSTRONG_STAFFCRYSTAL</t>
+        </is>
+      </c>
+      <c r="T76" s="37" t="n">
+        <v>1</v>
+      </c>
+      <c r="U76" s="37" t="inlineStr">
+        <is>
+          <t>OnEquip</t>
+        </is>
+      </c>
+      <c r="V76" s="37" t="inlineStr">
+        <is>
+          <t>StatModifier</t>
+        </is>
+      </c>
+      <c r="W76" s="37" t="inlineStr">
+        <is>
+          <t>PhysicalCoefficient</t>
+        </is>
+      </c>
+      <c r="X76" s="37" t="inlineStr">
+        <is>
+          <t>Multiply</t>
+        </is>
+      </c>
+      <c r="Y76" s="37" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="Z76" s="37" t="inlineStr">
+        <is>
+          <t>Part.StatModifier</t>
+        </is>
+      </c>
+      <c r="AA76" s="37" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="AB76" s="37" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="AC76" s="37" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="AD76" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE76" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF76" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG76" s="37" t="inlineStr">
+        <is>
+          <t>Unique</t>
+        </is>
+      </c>
+      <c r="AH76" s="37" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="AI76" s="37" t="n"/>
+      <c r="AJ76" s="37" t="inlineStr">
+        <is>
+          <t>武器插槽C</t>
+        </is>
+      </c>
+      <c r="AK76" s="37" t="n">
+        <v>65</v>
+      </c>
     </row>
     <row r="77" ht="22" customHeight="1" s="32">
       <c r="A77" s="37" t="inlineStr">
@@ -20680,6 +22688,90 @@
         <is>
           <t>0</t>
         </is>
+      </c>
+      <c r="R77" s="37" t="inlineStr">
+        <is>
+          <t>PE_STAFF_NARROWSTRONG_STAFFCRYSTAL_2</t>
+        </is>
+      </c>
+      <c r="S77" s="37" t="inlineStr">
+        <is>
+          <t>P_STAFF_NARROWSTRONG_STAFFCRYSTAL</t>
+        </is>
+      </c>
+      <c r="T77" s="37" t="n">
+        <v>2</v>
+      </c>
+      <c r="U77" s="37" t="inlineStr">
+        <is>
+          <t>OnEquip</t>
+        </is>
+      </c>
+      <c r="V77" s="37" t="inlineStr">
+        <is>
+          <t>StatModifier</t>
+        </is>
+      </c>
+      <c r="W77" s="37" t="inlineStr">
+        <is>
+          <t>ElementalCoefficient</t>
+        </is>
+      </c>
+      <c r="X77" s="37" t="inlineStr">
+        <is>
+          <t>Multiply</t>
+        </is>
+      </c>
+      <c r="Y77" s="37" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="Z77" s="37" t="inlineStr">
+        <is>
+          <t>Part.StatModifier</t>
+        </is>
+      </c>
+      <c r="AA77" s="37" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="AB77" s="37" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="AC77" s="37" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="AD77" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE77" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF77" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG77" s="37" t="inlineStr">
+        <is>
+          <t>Unique</t>
+        </is>
+      </c>
+      <c r="AH77" s="37" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="AI77" s="37" t="n"/>
+      <c r="AJ77" s="37" t="inlineStr">
+        <is>
+          <t>武器插槽C</t>
+        </is>
+      </c>
+      <c r="AK77" s="37" t="n">
+        <v>65</v>
       </c>
     </row>
     <row r="78" ht="22" customHeight="1" s="32">
@@ -20761,16 +22853,100 @@
           <t>0</t>
         </is>
       </c>
+      <c r="R78" s="37" t="inlineStr">
+        <is>
+          <t>PE_STAFF_NARROWSTRONG_STAFFCRYSTAL_3</t>
+        </is>
+      </c>
+      <c r="S78" s="37" t="inlineStr">
+        <is>
+          <t>P_STAFF_NARROWSTRONG_STAFFCRYSTAL</t>
+        </is>
+      </c>
+      <c r="T78" s="37" t="n">
+        <v>3</v>
+      </c>
+      <c r="U78" s="37" t="inlineStr">
+        <is>
+          <t>OnEquip</t>
+        </is>
+      </c>
+      <c r="V78" s="37" t="inlineStr">
+        <is>
+          <t>StatModifier</t>
+        </is>
+      </c>
+      <c r="W78" s="37" t="inlineStr">
+        <is>
+          <t>ExplosionRadius</t>
+        </is>
+      </c>
+      <c r="X78" s="37" t="inlineStr">
+        <is>
+          <t>Multiply</t>
+        </is>
+      </c>
+      <c r="Y78" s="37" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="Z78" s="37" t="inlineStr">
+        <is>
+          <t>Part.StatModifier</t>
+        </is>
+      </c>
+      <c r="AA78" s="37" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="AB78" s="37" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="AC78" s="37" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="AD78" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE78" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF78" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG78" s="37" t="inlineStr">
+        <is>
+          <t>Unique</t>
+        </is>
+      </c>
+      <c r="AH78" s="37" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="AI78" s="37" t="n"/>
+      <c r="AJ78" s="37" t="inlineStr">
+        <is>
+          <t>武器插槽C</t>
+        </is>
+      </c>
+      <c r="AK78" s="37" t="n">
+        <v>65</v>
+      </c>
     </row>
     <row r="79" ht="75" customHeight="1" s="32">
       <c r="A79" s="37" t="inlineStr">
         <is>
-          <t>AUDIT_WEAPON_SLOTS_C_43</t>
+          <t>P_LONGSWORD_HASTE_GRIP</t>
         </is>
       </c>
       <c r="B79" s="37" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>P_LONGSWORD_HASTE_GRIP</t>
         </is>
       </c>
       <c r="C79" s="37" t="inlineStr">
@@ -20783,7 +22959,11 @@
           <t>Grip</t>
         </is>
       </c>
-      <c r="E79" s="37" t="n"/>
+      <c r="E79" s="37" t="inlineStr">
+        <is>
+          <t>攻速剑柄</t>
+        </is>
+      </c>
       <c r="F79" s="37" t="inlineStr">
         <is>
           <t>效果：攻击速度+20%</t>
@@ -20791,34 +22971,30 @@
       </c>
       <c r="G79" s="37" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Common</t>
         </is>
       </c>
       <c r="H79" s="37" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Grip|Numeric</t>
         </is>
       </c>
       <c r="I79" s="37" t="inlineStr">
         <is>
-          <t>false</t>
+          <t>true</t>
         </is>
       </c>
       <c r="J79" s="37" t="inlineStr">
         <is>
-          <t>Unimplemented</t>
+          <t>Approved</t>
         </is>
       </c>
       <c r="K79" s="37" t="inlineStr">
         <is>
-          <t>Disabled</t>
-        </is>
-      </c>
-      <c r="L79" s="37" t="inlineStr">
-        <is>
-          <t>Unnamed workbook row; no stable PartId assigned.</t>
-        </is>
-      </c>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="L79" s="37" t="n"/>
       <c r="M79" s="37" t="inlineStr">
         <is>
           <t>武器插槽C</t>
@@ -20831,13 +23007,95 @@
       </c>
       <c r="O79" s="37" t="inlineStr">
         <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="P79" s="37" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="P79" s="37" t="n">
+        <v>30</v>
+      </c>
+      <c r="R79" s="37" t="inlineStr">
+        <is>
+          <t>PE_STAFF_SLOWWIDE_STAFFCRYSTAL_1</t>
+        </is>
+      </c>
+      <c r="S79" s="37" t="inlineStr">
+        <is>
+          <t>P_STAFF_SLOWWIDE_STAFFCRYSTAL</t>
+        </is>
+      </c>
+      <c r="T79" s="37" t="n">
+        <v>1</v>
+      </c>
+      <c r="U79" s="37" t="inlineStr">
+        <is>
+          <t>OnEquip</t>
+        </is>
+      </c>
+      <c r="V79" s="37" t="inlineStr">
+        <is>
+          <t>StatModifier</t>
+        </is>
+      </c>
+      <c r="W79" s="37" t="inlineStr">
+        <is>
+          <t>AttackSpeed</t>
+        </is>
+      </c>
+      <c r="X79" s="37" t="inlineStr">
+        <is>
+          <t>Multiply</t>
+        </is>
+      </c>
+      <c r="Y79" s="37" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="Z79" s="37" t="inlineStr">
+        <is>
+          <t>Part.StatModifier</t>
+        </is>
+      </c>
+      <c r="AA79" s="37" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="AB79" s="37" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="AC79" s="37" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="AD79" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE79" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF79" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG79" s="37" t="inlineStr">
+        <is>
+          <t>Unique</t>
+        </is>
+      </c>
+      <c r="AH79" s="37" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="AI79" s="37" t="n"/>
+      <c r="AJ79" s="37" t="inlineStr">
+        <is>
+          <t>武器插槽C</t>
+        </is>
+      </c>
+      <c r="AK79" s="37" t="n">
+        <v>67</v>
       </c>
     </row>
     <row r="80" ht="22" customHeight="1" s="32">
@@ -20917,6 +23175,90 @@
           <t>0</t>
         </is>
       </c>
+      <c r="R80" s="37" t="inlineStr">
+        <is>
+          <t>PE_STAFF_SLOWWIDE_STAFFCRYSTAL_2</t>
+        </is>
+      </c>
+      <c r="S80" s="37" t="inlineStr">
+        <is>
+          <t>P_STAFF_SLOWWIDE_STAFFCRYSTAL</t>
+        </is>
+      </c>
+      <c r="T80" s="37" t="n">
+        <v>2</v>
+      </c>
+      <c r="U80" s="37" t="inlineStr">
+        <is>
+          <t>OnEquip</t>
+        </is>
+      </c>
+      <c r="V80" s="37" t="inlineStr">
+        <is>
+          <t>StatModifier</t>
+        </is>
+      </c>
+      <c r="W80" s="37" t="inlineStr">
+        <is>
+          <t>ExplosionRadius</t>
+        </is>
+      </c>
+      <c r="X80" s="37" t="inlineStr">
+        <is>
+          <t>Multiply</t>
+        </is>
+      </c>
+      <c r="Y80" s="37" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="Z80" s="37" t="inlineStr">
+        <is>
+          <t>Part.StatModifier</t>
+        </is>
+      </c>
+      <c r="AA80" s="37" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="AB80" s="37" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="AC80" s="37" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="AD80" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE80" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF80" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG80" s="37" t="inlineStr">
+        <is>
+          <t>Unique</t>
+        </is>
+      </c>
+      <c r="AH80" s="37" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="AI80" s="37" t="n"/>
+      <c r="AJ80" s="37" t="inlineStr">
+        <is>
+          <t>武器插槽C</t>
+        </is>
+      </c>
+      <c r="AK80" s="37" t="n">
+        <v>67</v>
+      </c>
     </row>
     <row r="81" ht="22" customHeight="1" s="32">
       <c r="A81" s="37" t="inlineStr">
@@ -20995,6 +23337,90 @@
           <t>0</t>
         </is>
       </c>
+      <c r="R81" s="37" t="inlineStr">
+        <is>
+          <t>PE_WHIP_HASTE_WHIPBODY_1</t>
+        </is>
+      </c>
+      <c r="S81" s="37" t="inlineStr">
+        <is>
+          <t>P_WHIP_HASTE_WHIPBODY</t>
+        </is>
+      </c>
+      <c r="T81" s="37" t="n">
+        <v>1</v>
+      </c>
+      <c r="U81" s="37" t="inlineStr">
+        <is>
+          <t>OnEquip</t>
+        </is>
+      </c>
+      <c r="V81" s="37" t="inlineStr">
+        <is>
+          <t>StatModifier</t>
+        </is>
+      </c>
+      <c r="W81" s="37" t="inlineStr">
+        <is>
+          <t>AttackSpeed</t>
+        </is>
+      </c>
+      <c r="X81" s="37" t="inlineStr">
+        <is>
+          <t>Multiply</t>
+        </is>
+      </c>
+      <c r="Y81" s="37" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="Z81" s="37" t="inlineStr">
+        <is>
+          <t>Part.StatModifier</t>
+        </is>
+      </c>
+      <c r="AA81" s="37" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="AB81" s="37" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="AC81" s="37" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="AD81" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE81" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF81" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG81" s="37" t="inlineStr">
+        <is>
+          <t>Unique</t>
+        </is>
+      </c>
+      <c r="AH81" s="37" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="AI81" s="37" t="n"/>
+      <c r="AJ81" s="37" t="inlineStr">
+        <is>
+          <t>武器插槽C</t>
+        </is>
+      </c>
+      <c r="AK81" s="37" t="n">
+        <v>73</v>
+      </c>
     </row>
     <row r="82" ht="22" customHeight="1" s="32">
       <c r="A82" s="37" t="inlineStr">
@@ -21073,16 +23499,100 @@
           <t>0</t>
         </is>
       </c>
+      <c r="R82" s="37" t="inlineStr">
+        <is>
+          <t>PE_WHIP_KILLHEAL_WHIPBODY_1</t>
+        </is>
+      </c>
+      <c r="S82" s="37" t="inlineStr">
+        <is>
+          <t>P_WHIP_KILLHEAL_WHIPBODY</t>
+        </is>
+      </c>
+      <c r="T82" s="37" t="n">
+        <v>1</v>
+      </c>
+      <c r="U82" s="37" t="inlineStr">
+        <is>
+          <t>OnKill</t>
+        </is>
+      </c>
+      <c r="V82" s="37" t="inlineStr">
+        <is>
+          <t>UniqueBehavior</t>
+        </is>
+      </c>
+      <c r="W82" s="37" t="inlineStr">
+        <is>
+          <t>OnKill</t>
+        </is>
+      </c>
+      <c r="X82" s="37" t="inlineStr">
+        <is>
+          <t>Add</t>
+        </is>
+      </c>
+      <c r="Y82" s="37" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="Z82" s="37" t="inlineStr">
+        <is>
+          <t>Part.OnKillHealPercent</t>
+        </is>
+      </c>
+      <c r="AA82" s="37" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="AB82" s="37" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="AC82" s="37" t="inlineStr">
+        <is>
+          <t>HealMaxHpPercent</t>
+        </is>
+      </c>
+      <c r="AD82" s="37" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="AE82" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF82" s="37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG82" s="37" t="inlineStr">
+        <is>
+          <t>Unique</t>
+        </is>
+      </c>
+      <c r="AH82" s="37" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="AI82" s="37" t="n"/>
+      <c r="AJ82" s="37" t="inlineStr">
+        <is>
+          <t>武器插槽C</t>
+        </is>
+      </c>
+      <c r="AK82" s="37" t="n">
+        <v>74</v>
+      </c>
     </row>
     <row r="83" ht="22" customHeight="1" s="32">
       <c r="A83" s="37" t="inlineStr">
         <is>
-          <t>AUDIT_WEAPON_SLOTS_C_47</t>
+          <t>P_LONGSWORD_HEAVY_GRIP</t>
         </is>
       </c>
       <c r="B83" s="37" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>P_LONGSWORD_HEAVY_GRIP</t>
         </is>
       </c>
       <c r="C83" s="37" t="inlineStr">
@@ -21095,7 +23605,11 @@
           <t>Grip</t>
         </is>
       </c>
-      <c r="E83" s="37" t="n"/>
+      <c r="E83" s="37" t="inlineStr">
+        <is>
+          <t>重击剑柄</t>
+        </is>
+      </c>
       <c r="F83" s="37" t="inlineStr">
         <is>
           <t>效果：攻击速度-30%，伤害倍率+50%</t>
@@ -21103,34 +23617,30 @@
       </c>
       <c r="G83" s="37" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Common</t>
         </is>
       </c>
       <c r="H83" s="37" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Grip|Numeric</t>
         </is>
       </c>
       <c r="I83" s="37" t="inlineStr">
         <is>
-          <t>false</t>
+          <t>true</t>
         </is>
       </c>
       <c r="J83" s="37" t="inlineStr">
         <is>
-          <t>Unimplemented</t>
+          <t>Approved</t>
         </is>
       </c>
       <c r="K83" s="37" t="inlineStr">
         <is>
-          <t>Disabled</t>
-        </is>
-      </c>
-      <c r="L83" s="37" t="inlineStr">
-        <is>
-          <t>Unnamed workbook row; no stable PartId assigned.</t>
-        </is>
-      </c>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="L83" s="37" t="n"/>
       <c r="M83" s="37" t="inlineStr">
         <is>
           <t>武器插槽C</t>
@@ -21143,24 +23653,22 @@
       </c>
       <c r="O83" s="37" t="inlineStr">
         <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="P83" s="37" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="P83" s="37" t="n">
+        <v>30</v>
       </c>
     </row>
     <row r="84" ht="22" customHeight="1" s="32">
       <c r="A84" s="37" t="inlineStr">
         <is>
-          <t>AUDIT_WEAPON_SLOTS_C_48</t>
+          <t>P_GUN_TRIPLESPREAD_MUZZLE</t>
         </is>
       </c>
       <c r="B84" s="37" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>P_GUN_TRIPLESPREAD_MUZZLE</t>
         </is>
       </c>
       <c r="C84" s="37" t="inlineStr">
@@ -21173,7 +23681,11 @@
           <t>Muzzle</t>
         </is>
       </c>
-      <c r="E84" s="37" t="n"/>
+      <c r="E84" s="37" t="inlineStr">
+        <is>
+          <t>三发散射枪口</t>
+        </is>
+      </c>
       <c r="F84" s="37" t="inlineStr">
         <is>
           <t>效果：弹道固定为3，武器集中性固定为60°</t>
@@ -21181,34 +23693,30 @@
       </c>
       <c r="G84" s="37" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Rare</t>
         </is>
       </c>
       <c r="H84" s="37" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Muzzle|Numeric</t>
         </is>
       </c>
       <c r="I84" s="37" t="inlineStr">
         <is>
-          <t>false</t>
+          <t>true</t>
         </is>
       </c>
       <c r="J84" s="37" t="inlineStr">
         <is>
-          <t>Unimplemented</t>
+          <t>Approved</t>
         </is>
       </c>
       <c r="K84" s="37" t="inlineStr">
         <is>
-          <t>Disabled</t>
-        </is>
-      </c>
-      <c r="L84" s="37" t="inlineStr">
-        <is>
-          <t>Unnamed workbook row; no stable PartId assigned.</t>
-        </is>
-      </c>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="L84" s="37" t="n"/>
       <c r="M84" s="37" t="inlineStr">
         <is>
           <t>武器插槽C</t>
@@ -21221,13 +23729,11 @@
       </c>
       <c r="O84" s="37" t="inlineStr">
         <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="P84" s="37" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="P84" s="37" t="n">
+        <v>45</v>
       </c>
     </row>
     <row r="85" ht="22" customHeight="1" s="32">
@@ -22013,12 +24519,12 @@
     <row r="95" ht="22" customHeight="1" s="32">
       <c r="A95" s="37" t="inlineStr">
         <is>
-          <t>AUDIT_WEAPON_SLOTS_C_59</t>
+          <t>P_STAFF_DUALSPREAD_STAFFBODY</t>
         </is>
       </c>
       <c r="B95" s="37" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>P_STAFF_DUALSPREAD_STAFFBODY</t>
         </is>
       </c>
       <c r="C95" s="37" t="inlineStr">
@@ -22031,7 +24537,11 @@
           <t>StaffBody</t>
         </is>
       </c>
-      <c r="E95" s="37" t="n"/>
+      <c r="E95" s="37" t="inlineStr">
+        <is>
+          <t>双发散射杖体</t>
+        </is>
+      </c>
       <c r="F95" s="37" t="inlineStr">
         <is>
           <t>效果：弹道固定为2，武器集中性固定为60°</t>
@@ -22039,34 +24549,30 @@
       </c>
       <c r="G95" s="37" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Rare</t>
         </is>
       </c>
       <c r="H95" s="37" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>StaffBody|Numeric</t>
         </is>
       </c>
       <c r="I95" s="37" t="inlineStr">
         <is>
-          <t>false</t>
+          <t>true</t>
         </is>
       </c>
       <c r="J95" s="37" t="inlineStr">
         <is>
-          <t>Unimplemented</t>
+          <t>Approved</t>
         </is>
       </c>
       <c r="K95" s="37" t="inlineStr">
         <is>
-          <t>Disabled</t>
-        </is>
-      </c>
-      <c r="L95" s="37" t="inlineStr">
-        <is>
-          <t>Unnamed workbook row; no stable PartId assigned.</t>
-        </is>
-      </c>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="L95" s="37" t="n"/>
       <c r="M95" s="37" t="inlineStr">
         <is>
           <t>武器插槽C</t>
@@ -22079,13 +24585,11 @@
       </c>
       <c r="O95" s="37" t="inlineStr">
         <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="P95" s="37" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="P95" s="37" t="n">
+        <v>45</v>
       </c>
     </row>
     <row r="96" ht="22" customHeight="1" s="32">
@@ -22407,12 +24911,12 @@
     <row r="100" ht="22" customHeight="1" s="32">
       <c r="A100" s="37" t="inlineStr">
         <is>
-          <t>AUDIT_WEAPON_SLOTS_C_64</t>
+          <t>P_STAFF_WIDEWEAK_STAFFCRYSTAL</t>
         </is>
       </c>
       <c r="B100" s="37" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>P_STAFF_WIDEWEAK_STAFFCRYSTAL</t>
         </is>
       </c>
       <c r="C100" s="37" t="inlineStr">
@@ -22425,7 +24929,11 @@
           <t>StaffCrystal</t>
         </is>
       </c>
-      <c r="E100" s="37" t="n"/>
+      <c r="E100" s="37" t="inlineStr">
+        <is>
+          <t>大范围减伤杖晶</t>
+        </is>
+      </c>
       <c r="F100" s="37" t="inlineStr">
         <is>
           <t>效果：伤害倍率-30%，爆炸范围+50%</t>
@@ -22433,34 +24941,30 @@
       </c>
       <c r="G100" s="37" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Common</t>
         </is>
       </c>
       <c r="H100" s="37" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>StaffCrystal|Numeric</t>
         </is>
       </c>
       <c r="I100" s="37" t="inlineStr">
         <is>
-          <t>false</t>
+          <t>true</t>
         </is>
       </c>
       <c r="J100" s="37" t="inlineStr">
         <is>
-          <t>Unimplemented</t>
+          <t>Approved</t>
         </is>
       </c>
       <c r="K100" s="37" t="inlineStr">
         <is>
-          <t>Disabled</t>
-        </is>
-      </c>
-      <c r="L100" s="37" t="inlineStr">
-        <is>
-          <t>Unnamed workbook row; no stable PartId assigned.</t>
-        </is>
-      </c>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="L100" s="37" t="n"/>
       <c r="M100" s="37" t="inlineStr">
         <is>
           <t>武器插槽C</t>
@@ -22473,24 +24977,22 @@
       </c>
       <c r="O100" s="37" t="inlineStr">
         <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="P100" s="37" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="P100" s="37" t="n">
+        <v>30</v>
       </c>
     </row>
     <row r="101" ht="22" customHeight="1" s="32">
       <c r="A101" s="37" t="inlineStr">
         <is>
-          <t>AUDIT_WEAPON_SLOTS_C_65</t>
+          <t>P_STAFF_NARROWSTRONG_STAFFCRYSTAL</t>
         </is>
       </c>
       <c r="B101" s="37" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>P_STAFF_NARROWSTRONG_STAFFCRYSTAL</t>
         </is>
       </c>
       <c r="C101" s="37" t="inlineStr">
@@ -22503,7 +25005,11 @@
           <t>StaffCrystal</t>
         </is>
       </c>
-      <c r="E101" s="37" t="n"/>
+      <c r="E101" s="37" t="inlineStr">
+        <is>
+          <t>高伤小范围杖晶</t>
+        </is>
+      </c>
       <c r="F101" s="37" t="inlineStr">
         <is>
           <t>效果：伤害倍率+70%，爆炸范围-50%</t>
@@ -22511,34 +25017,30 @@
       </c>
       <c r="G101" s="37" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Common</t>
         </is>
       </c>
       <c r="H101" s="37" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>StaffCrystal|Numeric</t>
         </is>
       </c>
       <c r="I101" s="37" t="inlineStr">
         <is>
-          <t>false</t>
+          <t>true</t>
         </is>
       </c>
       <c r="J101" s="37" t="inlineStr">
         <is>
-          <t>Unimplemented</t>
+          <t>Approved</t>
         </is>
       </c>
       <c r="K101" s="37" t="inlineStr">
         <is>
-          <t>Disabled</t>
-        </is>
-      </c>
-      <c r="L101" s="37" t="inlineStr">
-        <is>
-          <t>Unnamed workbook row; no stable PartId assigned.</t>
-        </is>
-      </c>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="L101" s="37" t="n"/>
       <c r="M101" s="37" t="inlineStr">
         <is>
           <t>武器插槽C</t>
@@ -22551,13 +25053,11 @@
       </c>
       <c r="O101" s="37" t="inlineStr">
         <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="P101" s="37" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="P101" s="37" t="n">
+        <v>30</v>
       </c>
     </row>
     <row r="102" ht="22" customHeight="1" s="32">
@@ -22641,12 +25141,12 @@
     <row r="103" ht="22" customHeight="1" s="32">
       <c r="A103" s="37" t="inlineStr">
         <is>
-          <t>AUDIT_WEAPON_SLOTS_C_67</t>
+          <t>P_STAFF_SLOWWIDE_STAFFCRYSTAL</t>
         </is>
       </c>
       <c r="B103" s="37" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>P_STAFF_SLOWWIDE_STAFFCRYSTAL</t>
         </is>
       </c>
       <c r="C103" s="37" t="inlineStr">
@@ -22659,7 +25159,11 @@
           <t>StaffCrystal</t>
         </is>
       </c>
-      <c r="E103" s="37" t="n"/>
+      <c r="E103" s="37" t="inlineStr">
+        <is>
+          <t>减攻速大范围杖晶</t>
+        </is>
+      </c>
       <c r="F103" s="37" t="inlineStr">
         <is>
           <t>效果：攻击速度-30%，爆炸范围+50%</t>
@@ -22667,34 +25171,30 @@
       </c>
       <c r="G103" s="37" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Common</t>
         </is>
       </c>
       <c r="H103" s="37" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>StaffCrystal|Numeric</t>
         </is>
       </c>
       <c r="I103" s="37" t="inlineStr">
         <is>
-          <t>false</t>
+          <t>true</t>
         </is>
       </c>
       <c r="J103" s="37" t="inlineStr">
         <is>
-          <t>Unimplemented</t>
+          <t>Approved</t>
         </is>
       </c>
       <c r="K103" s="37" t="inlineStr">
         <is>
-          <t>Disabled</t>
-        </is>
-      </c>
-      <c r="L103" s="37" t="inlineStr">
-        <is>
-          <t>Unnamed workbook row; no stable PartId assigned.</t>
-        </is>
-      </c>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="L103" s="37" t="n"/>
       <c r="M103" s="37" t="inlineStr">
         <is>
           <t>武器插槽C</t>
@@ -22707,13 +25207,11 @@
       </c>
       <c r="O103" s="37" t="inlineStr">
         <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="P103" s="37" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="P103" s="37" t="n">
+        <v>30</v>
       </c>
     </row>
     <row r="104" ht="22" customHeight="1" s="32">
@@ -23109,12 +25607,12 @@
     <row r="109" ht="22" customHeight="1" s="32">
       <c r="A109" s="37" t="inlineStr">
         <is>
-          <t>AUDIT_WEAPON_SLOTS_C_73</t>
+          <t>P_WHIP_HASTE_WHIPBODY</t>
         </is>
       </c>
       <c r="B109" s="37" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>P_WHIP_HASTE_WHIPBODY</t>
         </is>
       </c>
       <c r="C109" s="37" t="inlineStr">
@@ -23127,7 +25625,11 @@
           <t>WhipBody</t>
         </is>
       </c>
-      <c r="E109" s="37" t="n"/>
+      <c r="E109" s="37" t="inlineStr">
+        <is>
+          <t>攻速鞭体</t>
+        </is>
+      </c>
       <c r="F109" s="37" t="inlineStr">
         <is>
           <t>效果：攻击速度+20%</t>
@@ -23135,34 +25637,30 @@
       </c>
       <c r="G109" s="37" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Common</t>
         </is>
       </c>
       <c r="H109" s="37" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>WhipBody|Numeric</t>
         </is>
       </c>
       <c r="I109" s="37" t="inlineStr">
         <is>
-          <t>false</t>
+          <t>true</t>
         </is>
       </c>
       <c r="J109" s="37" t="inlineStr">
         <is>
-          <t>Unimplemented</t>
+          <t>Approved</t>
         </is>
       </c>
       <c r="K109" s="37" t="inlineStr">
         <is>
-          <t>Disabled</t>
-        </is>
-      </c>
-      <c r="L109" s="37" t="inlineStr">
-        <is>
-          <t>Unnamed workbook row; no stable PartId assigned.</t>
-        </is>
-      </c>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="L109" s="37" t="n"/>
       <c r="M109" s="37" t="inlineStr">
         <is>
           <t>武器插槽C</t>
@@ -23175,24 +25673,22 @@
       </c>
       <c r="O109" s="37" t="inlineStr">
         <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="P109" s="37" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="P109" s="37" t="n">
+        <v>30</v>
       </c>
     </row>
     <row r="110" ht="22" customHeight="1" s="32">
       <c r="A110" s="37" t="inlineStr">
         <is>
-          <t>AUDIT_WEAPON_SLOTS_C_74</t>
+          <t>P_WHIP_KILLHEAL_WHIPBODY</t>
         </is>
       </c>
       <c r="B110" s="37" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>P_WHIP_KILLHEAL_WHIPBODY</t>
         </is>
       </c>
       <c r="C110" s="37" t="inlineStr">
@@ -23205,7 +25701,11 @@
           <t>WhipBody</t>
         </is>
       </c>
-      <c r="E110" s="37" t="n"/>
+      <c r="E110" s="37" t="inlineStr">
+        <is>
+          <t>击杀吸血鞭体</t>
+        </is>
+      </c>
       <c r="F110" s="37" t="inlineStr">
         <is>
           <t>效果：每击杀一名敌方单位，回复5%最大生命值</t>
@@ -23213,34 +25713,30 @@
       </c>
       <c r="G110" s="37" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Rare</t>
         </is>
       </c>
       <c r="H110" s="37" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>WhipBody|UniqueBehavior</t>
         </is>
       </c>
       <c r="I110" s="37" t="inlineStr">
         <is>
-          <t>false</t>
+          <t>true</t>
         </is>
       </c>
       <c r="J110" s="37" t="inlineStr">
         <is>
-          <t>Unimplemented</t>
+          <t>Approved</t>
         </is>
       </c>
       <c r="K110" s="37" t="inlineStr">
         <is>
-          <t>Disabled</t>
-        </is>
-      </c>
-      <c r="L110" s="37" t="inlineStr">
-        <is>
-          <t>Unnamed workbook row; no stable PartId assigned.</t>
-        </is>
-      </c>
+          <t>Implemented</t>
+        </is>
+      </c>
+      <c r="L110" s="37" t="n"/>
       <c r="M110" s="37" t="inlineStr">
         <is>
           <t>武器插槽C</t>
@@ -23253,13 +25749,11 @@
       </c>
       <c r="O110" s="37" t="inlineStr">
         <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="P110" s="37" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="P110" s="37" t="n">
+        <v>45</v>
       </c>
     </row>
     <row r="111" ht="22" customHeight="1" s="32">
@@ -23842,37 +26336,37 @@
     <dataValidation sqref="K46:K123" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" errorTitle="无效选项" error="只能从下拉列表中选择有效值。" promptTitle="请选择" prompt="请从下拉列表选择，不能输入列表外的值。" type="list" errorStyle="stop">
       <formula1>=DV_Logic_Parts_ImplementationStatus</formula1>
     </dataValidation>
-    <dataValidation sqref="S46:S55" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" errorTitle="无效选项" error="只能从下拉列表中选择有效值。" promptTitle="请选择" prompt="请从下拉列表选择，不能输入列表外的值。" type="list" errorStyle="stop">
+    <dataValidation sqref="S46:S82" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" errorTitle="无效选项" error="只能从下拉列表中选择有效值。" promptTitle="请选择" prompt="请从下拉列表选择，不能输入列表外的值。" type="list" errorStyle="stop">
       <formula1>INDIRECT("tblParts[PartId]")</formula1>
     </dataValidation>
-    <dataValidation sqref="U46:U55" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" errorTitle="无效选项" error="只能从下拉列表中选择有效值。" promptTitle="请选择" prompt="请从下拉列表选择，不能输入列表外的值。" type="list" errorStyle="stop">
+    <dataValidation sqref="U46:U82" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" errorTitle="无效选项" error="只能从下拉列表中选择有效值。" promptTitle="请选择" prompt="请从下拉列表选择，不能输入列表外的值。" type="list" errorStyle="stop">
       <formula1>=DV_Logic_PartEffects_Trigger</formula1>
     </dataValidation>
-    <dataValidation sqref="V46:V55" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" errorTitle="无效选项" error="只能从下拉列表中选择有效值。" promptTitle="请选择" prompt="请从下拉列表选择，不能输入列表外的值。" type="list" errorStyle="stop">
+    <dataValidation sqref="V46:V82" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" errorTitle="无效选项" error="只能从下拉列表中选择有效值。" promptTitle="请选择" prompt="请从下拉列表选择，不能输入列表外的值。" type="list" errorStyle="stop">
       <formula1>=DV_Logic_PartEffects_EffectKind</formula1>
     </dataValidation>
-    <dataValidation sqref="W46:W55" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" errorTitle="无效选项" error="只能从下拉列表中选择有效值。" promptTitle="请选择" prompt="请从下拉列表选择，不能输入列表外的值。" type="list" errorStyle="stop">
+    <dataValidation sqref="W46:W82" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" errorTitle="无效选项" error="只能从下拉列表中选择有效值。" promptTitle="请选择" prompt="请从下拉列表选择，不能输入列表外的值。" type="list" errorStyle="stop">
       <formula1>=DV_Logic_PartEffects_Target</formula1>
     </dataValidation>
-    <dataValidation sqref="X46:X55" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" errorTitle="无效选项" error="只能从下拉列表中选择有效值。" promptTitle="请选择" prompt="请从下拉列表选择，不能输入列表外的值。" type="list" errorStyle="stop">
+    <dataValidation sqref="X46:X82" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" errorTitle="无效选项" error="只能从下拉列表中选择有效值。" promptTitle="请选择" prompt="请从下拉列表选择，不能输入列表外的值。" type="list" errorStyle="stop">
       <formula1>=DV_Logic_PartEffects_ValueOp</formula1>
     </dataValidation>
-    <dataValidation sqref="Z46:Z55" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" errorTitle="无效选项" error="只能从下拉列表中选择有效值。" promptTitle="请选择" prompt="请从下拉列表选择，不能输入列表外的值。" type="list" errorStyle="stop">
+    <dataValidation sqref="Z46:Z82" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" errorTitle="无效选项" error="只能从下拉列表中选择有效值。" promptTitle="请选择" prompt="请从下拉列表选择，不能输入列表外的值。" type="list" errorStyle="stop">
       <formula1>=DV_Logic_PartEffects_BehaviorId</formula1>
     </dataValidation>
-    <dataValidation sqref="AA46:AA55" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" errorTitle="无效选项" error="只能从下拉列表中选择有效值。" promptTitle="请选择" prompt="请从下拉列表选择，不能输入列表外的值。" type="list" errorStyle="stop">
+    <dataValidation sqref="AA46:AA82" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" errorTitle="无效选项" error="只能从下拉列表中选择有效值。" promptTitle="请选择" prompt="请从下拉列表选择，不能输入列表外的值。" type="list" errorStyle="stop">
       <formula1>=DV_Logic_PartEffects_FormulaId</formula1>
     </dataValidation>
-    <dataValidation sqref="AB46:AB55" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" errorTitle="无效选项" error="只能从下拉列表中选择有效值。" promptTitle="请选择" prompt="请从下拉列表选择，不能输入列表外的值。" type="list" errorStyle="stop">
+    <dataValidation sqref="AB46:AB82" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" errorTitle="无效选项" error="只能从下拉列表中选择有效值。" promptTitle="请选择" prompt="请从下拉列表选择，不能输入列表外的值。" type="list" errorStyle="stop">
       <formula1>=DV_Logic_PartEffects_AttackPatternId</formula1>
     </dataValidation>
-    <dataValidation sqref="AC46:AC55" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" errorTitle="无效选项" error="只能从下拉列表中选择有效值。" promptTitle="请选择" prompt="请从下拉列表选择，不能输入列表外的值。" type="list" errorStyle="stop">
+    <dataValidation sqref="AC46:AC82" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" errorTitle="无效选项" error="只能从下拉列表中选择有效值。" promptTitle="请选择" prompt="请从下拉列表选择，不能输入列表外的值。" type="list" errorStyle="stop">
       <formula1>=DV_Logic_PartEffects_ParamName</formula1>
     </dataValidation>
-    <dataValidation sqref="AG46:AG55" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" errorTitle="无效选项" error="只能从下拉列表中选择有效值。" promptTitle="请选择" prompt="请从下拉列表选择，不能输入列表外的值。" type="list" errorStyle="stop">
+    <dataValidation sqref="AG46:AG82" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" errorTitle="无效选项" error="只能从下拉列表中选择有效值。" promptTitle="请选择" prompt="请从下拉列表选择，不能输入列表外的值。" type="list" errorStyle="stop">
       <formula1>=DV_Logic_PartEffects_StackPolicy</formula1>
     </dataValidation>
-    <dataValidation sqref="AH46:AH55" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" errorTitle="无效选项" error="只能从下拉列表中选择有效值。" promptTitle="请选择" prompt="请从下拉列表选择，不能输入列表外的值。" type="list" errorStyle="stop">
+    <dataValidation sqref="AH46:AH82" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" errorTitle="无效选项" error="只能从下拉列表中选择有效值。" promptTitle="请选择" prompt="请从下拉列表选择，不能输入列表外的值。" type="list" errorStyle="stop">
       <formula1>=DV_Logic_PartEffects_Enabled</formula1>
     </dataValidation>
     <dataValidation sqref="O46:O123" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" errorTitle="无效选项" error="只能从下拉列表中选择有效值。" promptTitle="请选择" prompt="请从下拉列表选择，不能输入列表外的值。" type="list" errorStyle="stop">

</xml_diff>

<commit_message>
[PROGRAMMER] Plan67: name all 70 weapon parts and import their icons
- ReEchoData.xlsx: assign DisplayName + unique PartId (P_AUDIT_C_*) to the 45
  audit shell parts (kept disabled); correct 2 bow DisplayNames to match icons.
- Regenerated parts.csv (70 named parts) via sync.
- Imported 70 part icon textures to /Game/ReEcho/Textures/UI/WeaponParts/Icons/
  T_....uasset, one per PartId; ResolveWeaponPartIcon lazy-load path resolves all.
- validate_project.py gate still green; no C++ change (prebuilt unchanged).
</commit_message>
<xml_diff>
--- a/Design/Data/ReEchoData.xlsx
+++ b/Design/Data/ReEchoData.xlsx
@@ -18909,7 +18909,7 @@
       </c>
       <c r="E54" s="37" t="inlineStr">
         <is>
-          <t>穿刺箭头</t>
+          <t>暴击穿透箭头</t>
         </is>
       </c>
       <c r="F54" s="37" t="inlineStr">
@@ -19060,7 +19060,7 @@
       </c>
       <c r="B55" s="37" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>P_AUDIT_C_19</t>
         </is>
       </c>
       <c r="C55" s="37" t="inlineStr">
@@ -19073,7 +19073,11 @@
           <t>Arrowhead</t>
         </is>
       </c>
-      <c r="E55" s="37" t="n"/>
+      <c r="E55" s="37" t="inlineStr">
+        <is>
+          <t>暴击流血箭头</t>
+        </is>
+      </c>
       <c r="F55" s="37" t="inlineStr">
         <is>
           <t>效果：箭命中敌人且暴击后，敌人获得【流血】，持续3秒，可以叠加</t>
@@ -19106,7 +19110,7 @@
       </c>
       <c r="L55" s="37" t="inlineStr">
         <is>
-          <t>Unnamed workbook row; no stable PartId assigned.</t>
+          <t>Disabled placeholder; part effect not yet implemented.</t>
         </is>
       </c>
       <c r="M55" s="37" t="inlineStr">
@@ -19237,7 +19241,7 @@
       </c>
       <c r="E56" s="37" t="inlineStr">
         <is>
-          <t>多发箭头</t>
+          <t>三连箭头</t>
         </is>
       </c>
       <c r="F56" s="37" t="inlineStr">
@@ -19388,7 +19392,7 @@
       </c>
       <c r="B57" s="37" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>P_AUDIT_C_21</t>
         </is>
       </c>
       <c r="C57" s="37" t="inlineStr">
@@ -19401,7 +19405,11 @@
           <t>Arrowhead</t>
         </is>
       </c>
-      <c r="E57" s="37" t="n"/>
+      <c r="E57" s="37" t="inlineStr">
+        <is>
+          <t>碎片掉落箭头</t>
+        </is>
+      </c>
       <c r="F57" s="37" t="inlineStr">
         <is>
           <t>效果：击杀一名敌方单位后，额外掉落1时间碎片</t>
@@ -19434,7 +19442,7 @@
       </c>
       <c r="L57" s="37" t="inlineStr">
         <is>
-          <t>Unnamed workbook row; no stable PartId assigned.</t>
+          <t>Disabled placeholder; part effect not yet implemented.</t>
         </is>
       </c>
       <c r="M57" s="37" t="inlineStr">
@@ -19870,7 +19878,7 @@
       </c>
       <c r="B60" s="37" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>P_AUDIT_C_24</t>
         </is>
       </c>
       <c r="C60" s="37" t="inlineStr">
@@ -19883,7 +19891,11 @@
           <t>Bowstring</t>
         </is>
       </c>
-      <c r="E60" s="37" t="n"/>
+      <c r="E60" s="37" t="inlineStr">
+        <is>
+          <t>击杀移速弓弦</t>
+        </is>
+      </c>
       <c r="F60" s="37" t="inlineStr">
         <is>
           <t>效果：击杀一名敌方单位后，移动速度+20%，持续5s。不可叠加</t>
@@ -19916,7 +19928,7 @@
       </c>
       <c r="L60" s="37" t="inlineStr">
         <is>
-          <t>Unnamed workbook row; no stable PartId assigned.</t>
+          <t>Disabled placeholder; part effect not yet implemented.</t>
         </is>
       </c>
       <c r="M60" s="37" t="inlineStr">
@@ -20032,7 +20044,7 @@
       </c>
       <c r="B61" s="37" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>P_AUDIT_C_25</t>
         </is>
       </c>
       <c r="C61" s="37" t="inlineStr">
@@ -20045,7 +20057,11 @@
           <t>Bowstring</t>
         </is>
       </c>
-      <c r="E61" s="37" t="n"/>
+      <c r="E61" s="37" t="inlineStr">
+        <is>
+          <t>连击双速弓弦</t>
+        </is>
+      </c>
       <c r="F61" s="37" t="inlineStr">
         <is>
           <t>效果：每次攻击后，攻击速度和移动速度+4%。这个效果最多叠加5层，持续5s，若1秒内没有攻击行为，层数自然流失。</t>
@@ -20078,7 +20094,7 @@
       </c>
       <c r="L61" s="37" t="inlineStr">
         <is>
-          <t>Unnamed workbook row; no stable PartId assigned.</t>
+          <t>Disabled placeholder; part effect not yet implemented.</t>
         </is>
       </c>
       <c r="M61" s="37" t="inlineStr">
@@ -20194,7 +20210,7 @@
       </c>
       <c r="B62" s="37" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>P_AUDIT_C_26</t>
         </is>
       </c>
       <c r="C62" s="37" t="inlineStr">
@@ -20207,7 +20223,11 @@
           <t>RotaryBlade</t>
         </is>
       </c>
-      <c r="E62" s="37" t="n"/>
+      <c r="E62" s="37" t="inlineStr">
+        <is>
+          <t>群攻成长旋刃</t>
+        </is>
+      </c>
       <c r="F62" s="37" t="inlineStr">
         <is>
           <t>效果：每次攻击同时命中4名敌人后，攻击范围+2%，持续5s。这个效果可以叠加。</t>
@@ -20240,7 +20260,7 @@
       </c>
       <c r="L62" s="37" t="inlineStr">
         <is>
-          <t>Unnamed workbook row; no stable PartId assigned.</t>
+          <t>Disabled placeholder; part effect not yet implemented.</t>
         </is>
       </c>
       <c r="M62" s="37" t="inlineStr">
@@ -20356,7 +20376,7 @@
       </c>
       <c r="B63" s="37" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>P_AUDIT_C_27</t>
         </is>
       </c>
       <c r="C63" s="37" t="inlineStr">
@@ -20369,7 +20389,11 @@
           <t>RotaryBlade</t>
         </is>
       </c>
-      <c r="E63" s="37" t="n"/>
+      <c r="E63" s="37" t="inlineStr">
+        <is>
+          <t>命中吸血旋刃</t>
+        </is>
+      </c>
       <c r="F63" s="37" t="inlineStr">
         <is>
           <t>效果：每次攻击，每命中一名敌方单位，回复自身1%最大生命值</t>
@@ -20402,7 +20426,7 @@
       </c>
       <c r="L63" s="37" t="inlineStr">
         <is>
-          <t>Unnamed workbook row; no stable PartId assigned.</t>
+          <t>Disabled placeholder; part effect not yet implemented.</t>
         </is>
       </c>
       <c r="M63" s="37" t="inlineStr">
@@ -20678,7 +20702,7 @@
       </c>
       <c r="B65" s="37" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>P_AUDIT_C_29</t>
         </is>
       </c>
       <c r="C65" s="37" t="inlineStr">
@@ -20691,7 +20715,11 @@
           <t>RotaryBlade</t>
         </is>
       </c>
-      <c r="E65" s="37" t="n"/>
+      <c r="E65" s="37" t="inlineStr">
+        <is>
+          <t>晕眩旋刃</t>
+        </is>
+      </c>
       <c r="F65" s="37" t="inlineStr">
         <is>
           <t>效果：每次攻击有20%概率将敌人【晕眩】，持续1s</t>
@@ -20724,7 +20752,7 @@
       </c>
       <c r="L65" s="37" t="inlineStr">
         <is>
-          <t>Unnamed workbook row; no stable PartId assigned.</t>
+          <t>Disabled placeholder; part effect not yet implemented.</t>
         </is>
       </c>
       <c r="M65" s="37" t="inlineStr">
@@ -20840,7 +20868,7 @@
       </c>
       <c r="B66" s="37" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>P_AUDIT_C_30</t>
         </is>
       </c>
       <c r="C66" s="37" t="inlineStr">
@@ -20853,7 +20881,11 @@
           <t>RotaryBlade</t>
         </is>
       </c>
-      <c r="E66" s="37" t="n"/>
+      <c r="E66" s="37" t="inlineStr">
+        <is>
+          <t>流血旋刃</t>
+        </is>
+      </c>
       <c r="F66" s="37" t="inlineStr">
         <is>
           <t>效果：敌方单位被命中3次后，获得【流血】，持续3s，可以叠加</t>
@@ -20886,7 +20918,7 @@
       </c>
       <c r="L66" s="37" t="inlineStr">
         <is>
-          <t>Unnamed workbook row; no stable PartId assigned.</t>
+          <t>Disabled placeholder; part effect not yet implemented.</t>
         </is>
       </c>
       <c r="M66" s="37" t="inlineStr">
@@ -21002,7 +21034,7 @@
       </c>
       <c r="B67" s="37" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>P_AUDIT_C_31</t>
         </is>
       </c>
       <c r="C67" s="37" t="inlineStr">
@@ -21015,7 +21047,11 @@
           <t>RotaryBlade</t>
         </is>
       </c>
-      <c r="E67" s="37" t="n"/>
+      <c r="E67" s="37" t="inlineStr">
+        <is>
+          <t>外圈增伤旋刃</t>
+        </is>
+      </c>
       <c r="F67" s="37" t="inlineStr">
         <is>
           <t>效果：外圈敌人受到的额外伤害倍率+40%</t>
@@ -21048,7 +21084,7 @@
       </c>
       <c r="L67" s="37" t="inlineStr">
         <is>
-          <t>Unnamed workbook row; no stable PartId assigned.</t>
+          <t>Disabled placeholder; part effect not yet implemented.</t>
         </is>
       </c>
       <c r="M67" s="37" t="inlineStr">
@@ -21164,7 +21200,7 @@
       </c>
       <c r="B68" s="37" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>P_AUDIT_C_32</t>
         </is>
       </c>
       <c r="C68" s="37" t="inlineStr">
@@ -21177,7 +21213,11 @@
           <t>Grip</t>
         </is>
       </c>
-      <c r="E68" s="37" t="n"/>
+      <c r="E68" s="37" t="inlineStr">
+        <is>
+          <t>镰刃命中移速握柄</t>
+        </is>
+      </c>
       <c r="F68" s="37" t="inlineStr">
         <is>
           <t>效果：每次攻击，每命中一名敌方单位，获得1%移动速度，持续5s。这个效果最多叠加30层</t>
@@ -21210,7 +21250,7 @@
       </c>
       <c r="L68" s="37" t="inlineStr">
         <is>
-          <t>Unnamed workbook row; no stable PartId assigned.</t>
+          <t>Disabled placeholder; part effect not yet implemented.</t>
         </is>
       </c>
       <c r="M68" s="37" t="inlineStr">
@@ -21326,7 +21366,7 @@
       </c>
       <c r="B69" s="37" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>P_AUDIT_C_33</t>
         </is>
       </c>
       <c r="C69" s="37" t="inlineStr">
@@ -21339,7 +21379,11 @@
           <t>Grip</t>
         </is>
       </c>
-      <c r="E69" s="37" t="n"/>
+      <c r="E69" s="37" t="inlineStr">
+        <is>
+          <t>群攻无敌握柄</t>
+        </is>
+      </c>
       <c r="F69" s="37" t="inlineStr">
         <is>
           <t>效果：攻击速度-50%。每次攻击，同时命中4名敌方单位时，获得【无敌】，持续0.5秒</t>
@@ -21372,7 +21416,7 @@
       </c>
       <c r="L69" s="37" t="inlineStr">
         <is>
-          <t>Unnamed workbook row; no stable PartId assigned.</t>
+          <t>Disabled placeholder; part effect not yet implemented.</t>
         </is>
       </c>
       <c r="M69" s="37" t="inlineStr">
@@ -21488,7 +21532,7 @@
       </c>
       <c r="B70" s="37" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>P_AUDIT_C_34</t>
         </is>
       </c>
       <c r="C70" s="37" t="inlineStr">
@@ -21501,7 +21545,11 @@
           <t>Grip</t>
         </is>
       </c>
-      <c r="E70" s="37" t="n"/>
+      <c r="E70" s="37" t="inlineStr">
+        <is>
+          <t>镰刃命中攻速握柄</t>
+        </is>
+      </c>
       <c r="F70" s="37" t="inlineStr">
         <is>
           <t>效果：每次攻击，每命中一名敌方单位，获得1%攻击速度，持续5s。这个效果最多叠加30层</t>
@@ -21534,7 +21582,7 @@
       </c>
       <c r="L70" s="37" t="inlineStr">
         <is>
-          <t>Unnamed workbook row; no stable PartId assigned.</t>
+          <t>Disabled placeholder; part effect not yet implemented.</t>
         </is>
       </c>
       <c r="M70" s="37" t="inlineStr">
@@ -21650,7 +21698,7 @@
       </c>
       <c r="B71" s="37" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>P_AUDIT_C_35</t>
         </is>
       </c>
       <c r="C71" s="37" t="inlineStr">
@@ -21663,7 +21711,11 @@
           <t>Grip</t>
         </is>
       </c>
-      <c r="E71" s="37" t="n"/>
+      <c r="E71" s="37" t="inlineStr">
+        <is>
+          <t>投掷召回链</t>
+        </is>
+      </c>
       <c r="F71" s="37" t="inlineStr">
         <is>
           <t>效果：你现在点击右键可以向前掷出镰刀并停留在其目标出。再次点击右键后，可将其召回
@@ -21700,7 +21752,7 @@
       </c>
       <c r="L71" s="37" t="inlineStr">
         <is>
-          <t>Unnamed workbook row; no stable PartId assigned.</t>
+          <t>Disabled placeholder; part effect not yet implemented.</t>
         </is>
       </c>
       <c r="M71" s="37" t="inlineStr">
@@ -22136,7 +22188,7 @@
       </c>
       <c r="B74" s="37" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>P_AUDIT_C_38</t>
         </is>
       </c>
       <c r="C74" s="37" t="inlineStr">
@@ -22149,7 +22201,11 @@
           <t>SwordBlade</t>
         </is>
       </c>
-      <c r="E74" s="37" t="n"/>
+      <c r="E74" s="37" t="inlineStr">
+        <is>
+          <t>群攻成长剑刃</t>
+        </is>
+      </c>
       <c r="F74" s="37" t="inlineStr">
         <is>
           <t>效果：每次攻击同时命中4名敌人后，攻击范围+2%，持续5s。这个效果可以叠加。</t>
@@ -22182,7 +22238,7 @@
       </c>
       <c r="L74" s="37" t="inlineStr">
         <is>
-          <t>Unnamed workbook row; no stable PartId assigned.</t>
+          <t>Disabled placeholder; part effect not yet implemented.</t>
         </is>
       </c>
       <c r="M74" s="37" t="inlineStr">
@@ -22458,7 +22514,7 @@
       </c>
       <c r="B76" s="37" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>P_AUDIT_C_40</t>
         </is>
       </c>
       <c r="C76" s="37" t="inlineStr">
@@ -22471,7 +22527,11 @@
           <t>SwordBlade</t>
         </is>
       </c>
-      <c r="E76" s="37" t="n"/>
+      <c r="E76" s="37" t="inlineStr">
+        <is>
+          <t>命中碎片剑刃</t>
+        </is>
+      </c>
       <c r="F76" s="37" t="inlineStr">
         <is>
           <t>效果：每命中5名敌方单位，掉落1时间碎片</t>
@@ -22504,7 +22564,7 @@
       </c>
       <c r="L76" s="37" t="inlineStr">
         <is>
-          <t>Unnamed workbook row; no stable PartId assigned.</t>
+          <t>Disabled placeholder; part effect not yet implemented.</t>
         </is>
       </c>
       <c r="M76" s="37" t="inlineStr">
@@ -22620,7 +22680,7 @@
       </c>
       <c r="B77" s="37" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>P_AUDIT_C_41</t>
         </is>
       </c>
       <c r="C77" s="37" t="inlineStr">
@@ -22633,7 +22693,11 @@
           <t>SwordBlade</t>
         </is>
       </c>
-      <c r="E77" s="37" t="n"/>
+      <c r="E77" s="37" t="inlineStr">
+        <is>
+          <t>暴击流血剑刃</t>
+        </is>
+      </c>
       <c r="F77" s="37" t="inlineStr">
         <is>
           <t>效果：命中敌方且暴击时，敌方单位获得【流血】，持续3s，可以叠加</t>
@@ -22666,7 +22730,7 @@
       </c>
       <c r="L77" s="37" t="inlineStr">
         <is>
-          <t>Unnamed workbook row; no stable PartId assigned.</t>
+          <t>Disabled placeholder; part effect not yet implemented.</t>
         </is>
       </c>
       <c r="M77" s="37" t="inlineStr">
@@ -22782,7 +22846,7 @@
       </c>
       <c r="B78" s="37" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>P_AUDIT_C_42</t>
         </is>
       </c>
       <c r="C78" s="37" t="inlineStr">
@@ -22795,7 +22859,11 @@
           <t>SwordBlade</t>
         </is>
       </c>
-      <c r="E78" s="37" t="n"/>
+      <c r="E78" s="37" t="inlineStr">
+        <is>
+          <t>群攻陨星剑刃</t>
+        </is>
+      </c>
       <c r="F78" s="37" t="inlineStr">
         <is>
           <t>效果：当你单次命中超过6名敌方单位时，在距离你最近的敌方单位处坠落一颗流星，造成爆炸
@@ -22830,7 +22898,7 @@
       </c>
       <c r="L78" s="37" t="inlineStr">
         <is>
-          <t>Unnamed workbook row; no stable PartId assigned.</t>
+          <t>Disabled placeholder; part effect not yet implemented.</t>
         </is>
       </c>
       <c r="M78" s="37" t="inlineStr">
@@ -23106,7 +23174,7 @@
       </c>
       <c r="B80" s="37" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>P_AUDIT_C_44</t>
         </is>
       </c>
       <c r="C80" s="37" t="inlineStr">
@@ -23119,7 +23187,11 @@
           <t>Grip</t>
         </is>
       </c>
-      <c r="E80" s="37" t="n"/>
+      <c r="E80" s="37" t="inlineStr">
+        <is>
+          <t>命中移速剑柄</t>
+        </is>
+      </c>
       <c r="F80" s="37" t="inlineStr">
         <is>
           <t>效果：每次攻击，每命中一名敌方单位，获得1%移动速度，持续5s。这个效果最多叠加30层</t>
@@ -23152,7 +23224,7 @@
       </c>
       <c r="L80" s="37" t="inlineStr">
         <is>
-          <t>Unnamed workbook row; no stable PartId assigned.</t>
+          <t>Disabled placeholder; part effect not yet implemented.</t>
         </is>
       </c>
       <c r="M80" s="37" t="inlineStr">
@@ -23268,7 +23340,7 @@
       </c>
       <c r="B81" s="37" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>P_AUDIT_C_45</t>
         </is>
       </c>
       <c r="C81" s="37" t="inlineStr">
@@ -23281,7 +23353,11 @@
           <t>Grip</t>
         </is>
       </c>
-      <c r="E81" s="37" t="n"/>
+      <c r="E81" s="37" t="inlineStr">
+        <is>
+          <t>命中攻速剑柄</t>
+        </is>
+      </c>
       <c r="F81" s="37" t="inlineStr">
         <is>
           <t>效果：每次攻击，每命中一名敌方单位，获得1%攻击速度，持续5s。这个效果最多叠加30层</t>
@@ -23314,7 +23390,7 @@
       </c>
       <c r="L81" s="37" t="inlineStr">
         <is>
-          <t>Unnamed workbook row; no stable PartId assigned.</t>
+          <t>Disabled placeholder; part effect not yet implemented.</t>
         </is>
       </c>
       <c r="M81" s="37" t="inlineStr">
@@ -23430,7 +23506,7 @@
       </c>
       <c r="B82" s="37" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>P_AUDIT_C_46</t>
         </is>
       </c>
       <c r="C82" s="37" t="inlineStr">
@@ -23443,7 +23519,11 @@
           <t>Grip</t>
         </is>
       </c>
-      <c r="E82" s="37" t="n"/>
+      <c r="E82" s="37" t="inlineStr">
+        <is>
+          <t>晕眩剑柄</t>
+        </is>
+      </c>
       <c r="F82" s="37" t="inlineStr">
         <is>
           <t>效果：每次攻击，有20%概率将敌人【晕眩】，持续1s</t>
@@ -23476,7 +23556,7 @@
       </c>
       <c r="L82" s="37" t="inlineStr">
         <is>
-          <t>Unnamed workbook row; no stable PartId assigned.</t>
+          <t>Disabled placeholder; part effect not yet implemented.</t>
         </is>
       </c>
       <c r="M82" s="37" t="inlineStr">
@@ -23744,7 +23824,7 @@
       </c>
       <c r="B85" s="37" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>P_AUDIT_C_49</t>
         </is>
       </c>
       <c r="C85" s="37" t="inlineStr">
@@ -23757,7 +23837,11 @@
           <t>Muzzle</t>
         </is>
       </c>
-      <c r="E85" s="37" t="n"/>
+      <c r="E85" s="37" t="inlineStr">
+        <is>
+          <t>极限蓄能枪口</t>
+        </is>
+      </c>
       <c r="F85" s="37" t="inlineStr">
         <is>
           <t>效果：攻击速度-500%，伤害倍率+180%</t>
@@ -23790,7 +23874,7 @@
       </c>
       <c r="L85" s="37" t="inlineStr">
         <is>
-          <t>Unnamed workbook row; no stable PartId assigned.</t>
+          <t>Disabled placeholder; part effect not yet implemented.</t>
         </is>
       </c>
       <c r="M85" s="37" t="inlineStr">
@@ -23822,7 +23906,7 @@
       </c>
       <c r="B86" s="37" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>P_AUDIT_C_50</t>
         </is>
       </c>
       <c r="C86" s="37" t="inlineStr">
@@ -23835,7 +23919,11 @@
           <t>Muzzle</t>
         </is>
       </c>
-      <c r="E86" s="37" t="n"/>
+      <c r="E86" s="37" t="inlineStr">
+        <is>
+          <t>连发枪口</t>
+        </is>
+      </c>
       <c r="F86" s="37" t="inlineStr">
         <is>
           <t>效果：攻击速度+50%</t>
@@ -23868,7 +23956,7 @@
       </c>
       <c r="L86" s="37" t="inlineStr">
         <is>
-          <t>Unnamed workbook row; no stable PartId assigned.</t>
+          <t>Disabled placeholder; part effect not yet implemented.</t>
         </is>
       </c>
       <c r="M86" s="37" t="inlineStr">
@@ -23900,7 +23988,7 @@
       </c>
       <c r="B87" s="37" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>P_AUDIT_C_51</t>
         </is>
       </c>
       <c r="C87" s="37" t="inlineStr">
@@ -23913,7 +24001,11 @@
           <t>Muzzle</t>
         </is>
       </c>
-      <c r="E87" s="37" t="n"/>
+      <c r="E87" s="37" t="inlineStr">
+        <is>
+          <t>爆炸枪口</t>
+        </is>
+      </c>
       <c r="F87" s="37" t="inlineStr">
         <is>
           <t>效果：子弹变为爆炸物。爆炸范围1m</t>
@@ -23946,7 +24038,7 @@
       </c>
       <c r="L87" s="37" t="inlineStr">
         <is>
-          <t>Unnamed workbook row; no stable PartId assigned.</t>
+          <t>Disabled placeholder; part effect not yet implemented.</t>
         </is>
       </c>
       <c r="M87" s="37" t="inlineStr">
@@ -23978,7 +24070,7 @@
       </c>
       <c r="B88" s="37" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>P_AUDIT_C_52</t>
         </is>
       </c>
       <c r="C88" s="37" t="inlineStr">
@@ -23991,7 +24083,11 @@
           <t>Muzzle</t>
         </is>
       </c>
-      <c r="E88" s="37" t="n"/>
+      <c r="E88" s="37" t="inlineStr">
+        <is>
+          <t>暴击穿透枪口</t>
+        </is>
+      </c>
       <c r="F88" s="37" t="inlineStr">
         <is>
           <t>效果：子弹命中敌人且暴击后，会穿透该敌人</t>
@@ -24024,7 +24120,7 @@
       </c>
       <c r="L88" s="37" t="inlineStr">
         <is>
-          <t>Unnamed workbook row; no stable PartId assigned.</t>
+          <t>Disabled placeholder; part effect not yet implemented.</t>
         </is>
       </c>
       <c r="M88" s="37" t="inlineStr">
@@ -24056,7 +24152,7 @@
       </c>
       <c r="B89" s="37" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>P_AUDIT_C_53</t>
         </is>
       </c>
       <c r="C89" s="37" t="inlineStr">
@@ -24069,7 +24165,11 @@
           <t>Muzzle</t>
         </is>
       </c>
-      <c r="E89" s="37" t="n"/>
+      <c r="E89" s="37" t="inlineStr">
+        <is>
+          <t>命中流血枪口</t>
+        </is>
+      </c>
       <c r="F89" s="37" t="inlineStr">
         <is>
           <t>效果：每次命中敌方单位时，敌方单位有30%概率获得【流血】，持续3s，可以叠加</t>
@@ -24102,7 +24202,7 @@
       </c>
       <c r="L89" s="37" t="inlineStr">
         <is>
-          <t>Unnamed workbook row; no stable PartId assigned.</t>
+          <t>Disabled placeholder; part effect not yet implemented.</t>
         </is>
       </c>
       <c r="M89" s="37" t="inlineStr">
@@ -24134,7 +24234,7 @@
       </c>
       <c r="B90" s="37" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>P_AUDIT_C_54</t>
         </is>
       </c>
       <c r="C90" s="37" t="inlineStr">
@@ -24147,7 +24247,11 @@
           <t>GunAction</t>
         </is>
       </c>
-      <c r="E90" s="37" t="n"/>
+      <c r="E90" s="37" t="inlineStr">
+        <is>
+          <t>命中吸血枪机</t>
+        </is>
+      </c>
       <c r="F90" s="37" t="inlineStr">
         <is>
           <t>效果：每次命中敌方单位，回复1%最大生命值</t>
@@ -24180,7 +24284,7 @@
       </c>
       <c r="L90" s="37" t="inlineStr">
         <is>
-          <t>Unnamed workbook row; no stable PartId assigned.</t>
+          <t>Disabled placeholder; part effect not yet implemented.</t>
         </is>
       </c>
       <c r="M90" s="37" t="inlineStr">
@@ -24212,7 +24316,7 @@
       </c>
       <c r="B91" s="37" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>P_AUDIT_C_55</t>
         </is>
       </c>
       <c r="C91" s="37" t="inlineStr">
@@ -24225,7 +24329,11 @@
           <t>GunAction</t>
         </is>
       </c>
-      <c r="E91" s="37" t="n"/>
+      <c r="E91" s="37" t="inlineStr">
+        <is>
+          <t>命中碎片枪机</t>
+        </is>
+      </c>
       <c r="F91" s="37" t="inlineStr">
         <is>
           <t>效果：每命中5名敌方单位，掉落1时间碎片</t>
@@ -24258,7 +24366,7 @@
       </c>
       <c r="L91" s="37" t="inlineStr">
         <is>
-          <t>Unnamed workbook row; no stable PartId assigned.</t>
+          <t>Disabled placeholder; part effect not yet implemented.</t>
         </is>
       </c>
       <c r="M91" s="37" t="inlineStr">
@@ -24290,7 +24398,7 @@
       </c>
       <c r="B92" s="37" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>P_AUDIT_C_56</t>
         </is>
       </c>
       <c r="C92" s="37" t="inlineStr">
@@ -24303,7 +24411,11 @@
           <t>GunAction</t>
         </is>
       </c>
-      <c r="E92" s="37" t="n"/>
+      <c r="E92" s="37" t="inlineStr">
+        <is>
+          <t>连射攻速枪机</t>
+        </is>
+      </c>
       <c r="F92" s="37" t="inlineStr">
         <is>
           <t>效果：每次攻击，获得1%攻击速度，持续5s。这个效果最多叠加30层</t>
@@ -24336,7 +24448,7 @@
       </c>
       <c r="L92" s="37" t="inlineStr">
         <is>
-          <t>Unnamed workbook row; no stable PartId assigned.</t>
+          <t>Disabled placeholder; part effect not yet implemented.</t>
         </is>
       </c>
       <c r="M92" s="37" t="inlineStr">
@@ -24368,7 +24480,7 @@
       </c>
       <c r="B93" s="37" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>P_AUDIT_C_57</t>
         </is>
       </c>
       <c r="C93" s="37" t="inlineStr">
@@ -24381,7 +24493,11 @@
           <t>GunAction</t>
         </is>
       </c>
-      <c r="E93" s="37" t="n"/>
+      <c r="E93" s="37" t="inlineStr">
+        <is>
+          <t>连射移速枪机</t>
+        </is>
+      </c>
       <c r="F93" s="37" t="inlineStr">
         <is>
           <t>效果：每次攻击，获得1%移动速度，持续5s。这个效果最多叠加30层</t>
@@ -24414,7 +24530,7 @@
       </c>
       <c r="L93" s="37" t="inlineStr">
         <is>
-          <t>Unnamed workbook row; no stable PartId assigned.</t>
+          <t>Disabled placeholder; part effect not yet implemented.</t>
         </is>
       </c>
       <c r="M93" s="37" t="inlineStr">
@@ -24446,7 +24562,7 @@
       </c>
       <c r="B94" s="37" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>P_AUDIT_C_58</t>
         </is>
       </c>
       <c r="C94" s="37" t="inlineStr">
@@ -24459,7 +24575,11 @@
           <t>StaffBody</t>
         </is>
       </c>
-      <c r="E94" s="37" t="n"/>
+      <c r="E94" s="37" t="inlineStr">
+        <is>
+          <t>命中吸血杖体</t>
+        </is>
+      </c>
       <c r="F94" s="37" t="inlineStr">
         <is>
           <t>效果：每次攻击，每命中一名敌方单位，回复自身1%最大生命值</t>
@@ -24492,7 +24612,7 @@
       </c>
       <c r="L94" s="37" t="inlineStr">
         <is>
-          <t>Unnamed workbook row; no stable PartId assigned.</t>
+          <t>Disabled placeholder; part effect not yet implemented.</t>
         </is>
       </c>
       <c r="M94" s="37" t="inlineStr">
@@ -24600,7 +24720,7 @@
       </c>
       <c r="B96" s="37" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>P_AUDIT_C_60</t>
         </is>
       </c>
       <c r="C96" s="37" t="inlineStr">
@@ -24613,7 +24733,11 @@
           <t>StaffBody</t>
         </is>
       </c>
-      <c r="E96" s="37" t="n"/>
+      <c r="E96" s="37" t="inlineStr">
+        <is>
+          <t>命中移速杖体</t>
+        </is>
+      </c>
       <c r="F96" s="37" t="inlineStr">
         <is>
           <t>效果：每次攻击，每命中一名敌方单位，获得1%移动速度，持续5s。这个效果最多叠加30层</t>
@@ -24646,7 +24770,7 @@
       </c>
       <c r="L96" s="37" t="inlineStr">
         <is>
-          <t>Unnamed workbook row; no stable PartId assigned.</t>
+          <t>Disabled placeholder; part effect not yet implemented.</t>
         </is>
       </c>
       <c r="M96" s="37" t="inlineStr">
@@ -24678,7 +24802,7 @@
       </c>
       <c r="B97" s="37" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>P_AUDIT_C_61</t>
         </is>
       </c>
       <c r="C97" s="37" t="inlineStr">
@@ -24691,7 +24815,11 @@
           <t>StaffBody</t>
         </is>
       </c>
-      <c r="E97" s="37" t="n"/>
+      <c r="E97" s="37" t="inlineStr">
+        <is>
+          <t>命中攻速杖体</t>
+        </is>
+      </c>
       <c r="F97" s="37" t="inlineStr">
         <is>
           <t>效果：每次攻击，每命中一名敌方单位，获得1%攻击速度，持续5s。这个效果最多叠加30层</t>
@@ -24724,7 +24852,7 @@
       </c>
       <c r="L97" s="37" t="inlineStr">
         <is>
-          <t>Unnamed workbook row; no stable PartId assigned.</t>
+          <t>Disabled placeholder; part effect not yet implemented.</t>
         </is>
       </c>
       <c r="M97" s="37" t="inlineStr">
@@ -24756,7 +24884,7 @@
       </c>
       <c r="B98" s="37" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>P_AUDIT_C_62</t>
         </is>
       </c>
       <c r="C98" s="37" t="inlineStr">
@@ -24769,7 +24897,11 @@
           <t>StaffBody</t>
         </is>
       </c>
-      <c r="E98" s="37" t="n"/>
+      <c r="E98" s="37" t="inlineStr">
+        <is>
+          <t>群攻爆炸成长杖体</t>
+        </is>
+      </c>
       <c r="F98" s="37" t="inlineStr">
         <is>
           <t>效果：每次攻击同时命中4名敌人后，爆炸范围+2%，持续5s。这个效果可以叠加。</t>
@@ -24802,7 +24934,7 @@
       </c>
       <c r="L98" s="37" t="inlineStr">
         <is>
-          <t>Unnamed workbook row; no stable PartId assigned.</t>
+          <t>Disabled placeholder; part effect not yet implemented.</t>
         </is>
       </c>
       <c r="M98" s="37" t="inlineStr">
@@ -24834,7 +24966,7 @@
       </c>
       <c r="B99" s="37" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>P_AUDIT_C_63</t>
         </is>
       </c>
       <c r="C99" s="37" t="inlineStr">
@@ -24847,7 +24979,11 @@
           <t>StaffBody</t>
         </is>
       </c>
-      <c r="E99" s="37" t="n"/>
+      <c r="E99" s="37" t="inlineStr">
+        <is>
+          <t>近战副手杖体</t>
+        </is>
+      </c>
       <c r="F99" s="37" t="inlineStr">
         <is>
           <t>效果：你现在点击右键，可以挥动法杖进行近战攻击
@@ -24884,7 +25020,7 @@
       </c>
       <c r="L99" s="37" t="inlineStr">
         <is>
-          <t>Unnamed workbook row; no stable PartId assigned.</t>
+          <t>Disabled placeholder; part effect not yet implemented.</t>
         </is>
       </c>
       <c r="M99" s="37" t="inlineStr">
@@ -25068,7 +25204,7 @@
       </c>
       <c r="B102" s="37" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>P_AUDIT_C_66</t>
         </is>
       </c>
       <c r="C102" s="37" t="inlineStr">
@@ -25081,7 +25217,11 @@
           <t>StaffCrystal</t>
         </is>
       </c>
-      <c r="E102" s="37" t="n"/>
+      <c r="E102" s="37" t="inlineStr">
+        <is>
+          <t>命中碎片杖晶</t>
+        </is>
+      </c>
       <c r="F102" s="37" t="inlineStr">
         <is>
           <t>效果：每命中5名敌方单位，掉落1时间碎片</t>
@@ -25114,7 +25254,7 @@
       </c>
       <c r="L102" s="37" t="inlineStr">
         <is>
-          <t>Unnamed workbook row; no stable PartId assigned.</t>
+          <t>Disabled placeholder; part effect not yet implemented.</t>
         </is>
       </c>
       <c r="M102" s="37" t="inlineStr">
@@ -25222,7 +25362,7 @@
       </c>
       <c r="B104" s="37" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>P_AUDIT_C_68</t>
         </is>
       </c>
       <c r="C104" s="37" t="inlineStr">
@@ -25235,7 +25375,11 @@
           <t>StaffCrystal</t>
         </is>
       </c>
-      <c r="E104" s="37" t="n"/>
+      <c r="E104" s="37" t="inlineStr">
+        <is>
+          <t>中心晕眩杖晶</t>
+        </is>
+      </c>
       <c r="F104" s="37" t="inlineStr">
         <is>
           <t>效果：爆炸范围中心1m的敌人被【眩晕】，持续1s</t>
@@ -25268,7 +25412,7 @@
       </c>
       <c r="L104" s="37" t="inlineStr">
         <is>
-          <t>Unnamed workbook row; no stable PartId assigned.</t>
+          <t>Disabled placeholder; part effect not yet implemented.</t>
         </is>
       </c>
       <c r="M104" s="37" t="inlineStr">
@@ -25300,7 +25444,7 @@
       </c>
       <c r="B105" s="37" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>P_AUDIT_C_69</t>
         </is>
       </c>
       <c r="C105" s="37" t="inlineStr">
@@ -25313,7 +25457,11 @@
           <t>StaffCrystal</t>
         </is>
       </c>
-      <c r="E105" s="37" t="n"/>
+      <c r="E105" s="37" t="inlineStr">
+        <is>
+          <t>单体高伤杖晶</t>
+        </is>
+      </c>
       <c r="F105" s="37" t="inlineStr">
         <is>
           <t>效果：炮弹不会爆炸。伤害倍率+70%</t>
@@ -25346,7 +25494,7 @@
       </c>
       <c r="L105" s="37" t="inlineStr">
         <is>
-          <t>Unnamed workbook row; no stable PartId assigned.</t>
+          <t>Disabled placeholder; part effect not yet implemented.</t>
         </is>
       </c>
       <c r="M105" s="37" t="inlineStr">
@@ -25378,7 +25526,7 @@
       </c>
       <c r="B106" s="37" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>P_AUDIT_C_70</t>
         </is>
       </c>
       <c r="C106" s="37" t="inlineStr">
@@ -25391,7 +25539,11 @@
           <t>WhipBody</t>
         </is>
       </c>
-      <c r="E106" s="37" t="n"/>
+      <c r="E106" s="37" t="inlineStr">
+        <is>
+          <t>暴击流血鞭体</t>
+        </is>
+      </c>
       <c r="F106" s="37" t="inlineStr">
         <is>
           <t>效果：命中敌人且暴击后，敌人获得【流血】，持续3秒，可以叠加</t>
@@ -25424,7 +25576,7 @@
       </c>
       <c r="L106" s="37" t="inlineStr">
         <is>
-          <t>Unnamed workbook row; no stable PartId assigned.</t>
+          <t>Disabled placeholder; part effect not yet implemented.</t>
         </is>
       </c>
       <c r="M106" s="37" t="inlineStr">
@@ -25456,7 +25608,7 @@
       </c>
       <c r="B107" s="37" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>P_AUDIT_C_71</t>
         </is>
       </c>
       <c r="C107" s="37" t="inlineStr">
@@ -25469,7 +25621,11 @@
           <t>WhipBody</t>
         </is>
       </c>
-      <c r="E107" s="37" t="n"/>
+      <c r="E107" s="37" t="inlineStr">
+        <is>
+          <t>慢攻重击鞭体</t>
+        </is>
+      </c>
       <c r="F107" s="37" t="inlineStr">
         <is>
           <t>效果：攻击速度-30%，伤害倍率+40%（第二段+80%）</t>
@@ -25502,7 +25658,7 @@
       </c>
       <c r="L107" s="37" t="inlineStr">
         <is>
-          <t>Unnamed workbook row; no stable PartId assigned.</t>
+          <t>Disabled placeholder; part effect not yet implemented.</t>
         </is>
       </c>
       <c r="M107" s="37" t="inlineStr">
@@ -25534,7 +25690,7 @@
       </c>
       <c r="B108" s="37" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>P_AUDIT_C_72</t>
         </is>
       </c>
       <c r="C108" s="37" t="inlineStr">
@@ -25547,7 +25703,11 @@
           <t>WhipBody</t>
         </is>
       </c>
-      <c r="E108" s="37" t="n"/>
+      <c r="E108" s="37" t="inlineStr">
+        <is>
+          <t>去击退重击鞭体</t>
+        </is>
+      </c>
       <c r="F108" s="37" t="inlineStr">
         <is>
           <t>效果：第一段攻击不再附带【击退】效果，伤害倍率+40%（第二段+80%）</t>
@@ -25580,7 +25740,7 @@
       </c>
       <c r="L108" s="37" t="inlineStr">
         <is>
-          <t>Unnamed workbook row; no stable PartId assigned.</t>
+          <t>Disabled placeholder; part effect not yet implemented.</t>
         </is>
       </c>
       <c r="M108" s="37" t="inlineStr">
@@ -25764,7 +25924,7 @@
       </c>
       <c r="B111" s="37" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>P_AUDIT_C_75</t>
         </is>
       </c>
       <c r="C111" s="37" t="inlineStr">
@@ -25777,7 +25937,11 @@
           <t>Grip</t>
         </is>
       </c>
-      <c r="E111" s="37" t="n"/>
+      <c r="E111" s="37" t="inlineStr">
+        <is>
+          <t>第一段横扫握柄</t>
+        </is>
+      </c>
       <c r="F111" s="37" t="inlineStr">
         <is>
           <t>效果：只触发第一段攻击，并且第一段攻击外圈敌人也会受到额外伤害</t>
@@ -25810,7 +25974,7 @@
       </c>
       <c r="L111" s="37" t="inlineStr">
         <is>
-          <t>Unnamed workbook row; no stable PartId assigned.</t>
+          <t>Disabled placeholder; part effect not yet implemented.</t>
         </is>
       </c>
       <c r="M111" s="37" t="inlineStr">
@@ -25842,7 +26006,7 @@
       </c>
       <c r="B112" s="37" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>P_AUDIT_C_76</t>
         </is>
       </c>
       <c r="C112" s="37" t="inlineStr">
@@ -25855,7 +26019,11 @@
           <t>Grip</t>
         </is>
       </c>
-      <c r="E112" s="37" t="n"/>
+      <c r="E112" s="37" t="inlineStr">
+        <is>
+          <t>第二段刺击握柄</t>
+        </is>
+      </c>
       <c r="F112" s="37" t="inlineStr">
         <is>
           <t>效果：只触发第二段攻击，第二段攻击角度为60°</t>
@@ -25888,7 +26056,7 @@
       </c>
       <c r="L112" s="37" t="inlineStr">
         <is>
-          <t>Unnamed workbook row; no stable PartId assigned.</t>
+          <t>Disabled placeholder; part effect not yet implemented.</t>
         </is>
       </c>
       <c r="M112" s="37" t="inlineStr">
@@ -25920,7 +26088,7 @@
       </c>
       <c r="B113" s="37" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>P_AUDIT_C_77</t>
         </is>
       </c>
       <c r="C113" s="37" t="inlineStr">
@@ -25933,7 +26101,11 @@
           <t>Grip</t>
         </is>
       </c>
-      <c r="E113" s="37" t="n"/>
+      <c r="E113" s="37" t="inlineStr">
+        <is>
+          <t>鞭术命中移速握柄</t>
+        </is>
+      </c>
       <c r="F113" s="37" t="inlineStr">
         <is>
           <t>效果：每次攻击，每命中一名敌方单位，获得1%移动速度，持续5s。这个效果最多叠加30层</t>
@@ -25966,7 +26138,7 @@
       </c>
       <c r="L113" s="37" t="inlineStr">
         <is>
-          <t>Unnamed workbook row; no stable PartId assigned.</t>
+          <t>Disabled placeholder; part effect not yet implemented.</t>
         </is>
       </c>
       <c r="M113" s="37" t="inlineStr">
@@ -25998,7 +26170,7 @@
       </c>
       <c r="B114" s="37" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>P_AUDIT_C_78</t>
         </is>
       </c>
       <c r="C114" s="37" t="inlineStr">
@@ -26011,7 +26183,11 @@
           <t>Grip</t>
         </is>
       </c>
-      <c r="E114" s="37" t="n"/>
+      <c r="E114" s="37" t="inlineStr">
+        <is>
+          <t>鞭术命中攻速握柄</t>
+        </is>
+      </c>
       <c r="F114" s="37" t="inlineStr">
         <is>
           <t>效果：每次攻击，每命中一名敌方单位，获得1%攻击速度，持续5s。这个效果最多叠加30层</t>
@@ -26044,7 +26220,7 @@
       </c>
       <c r="L114" s="37" t="inlineStr">
         <is>
-          <t>Unnamed workbook row; no stable PartId assigned.</t>
+          <t>Disabled placeholder; part effect not yet implemented.</t>
         </is>
       </c>
       <c r="M114" s="37" t="inlineStr">
@@ -26076,7 +26252,7 @@
       </c>
       <c r="B115" s="37" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>P_AUDIT_C_79</t>
         </is>
       </c>
       <c r="C115" s="37" t="inlineStr">
@@ -26089,7 +26265,11 @@
           <t>Grip</t>
         </is>
       </c>
-      <c r="E115" s="37" t="n"/>
+      <c r="E115" s="37" t="inlineStr">
+        <is>
+          <t>群攻延伸握柄</t>
+        </is>
+      </c>
       <c r="F115" s="37" t="inlineStr">
         <is>
           <t>效果：每次攻击同时命中4名敌人后，攻击范围+2%，持续5s。这个效果可以叠加。</t>
@@ -26122,7 +26302,7 @@
       </c>
       <c r="L115" s="37" t="inlineStr">
         <is>
-          <t>Unnamed workbook row; no stable PartId assigned.</t>
+          <t>Disabled placeholder; part effect not yet implemented.</t>
         </is>
       </c>
       <c r="M115" s="37" t="inlineStr">

</xml_diff>

<commit_message>
[PROGRAMMER] Plan67 Step1: shop price-ranges & drop-levels data layer (xlsx tables + sync export + schema/manifest/validate registration, prebuilt refresh)
Design/Data/ReEchoData.xlsx 缁忔祹绯荤粺 sheet: add tblShopPriceRanges (8 PriceCategory ranges) and tblShopDropLevels (8 encounter tiers); update _ExportMap; move 缁忔祹绯荤粺 out of LOCKED_REFERENCE_SHEETS (authored data table, not locked reference).

scripts/data/sync_xlsx_to_csv.py: register tblShopPriceRanges->shop_price_ranges.csv, tblShopDropLevels->shop_drop_levels.csv; remove 缁忔祹绯荤粺 from LOCKED_REFERENCE_SHEETS.

Content/Data/csv_schema.csv + reecho_data_manifest.csv: register both tables; scripts/validate_project.py: add CSV_TABLES entries + validate_table calls.

Content/Data/shop_price_ranges.csv, shop_drop_levels.csv: generated production CSV (sync publish PASS). Binaries/Win64: prebuilt refresh source b00fc4fdefe4 to satisfy sync gate.
</commit_message>
<xml_diff>
--- a/Design/Data/ReEchoData.xlsx
+++ b/Design/Data/ReEchoData.xlsx
@@ -574,7 +574,31 @@
 </file>
 
 <file path=xl/tables/table15.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="15" name="tblWorkbookMeta" displayName="tblWorkbookMeta" ref="A1:B8" headerRowCount="1" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="15" name="tblShopPriceRanges" displayName="tblShopPriceRanges" ref="A1:C9" headerRowCount="1">
+  <autoFilter ref="A1:C9"/>
+  <tableColumns count="3">
+    <tableColumn id="1" name="PriceCategory"/>
+    <tableColumn id="2" name="MinPrice"/>
+    <tableColumn id="3" name="MaxPrice"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
+</table>
+</file>
+
+<file path=xl/tables/table16.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="16" name="tblShopDropLevels" displayName="tblShopDropLevels" ref="A12:C20" headerRowCount="1">
+  <autoFilter ref="A12:C20"/>
+  <tableColumns count="3">
+    <tableColumn id="1" name="EncounterIndex"/>
+    <tableColumn id="2" name="FreeTier"/>
+    <tableColumn id="3" name="ShopTiers"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
+</table>
+</file>
+
+<file path=xl/tables/table17.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="17" name="tblWorkbookMeta" displayName="tblWorkbookMeta" ref="A1:B8" headerRowCount="1" totalsRowShown="0">
   <tableColumns count="2">
     <tableColumn id="1" name="Key"/>
     <tableColumn id="2" name="Value"/>
@@ -583,8 +607,8 @@
 </table>
 </file>
 
-<file path=xl/tables/table16.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="16" name="tblExportMap" displayName="tblExportMap" ref="A1:E18" headerRowCount="1" totalsRowShown="0">
+<file path=xl/tables/table18.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="18" name="tblExportMap" displayName="tblExportMap" ref="A1:E20" headerRowCount="1" totalsRowShown="0">
   <tableColumns count="5">
     <tableColumn id="1" name="SheetName"/>
     <tableColumn id="2" name="TableName"/>
@@ -596,8 +620,8 @@
 </table>
 </file>
 
-<file path=xl/tables/table17.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="17" name="tblRuntimeSmoke" displayName="tblRuntimeSmoke" ref="A3:J4" headerRowCount="1" totalsRowShown="0">
+<file path=xl/tables/table19.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="19" name="tblRuntimeSmoke" displayName="tblRuntimeSmoke" ref="A3:J4" headerRowCount="1" totalsRowShown="0">
   <tableColumns count="10">
     <tableColumn id="1" name="Id"/>
     <tableColumn id="2" name="DisplayNameKey"/>
@@ -611,35 +635,6 @@
     <tableColumn id="10" name="ModifierOp"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
-</file>
-
-<file path=xl/tables/table18.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="18" name="tblRuntimeSmokeEffects" displayName="tblRuntimeSmokeEffects" ref="L3:P4" headerRowCount="1" totalsRowShown="0">
-  <tableColumns count="5">
-    <tableColumn id="1" name="Id"/>
-    <tableColumn id="2" name="RuntimeRowId"/>
-    <tableColumn id="3" name="ParamName"/>
-    <tableColumn id="4" name="ValueOp"/>
-    <tableColumn id="5" name="Value"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
-</file>
-
-<file path=xl/tables/table19.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="19" name="tblAttributes" displayName="tblAttributes" ref="A1:G9" headerRowCount="1">
-  <autoFilter ref="A1:G9"/>
-  <tableColumns count="7">
-    <tableColumn id="1" name="Id"/>
-    <tableColumn id="2" name="DisplayName"/>
-    <tableColumn id="3" name="Tier"/>
-    <tableColumn id="4" name="IconName"/>
-    <tableColumn id="5" name="ValueKind"/>
-    <tableColumn id="6" name="DisplayOrder"/>
-    <tableColumn id="7" name="Explanation"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
 </table>
 </file>
 
@@ -667,6 +662,35 @@
     <tableColumn id="18" name="DisabledReason"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table20.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="20" name="tblRuntimeSmokeEffects" displayName="tblRuntimeSmokeEffects" ref="L3:P4" headerRowCount="1" totalsRowShown="0">
+  <tableColumns count="5">
+    <tableColumn id="1" name="Id"/>
+    <tableColumn id="2" name="RuntimeRowId"/>
+    <tableColumn id="3" name="ParamName"/>
+    <tableColumn id="4" name="ValueOp"/>
+    <tableColumn id="5" name="Value"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table21.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="21" name="tblAttributes" displayName="tblAttributes" ref="A1:G9" headerRowCount="1">
+  <autoFilter ref="A1:G9"/>
+  <tableColumns count="7">
+    <tableColumn id="1" name="Id"/>
+    <tableColumn id="2" name="DisplayName"/>
+    <tableColumn id="3" name="Tier"/>
+    <tableColumn id="4" name="IconName"/>
+    <tableColumn id="5" name="ValueKind"/>
+    <tableColumn id="6" name="DisplayOrder"/>
+    <tableColumn id="7" name="Explanation"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
 </table>
 </file>
 
@@ -2644,7 +2668,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:E20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13"/>
   <cols>
     <col width="13" customWidth="1" style="28" min="1" max="1"/>
@@ -3137,6 +3161,60 @@
       <c r="E18" s="0" t="inlineStr">
         <is>
           <t>100</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="0" t="inlineStr">
+        <is>
+          <t>经济系统</t>
+        </is>
+      </c>
+      <c r="B19" s="0" t="inlineStr">
+        <is>
+          <t>tblShopPriceRanges</t>
+        </is>
+      </c>
+      <c r="C19" s="0" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D19" s="0" t="inlineStr">
+        <is>
+          <t>shop_price_ranges.csv</t>
+        </is>
+      </c>
+      <c r="E19" s="0" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="0" t="inlineStr">
+        <is>
+          <t>经济系统</t>
+        </is>
+      </c>
+      <c r="B20" s="0" t="inlineStr">
+        <is>
+          <t>tblShopDropLevels</t>
+        </is>
+      </c>
+      <c r="C20" s="0" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D20" s="0" t="inlineStr">
+        <is>
+          <t>shop_drop_levels.csv</t>
+        </is>
+      </c>
+      <c r="E20" s="0" t="inlineStr">
+        <is>
+          <t>18</t>
         </is>
       </c>
     </row>
@@ -27220,18 +27298,246 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="L1:L1"/>
+  <dimension ref="A1:L20"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="13.81640625" defaultRowHeight="13"/>
   <sheetData>
     <row r="1" ht="39" customHeight="1" s="32">
+      <c r="A1" s="0" t="inlineStr">
+        <is>
+          <t>PriceCategory</t>
+        </is>
+      </c>
+      <c r="B1" s="0" t="inlineStr">
+        <is>
+          <t>MinPrice</t>
+        </is>
+      </c>
+      <c r="C1" s="0" t="inlineStr">
+        <is>
+          <t>MaxPrice</t>
+        </is>
+      </c>
       <c r="L1" s="26" t="inlineStr">
         <is>
           <t>ReferenceOnly：经济系统尚未迁移为生产 Table，本 Sheet 仅作说明。</t>
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" s="38" t="inlineStr">
+        <is>
+          <t>Core_Primordial</t>
+        </is>
+      </c>
+      <c r="B2" s="38" t="n">
+        <v>10</v>
+      </c>
+      <c r="C2" s="38" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="38" t="inlineStr">
+        <is>
+          <t>Core_Element</t>
+        </is>
+      </c>
+      <c r="B3" s="38" t="n">
+        <v>20</v>
+      </c>
+      <c r="C3" s="38" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="38" t="inlineStr">
+        <is>
+          <t>Rune</t>
+        </is>
+      </c>
+      <c r="B4" s="38" t="n">
+        <v>30</v>
+      </c>
+      <c r="C4" s="38" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="38" t="inlineStr">
+        <is>
+          <t>Weapon</t>
+        </is>
+      </c>
+      <c r="B5" s="38" t="n">
+        <v>10</v>
+      </c>
+      <c r="C5" s="38" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="38" t="inlineStr">
+        <is>
+          <t>Card_T1</t>
+        </is>
+      </c>
+      <c r="B6" s="38" t="n">
+        <v>30</v>
+      </c>
+      <c r="C6" s="38" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="38" t="inlineStr">
+        <is>
+          <t>Card_T2</t>
+        </is>
+      </c>
+      <c r="B7" s="38" t="n">
+        <v>100</v>
+      </c>
+      <c r="C7" s="38" t="n">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="38" t="inlineStr">
+        <is>
+          <t>Card_T3</t>
+        </is>
+      </c>
+      <c r="B8" s="38" t="n">
+        <v>150</v>
+      </c>
+      <c r="C8" s="38" t="n">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="38" t="inlineStr">
+        <is>
+          <t>PrismCrystal</t>
+        </is>
+      </c>
+      <c r="B9" s="38" t="n">
+        <v>100</v>
+      </c>
+      <c r="C9" s="38" t="n">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="0" t="inlineStr">
+        <is>
+          <t>EncounterIndex</t>
+        </is>
+      </c>
+      <c r="B12" s="0" t="inlineStr">
+        <is>
+          <t>FreeTier</t>
+        </is>
+      </c>
+      <c r="C12" s="0" t="inlineStr">
+        <is>
+          <t>ShopTiers</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="38" t="n">
+        <v>1</v>
+      </c>
+      <c r="B13" s="40" t="n"/>
+      <c r="C13" s="40" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="38" t="n">
+        <v>2</v>
+      </c>
+      <c r="B14" s="38" t="n">
+        <v>2</v>
+      </c>
+      <c r="C14" s="38" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="38" t="n">
+        <v>3</v>
+      </c>
+      <c r="B15" s="38" t="n">
+        <v>3</v>
+      </c>
+      <c r="C15" s="38" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="38" t="n">
+        <v>4</v>
+      </c>
+      <c r="B16" s="38" t="n">
+        <v>1</v>
+      </c>
+      <c r="C16" s="38" t="inlineStr">
+        <is>
+          <t>2|3</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="38" t="n">
+        <v>5</v>
+      </c>
+      <c r="B17" s="38" t="n">
+        <v>2</v>
+      </c>
+      <c r="C17" s="40" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="38" t="n">
+        <v>6</v>
+      </c>
+      <c r="B18" s="38" t="n">
+        <v>3</v>
+      </c>
+      <c r="C18" s="38" t="inlineStr">
+        <is>
+          <t>1|2</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="38" t="n">
+        <v>7</v>
+      </c>
+      <c r="B19" s="38" t="n">
+        <v>2</v>
+      </c>
+      <c r="C19" s="38" t="inlineStr">
+        <is>
+          <t>1|3</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="38" t="n">
+        <v>8</v>
+      </c>
+      <c r="B20" s="40" t="n"/>
+      <c r="C20" s="40" t="n"/>
+    </row>
   </sheetData>
-  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="0" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="0" sort="0"/>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="0" insertHyperlinks="1" autoFilter="0" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="0" formatCells="1" formatRows="1" sort="0"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="2">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+  </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
[PROGRAMMER] Plan76: retire 连发枪口 in 开普勒 source + regenerate CSVs
Disable P_GUN_RAPID_MUZZLE (Enabled=false, ImplementationStatus=Disabled, ShopEnabled=false, ShopPrice=0, DisabledReason=策划确认不想要) in ReEchoData.xlsx 武器插槽C; sync regenerates parts.csv / part_effects.csv. Refresh prebuilt binaries from -FullRebuild.
</commit_message>
<xml_diff>
--- a/Design/Data/ReEchoData.xlsx
+++ b/Design/Data/ReEchoData.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="属性S" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="元素体系Y" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="构筑体系G" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="角色体系J" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="武器体系W" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="武器插槽C" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="怪物体系M" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="状态Z" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="经济系统" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_WorkbookMeta" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_ExportMap" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_SystemData" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AttributeCatalog" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="属性S" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="元素体系Y" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="构筑体系G" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="角色体系J" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="武器体系W" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="武器插槽C" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="怪物体系M" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="状态Z" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="经济系统" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="_WorkbookMeta" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="_ExportMap" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="_SystemData" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="AttributeCatalog" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames>
     <definedName name="DV_Logic_Elements_Id">'_SystemData'!$R$2:$R$5</definedName>
@@ -24488,7 +24488,7 @@
       </c>
       <c r="I86" s="37" t="inlineStr">
         <is>
-          <t>true</t>
+          <t>false</t>
         </is>
       </c>
       <c r="J86" s="37" t="inlineStr">
@@ -24498,10 +24498,14 @@
       </c>
       <c r="K86" s="37" t="inlineStr">
         <is>
-          <t>Implemented</t>
-        </is>
-      </c>
-      <c r="L86" s="37" t="n"/>
+          <t>Disabled</t>
+        </is>
+      </c>
+      <c r="L86" s="37" t="inlineStr">
+        <is>
+          <t>策划确认不想要</t>
+        </is>
+      </c>
       <c r="M86" s="37" t="inlineStr">
         <is>
           <t>武器插槽C</t>
@@ -24514,12 +24518,12 @@
       </c>
       <c r="O86" s="37" t="inlineStr">
         <is>
-          <t>true</t>
+          <t>false</t>
         </is>
       </c>
       <c r="P86" s="37" t="inlineStr">
         <is>
-          <t>30</t>
+          <t>0</t>
         </is>
       </c>
       <c r="R86" s="37" t="inlineStr">
@@ -24604,10 +24608,14 @@
       </c>
       <c r="AH86" s="37" t="inlineStr">
         <is>
-          <t>true</t>
-        </is>
-      </c>
-      <c r="AI86" s="37" t="n"/>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="AI86" s="37" t="inlineStr">
+        <is>
+          <t>策划确认不想要</t>
+        </is>
+      </c>
       <c r="AJ86" s="37" t="inlineStr">
         <is>
           <t>武器插槽C</t>
@@ -29568,10 +29576,14 @@
       </c>
       <c r="AH114" s="37" t="inlineStr">
         <is>
-          <t>true</t>
-        </is>
-      </c>
-      <c r="AI114" s="37" t="n"/>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="AI114" s="37" t="inlineStr">
+        <is>
+          <t>策划确认不想要</t>
+        </is>
+      </c>
       <c r="AJ114" s="37" t="inlineStr">
         <is>
           <t>武器插槽C</t>

</xml_diff>

<commit_message>
[PROGRAMMER] Implement card outcome tooltips and disable two runes
</commit_message>
<xml_diff>
--- a/Design/Data/ReEchoData.xlsx
+++ b/Design/Data/ReEchoData.xlsx
@@ -19464,15 +19464,17 @@
         <x:v>Grip|UniqueBehavior|ActiveAttack</x:v>
       </x:c>
       <x:c r="I71" s="78" t="str">
-        <x:v>true</x:v>
+        <x:v>false</x:v>
       </x:c>
       <x:c r="J71" s="78" t="str">
         <x:v>Approved</x:v>
       </x:c>
       <x:c r="K71" s="78" t="str">
-        <x:v>Implemented</x:v>
-      </x:c>
-      <x:c r="L71" s="78"/>
+        <x:v>Disabled</x:v>
+      </x:c>
+      <x:c r="L71" s="78" t="str">
+        <x:v>策划确认禁用</x:v>
+      </x:c>
       <x:c r="M71" s="78" t="str">
         <x:v>武器插槽C</x:v>
       </x:c>
@@ -19480,10 +19482,10 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="O71" s="78" t="str">
-        <x:v>true</x:v>
+        <x:v>false</x:v>
       </x:c>
       <x:c r="P71" s="78" t="str">
-        <x:v>45</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="R71" s="78" t="str">
         <x:v>PE_BOW_CRITBLEED_ARROWHEAD_1</x:v>
@@ -20210,15 +20212,17 @@
         <x:v>SwordBlade|UniqueBehavior|Meteor</x:v>
       </x:c>
       <x:c r="I78" s="78" t="str">
-        <x:v>true</x:v>
+        <x:v>false</x:v>
       </x:c>
       <x:c r="J78" s="78" t="str">
         <x:v>Approved</x:v>
       </x:c>
       <x:c r="K78" s="78" t="str">
-        <x:v>Implemented</x:v>
-      </x:c>
-      <x:c r="L78" s="78"/>
+        <x:v>Disabled</x:v>
+      </x:c>
+      <x:c r="L78" s="78" t="str">
+        <x:v>策划确认禁用</x:v>
+      </x:c>
       <x:c r="M78" s="78" t="str">
         <x:v>武器插槽C</x:v>
       </x:c>
@@ -20226,10 +20230,10 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="O78" s="78" t="str">
-        <x:v>true</x:v>
+        <x:v>false</x:v>
       </x:c>
       <x:c r="P78" s="78" t="str">
-        <x:v>45</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="R78" s="78" t="str">
         <x:v>PE_SCYTHE_LIFESTEAL_ROTARYBLADE_1</x:v>
@@ -21130,9 +21134,11 @@
         <x:v>Unique</x:v>
       </x:c>
       <x:c r="AH86" s="78" t="str">
-        <x:v>true</x:v>
-      </x:c>
-      <x:c r="AI86" s="78"/>
+        <x:v>false</x:v>
+      </x:c>
+      <x:c r="AI86" s="78" t="str">
+        <x:v>策划确认禁用</x:v>
+      </x:c>
       <x:c r="AJ86" s="78" t="str">
         <x:v>武器插槽C</x:v>
       </x:c>
@@ -21236,9 +21242,11 @@
         <x:v>Unique</x:v>
       </x:c>
       <x:c r="AH87" s="78" t="str">
-        <x:v>true</x:v>
-      </x:c>
-      <x:c r="AI87" s="78"/>
+        <x:v>false</x:v>
+      </x:c>
+      <x:c r="AI87" s="78" t="str">
+        <x:v>策划确认禁用</x:v>
+      </x:c>
       <x:c r="AJ87" s="78" t="str">
         <x:v>武器插槽C</x:v>
       </x:c>
@@ -21660,9 +21668,11 @@
         <x:v>Unique</x:v>
       </x:c>
       <x:c r="AH91" s="78" t="str">
-        <x:v>true</x:v>
-      </x:c>
-      <x:c r="AI91" s="78"/>
+        <x:v>false</x:v>
+      </x:c>
+      <x:c r="AI91" s="78" t="str">
+        <x:v>策划确认禁用</x:v>
+      </x:c>
       <x:c r="AJ91" s="78" t="str">
         <x:v>武器插槽C</x:v>
       </x:c>
@@ -21766,9 +21776,11 @@
         <x:v>Unique</x:v>
       </x:c>
       <x:c r="AH92" s="78" t="str">
-        <x:v>true</x:v>
-      </x:c>
-      <x:c r="AI92" s="78"/>
+        <x:v>false</x:v>
+      </x:c>
+      <x:c r="AI92" s="78" t="str">
+        <x:v>策划确认禁用</x:v>
+      </x:c>
       <x:c r="AJ92" s="78" t="str">
         <x:v>武器插槽C</x:v>
       </x:c>

</xml_diff>

<commit_message>
balance(cards): tune tier-one card values and descriptions
</commit_message>
<xml_diff>
--- a/Design/Data/ReEchoData.xlsx
+++ b/Design/Data/ReEchoData.xlsx
@@ -9063,7 +9063,7 @@
       </c>
       <c r="E4" s="33" t="inlineStr">
         <is>
-          <t>移动速度+8%</t>
+          <t>移动速度+6%</t>
         </is>
       </c>
       <c r="F4" s="29" t="inlineStr">
@@ -9140,7 +9140,7 @@
       </c>
       <c r="X4" s="29" t="inlineStr">
         <is>
-          <t>0.08</t>
+          <t>0.06</t>
         </is>
       </c>
       <c r="Y4" s="29" t="inlineStr">
@@ -9182,7 +9182,7 @@
       </c>
       <c r="E5" s="33" t="inlineStr">
         <is>
-          <t>生命值与生命上限+6</t>
+          <t>生命值与生命上限+5</t>
         </is>
       </c>
       <c r="F5" s="29" t="inlineStr">
@@ -9259,7 +9259,7 @@
       </c>
       <c r="X5" s="29" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="Y5" s="29" t="inlineStr">
@@ -9301,7 +9301,7 @@
       </c>
       <c r="E6" s="33" t="inlineStr">
         <is>
-          <t>物理攻击力+3</t>
+          <t>物理攻击力+2</t>
         </is>
       </c>
       <c r="F6" s="29" t="inlineStr">
@@ -9378,7 +9378,7 @@
       </c>
       <c r="X6" s="29" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="Y6" s="29" t="inlineStr">
@@ -9420,7 +9420,7 @@
       </c>
       <c r="E7" s="33" t="inlineStr">
         <is>
-          <t>元素攻击力+3</t>
+          <t>元素攻击力+2</t>
         </is>
       </c>
       <c r="F7" s="29" t="inlineStr">
@@ -9497,7 +9497,7 @@
       </c>
       <c r="X7" s="29" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="Y7" s="29" t="inlineStr">
@@ -9539,7 +9539,7 @@
       </c>
       <c r="E8" s="33" t="inlineStr">
         <is>
-          <t>暴击率+10%，暴击效果+25%</t>
+          <t>暴击率+7%，暴击效果+15%</t>
         </is>
       </c>
       <c r="F8" s="29" t="inlineStr">
@@ -9616,7 +9616,7 @@
       </c>
       <c r="X8" s="29" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="Y8" s="29" t="inlineStr">
@@ -9658,7 +9658,7 @@
       </c>
       <c r="E9" s="33" t="inlineStr">
         <is>
-          <t>元素反应效能+20%</t>
+          <t>元素反应效能+12%</t>
         </is>
       </c>
       <c r="F9" s="29" t="inlineStr">
@@ -9735,7 +9735,7 @@
       </c>
       <c r="X9" s="29" t="inlineStr">
         <is>
-          <t>0.1</t>
+          <t>0.07</t>
         </is>
       </c>
       <c r="Y9" s="29" t="inlineStr">
@@ -9777,7 +9777,7 @@
       </c>
       <c r="E10" s="33" t="inlineStr">
         <is>
-          <t>回响效能+8%</t>
+          <t>回响效能+6%</t>
         </is>
       </c>
       <c r="F10" s="29" t="inlineStr">
@@ -9854,7 +9854,7 @@
       </c>
       <c r="X10" s="29" t="inlineStr">
         <is>
-          <t>0.25</t>
+          <t>0.15</t>
         </is>
       </c>
       <c r="Y10" s="29" t="inlineStr">
@@ -9977,7 +9977,7 @@
       </c>
       <c r="X11" s="29" t="inlineStr">
         <is>
-          <t>0.2</t>
+          <t>0.12</t>
         </is>
       </c>
       <c r="Y11" s="29" t="inlineStr">
@@ -10096,7 +10096,7 @@
       </c>
       <c r="X12" s="29" t="inlineStr">
         <is>
-          <t>0.08</t>
+          <t>0.06</t>
         </is>
       </c>
       <c r="Y12" s="29" t="inlineStr">
@@ -21355,8 +21355,6 @@
       <c r="O10" s="24" t="n"/>
       <c r="P10" s="24" t="n"/>
     </row>
-    <row r="11"/>
-    <row r="12"/>
     <row r="13" ht="25" customHeight="1" s="41">
       <c r="A13" s="42" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
[PROGRAMMER] Reconcile card workbook with current production CSV
Preserve production CSV bytes and original workbook protection. Restore static registration consistency and regression fixtures. Publication is paused at the user's request; no main integration or push performed.
</commit_message>
<xml_diff>
--- a/Design/Data/ReEchoData.xlsx
+++ b/Design/Data/ReEchoData.xlsx
@@ -846,7 +846,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="tblCardEffects" displayName="tblCardEffects" ref="Q3:AA104" headerRowCount="1" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="tblCardEffects" displayName="tblCardEffects" ref="Q3:AA106" headerRowCount="1" totalsRowShown="0">
   <tableColumns count="11">
     <tableColumn id="1" name="Id"/>
     <tableColumn id="2" name="CardId"/>
@@ -8879,12 +8879,12 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA112"/>
+  <dimension ref="A1:AA114"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="13.81640625" defaultRowHeight="13"/>
   <cols>
     <col width="25" customWidth="1" style="41" min="1" max="2"/>
@@ -12042,7 +12042,7 @@
       </c>
       <c r="E29" s="33" t="inlineStr">
         <is>
-          <t>你的回响每击杀15名敌人，物攻&amp;元攻永久+1
+          <t xml:space="preserve">你的回响每击杀15名敌人，物攻&amp;元攻永久+1
 你每击杀15名敌人，回响效能永久+2%</t>
         </is>
       </c>
@@ -13114,7 +13114,7 @@
       </c>
       <c r="E38" s="33" t="inlineStr">
         <is>
-          <t>你获得1000时间碎片，随机承受：
+          <t xml:space="preserve">你获得1000时间碎片，随机承受：
 你将不能再刷新商店/你将不能再购买额外卡牌组/敌人将不再掉落时间碎片</t>
         </is>
       </c>
@@ -14428,7 +14428,7 @@
       </c>
       <c r="E49" s="33" t="inlineStr">
         <is>
-          <t>完成任一任务后，获得666时间碎片：
+          <t xml:space="preserve">完成任一任务后，获得666时间碎片：
 击杀111个敌人/结束战斗时≥22生命值/结束战斗时≤3生命值</t>
         </is>
       </c>
@@ -15381,7 +15381,7 @@
       </c>
       <c r="E57" s="33" t="inlineStr">
         <is>
-          <t>你可以在商店赊账，欠款会收取10%利息/每关
+          <t xml:space="preserve">你可以在商店赊账，欠款会收取10%利息/每关
 第8关时，如果你还没有还清，会有很不好的事情发生！！</t>
         </is>
       </c>
@@ -16810,7 +16810,7 @@
       </c>
       <c r="E69" s="39" t="inlineStr">
         <is>
-          <t>每关结束后，你的时间碎片随机+200%或-50%；然后获得50时间碎片
+          <t xml:space="preserve">每关结束后，赌一把大的！攒够了家底以后，商店刷新永远为你开放！
 ——策划 爆培嘉 敬上</t>
         </is>
       </c>
@@ -16930,7 +16930,7 @@
       </c>
       <c r="E70" s="39" t="inlineStr">
         <is>
-          <t>随机获得任意数量项效果：1、暴击率+50%；2、物理攻击力+15；3、生命值调整为5
+          <t xml:space="preserve">选择后，你可能拥有至高无上的暴击数值，也可能从此一蹶不振！
 ——策划 斑 敬上</t>
         </is>
       </c>
@@ -17050,7 +17050,7 @@
       </c>
       <c r="E71" s="39" t="inlineStr">
         <is>
-          <t>回响触碰到敌方单位，会对其造成15物理伤害；触碰到你，转而回复10生命值。
+          <t xml:space="preserve">回响触碰到敌人，造成20物理伤害；如果是你，你回复10生命值。数值每关翻倍！
 ——策划 麦麦熊 敬上</t>
         </is>
       </c>
@@ -17170,7 +17170,7 @@
       </c>
       <c r="E72" s="39" t="inlineStr">
         <is>
-          <t>失去所有时间碎片。每失去15时间碎片，随机获得一些属性！
+          <t xml:space="preserve">失去所有时间碎片。每失去15时间碎片，随机获得一些属性！
 ——策划 呕乐兮 敬上</t>
         </is>
       </c>
@@ -17290,7 +17290,7 @@
       </c>
       <c r="E73" s="39" t="inlineStr">
         <is>
-          <t>每0.5秒，令身边4m内的随机1名敌人【眩晕】至本关结束
+          <t xml:space="preserve">身边的敌人都被你迷倒了！
 ——特别鸣谢 程序 T爷</t>
         </is>
       </c>
@@ -17410,7 +17410,7 @@
       </c>
       <c r="E74" s="39" t="inlineStr">
         <is>
-          <t>你累计承受55伤害后，随机获得5张卡牌
+          <t xml:space="preserve">你努力奔跑。下一关，1滴血换1张1级卡牌
 ——特别鸣谢 程序 Jo爷</t>
         </is>
       </c>
@@ -17530,7 +17530,7 @@
       </c>
       <c r="E75" s="39" t="inlineStr">
         <is>
-          <t>造成的所有物理伤害，随机被修正为可能带有很多0的数字！
+          <t xml:space="preserve">神秘人往你的物理伤害后面加随机个0
 ——特别鸣谢 美术 00</t>
         </is>
       </c>
@@ -17650,7 +17650,7 @@
       </c>
       <c r="E76" s="39" t="inlineStr">
         <is>
-          <t>你的时间碎片获取方式，被赋予“ELO”机制
+          <t xml:space="preserve">经济系统被赋予“ELO”机制
 ——特别鸣谢 美术 子涵</t>
         </is>
       </c>
@@ -17770,7 +17770,7 @@
       </c>
       <c r="E77" s="39" t="inlineStr">
         <is>
-          <t>每一关卡结束后，获得15生命值&amp;2元攻&amp;2物攻
+          <t xml:space="preserve">每一关卡结束后，随机获得巨额生命值/元攻/物攻
 ——特别鸣谢 美术 雯雯</t>
         </is>
       </c>
@@ -18017,7 +18017,7 @@
       <c r="K80" s="43" t="n"/>
       <c r="Q80" s="29" t="inlineStr">
         <is>
-          <t>G_4_1_SWING_BONUS</t>
+          <t xml:space="preserve">G_4_1_REFRESH</t>
         </is>
       </c>
       <c r="R80" s="29" t="inlineStr">
@@ -18042,33 +18042,29 @@
       </c>
       <c r="V80" s="29" t="inlineStr">
         <is>
-          <t>TimeShards</t>
+          <t xml:space="preserve">FreeShopRefresh</t>
         </is>
       </c>
       <c r="W80" s="29" t="inlineStr">
         <is>
-          <t>Add</t>
-        </is>
-      </c>
-      <c r="X80" s="29" t="inlineStr">
-        <is>
-          <t>50</t>
-        </is>
+          <t xml:space="preserve">Override</t>
+        </is>
+      </c>
+      <c r="X80" s="29" t="n">
+        <v>2000</v>
       </c>
       <c r="Y80" s="29" t="inlineStr">
         <is>
-          <t>Card.EasterShardSwing</t>
+          <t xml:space="preserve">Card.EasterShardThreshold</t>
         </is>
       </c>
       <c r="Z80" s="29" t="inlineStr">
         <is>
-          <t>Bonus</t>
-        </is>
-      </c>
-      <c r="AA80" s="29" t="inlineStr">
-        <is>
-          <t>50</t>
-        </is>
+          <t xml:space="preserve">Threshold</t>
+        </is>
+      </c>
+      <c r="AA80" s="29" t="n">
+        <v>2000</v>
       </c>
     </row>
     <row r="81" ht="22" customHeight="1" s="41">
@@ -18118,10 +18114,8 @@
           <t>Add</t>
         </is>
       </c>
-      <c r="X81" s="29" t="inlineStr">
-        <is>
-          <t>0.5</t>
-        </is>
+      <c r="X81" s="29" t="n">
+        <v>1</v>
       </c>
       <c r="Y81" s="29" t="inlineStr">
         <is>
@@ -18153,7 +18147,7 @@
       <c r="K82" s="43" t="n"/>
       <c r="Q82" s="29" t="inlineStr">
         <is>
-          <t>G_4_2_PHYSICAL</t>
+          <t xml:space="preserve">G_4_2_CRIT_EFFECT</t>
         </is>
       </c>
       <c r="R82" s="29" t="inlineStr">
@@ -18178,7 +18172,7 @@
       </c>
       <c r="V82" s="29" t="inlineStr">
         <is>
-          <t>PhysicalAttack</t>
+          <t xml:space="preserve">CriticalEffect</t>
         </is>
       </c>
       <c r="W82" s="29" t="inlineStr">
@@ -18186,10 +18180,8 @@
           <t>Add</t>
         </is>
       </c>
-      <c r="X82" s="29" t="inlineStr">
-        <is>
-          <t>15</t>
-        </is>
+      <c r="X82" s="29" t="n">
+        <v>3</v>
       </c>
       <c r="Y82" s="29" t="inlineStr">
         <is>
@@ -18293,22 +18285,20 @@
       <c r="K84" s="43" t="n"/>
       <c r="Q84" s="29" t="inlineStr">
         <is>
-          <t>G_4_3_CONTACT_DAMAGE</t>
+          <t xml:space="preserve">G_4_2_CRIT_PENALTY</t>
         </is>
       </c>
       <c r="R84" s="29" t="inlineStr">
         <is>
-          <t>G_4_3</t>
-        </is>
-      </c>
-      <c r="S84" s="29" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+          <t xml:space="preserve">G_4_2</t>
+        </is>
+      </c>
+      <c r="S84" s="29" t="n">
+        <v>4</v>
       </c>
       <c r="T84" s="29" t="inlineStr">
         <is>
-          <t>OnCompileRules</t>
+          <t xml:space="preserve">OnGrant</t>
         </is>
       </c>
       <c r="U84" s="29" t="inlineStr">
@@ -18318,33 +18308,29 @@
       </c>
       <c r="V84" s="29" t="inlineStr">
         <is>
-          <t>Damage</t>
+          <t xml:space="preserve">CritNegateAmplification</t>
         </is>
       </c>
       <c r="W84" s="29" t="inlineStr">
         <is>
-          <t>Add</t>
-        </is>
-      </c>
-      <c r="X84" s="29" t="inlineStr">
-        <is>
-          <t>15</t>
-        </is>
+          <t xml:space="preserve">Override</t>
+        </is>
+      </c>
+      <c r="X84" s="29" t="n">
+        <v>1</v>
       </c>
       <c r="Y84" s="29" t="inlineStr">
         <is>
-          <t>Card.EasterEchoContact</t>
+          <t xml:space="preserve">Card.EasterIndependentGrant</t>
         </is>
       </c>
       <c r="Z84" s="29" t="inlineStr">
         <is>
-          <t>PlayerHealing</t>
-        </is>
-      </c>
-      <c r="AA84" s="29" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+          <t xml:space="preserve">Chance</t>
+        </is>
+      </c>
+      <c r="AA84" s="29" t="n">
+        <v>0.5</v>
       </c>
     </row>
     <row r="85" ht="22" customHeight="1" s="41">
@@ -18361,12 +18347,12 @@
       <c r="K85" s="43" t="n"/>
       <c r="Q85" s="29" t="inlineStr">
         <is>
-          <t>G_4_4_HP</t>
+          <t xml:space="preserve">G_4_3_CONTACT_DAMAGE</t>
         </is>
       </c>
       <c r="R85" s="29" t="inlineStr">
         <is>
-          <t>G_4_4</t>
+          <t xml:space="preserve">G_4_3</t>
         </is>
       </c>
       <c r="S85" s="29" t="inlineStr">
@@ -18376,7 +18362,7 @@
       </c>
       <c r="T85" s="29" t="inlineStr">
         <is>
-          <t>OnGrant</t>
+          <t xml:space="preserve">OnCompileRules</t>
         </is>
       </c>
       <c r="U85" s="29" t="inlineStr">
@@ -18386,7 +18372,7 @@
       </c>
       <c r="V85" s="29" t="inlineStr">
         <is>
-          <t>HpMaxAndPoint</t>
+          <t xml:space="preserve">Damage</t>
         </is>
       </c>
       <c r="W85" s="29" t="inlineStr">
@@ -18394,25 +18380,21 @@
           <t>Add</t>
         </is>
       </c>
-      <c r="X85" s="29" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="X85" s="29" t="n">
+        <v>20</v>
       </c>
       <c r="Y85" s="29" t="inlineStr">
         <is>
-          <t>Card.EasterShardSacrifice</t>
+          <t xml:space="preserve">Card.EasterEchoContact</t>
         </is>
       </c>
       <c r="Z85" s="29" t="inlineStr">
         <is>
-          <t>ShardUnit</t>
-        </is>
-      </c>
-      <c r="AA85" s="29" t="inlineStr">
-        <is>
-          <t>15</t>
-        </is>
+          <t xml:space="preserve">PlayerHealing</t>
+        </is>
+      </c>
+      <c r="AA85" s="29" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="86" ht="22" customHeight="1" s="41">
@@ -18429,7 +18411,7 @@
       <c r="K86" s="43" t="n"/>
       <c r="Q86" s="39" t="inlineStr">
         <is>
-          <t>G_4_4_PHYSICAL</t>
+          <t xml:space="preserve">G_4_4_HP</t>
         </is>
       </c>
       <c r="R86" s="39" t="inlineStr">
@@ -18437,10 +18419,8 @@
           <t>G_4_4</t>
         </is>
       </c>
-      <c r="S86" s="39" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="S86" s="39" t="n">
+        <v>1</v>
       </c>
       <c r="T86" s="39" t="inlineStr">
         <is>
@@ -18454,7 +18434,7 @@
       </c>
       <c r="V86" s="39" t="inlineStr">
         <is>
-          <t>PhysicalAttack</t>
+          <t xml:space="preserve">HpMaxAndPoint</t>
         </is>
       </c>
       <c r="W86" s="39" t="inlineStr">
@@ -18497,7 +18477,7 @@
       <c r="K87" s="43" t="n"/>
       <c r="Q87" s="39" t="inlineStr">
         <is>
-          <t>G_4_4_ELEMENTAL</t>
+          <t xml:space="preserve">G_4_4_PHYSICAL</t>
         </is>
       </c>
       <c r="R87" s="39" t="inlineStr">
@@ -18505,10 +18485,8 @@
           <t>G_4_4</t>
         </is>
       </c>
-      <c r="S87" s="39" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="S87" s="39" t="n">
+        <v>2</v>
       </c>
       <c r="T87" s="39" t="inlineStr">
         <is>
@@ -18522,7 +18500,7 @@
       </c>
       <c r="V87" s="39" t="inlineStr">
         <is>
-          <t>ElementalAttack</t>
+          <t xml:space="preserve">PhysicalAttack</t>
         </is>
       </c>
       <c r="W87" s="39" t="inlineStr">
@@ -18565,7 +18543,7 @@
       <c r="K88" s="43" t="n"/>
       <c r="Q88" s="39" t="inlineStr">
         <is>
-          <t>G_4_4_CRIT_RATE</t>
+          <t xml:space="preserve">G_4_4_ELEMENTAL</t>
         </is>
       </c>
       <c r="R88" s="39" t="inlineStr">
@@ -18573,10 +18551,8 @@
           <t>G_4_4</t>
         </is>
       </c>
-      <c r="S88" s="39" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
+      <c r="S88" s="39" t="n">
+        <v>3</v>
       </c>
       <c r="T88" s="39" t="inlineStr">
         <is>
@@ -18590,7 +18566,7 @@
       </c>
       <c r="V88" s="39" t="inlineStr">
         <is>
-          <t>CriticalRate</t>
+          <t xml:space="preserve">ElementalAttack</t>
         </is>
       </c>
       <c r="W88" s="39" t="inlineStr">
@@ -18598,10 +18574,8 @@
           <t>Add</t>
         </is>
       </c>
-      <c r="X88" s="39" t="inlineStr">
-        <is>
-          <t>0.05</t>
-        </is>
+      <c r="X88" s="39" t="n">
+        <v>1</v>
       </c>
       <c r="Y88" s="39" t="inlineStr">
         <is>
@@ -18633,7 +18607,7 @@
       <c r="K89" s="43" t="n"/>
       <c r="Q89" s="39" t="inlineStr">
         <is>
-          <t>G_4_4_CRIT_EFFECT</t>
+          <t xml:space="preserve">G_4_4_CRIT_RATE</t>
         </is>
       </c>
       <c r="R89" s="39" t="inlineStr">
@@ -18641,10 +18615,8 @@
           <t>G_4_4</t>
         </is>
       </c>
-      <c r="S89" s="39" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
+      <c r="S89" s="39" t="n">
+        <v>4</v>
       </c>
       <c r="T89" s="39" t="inlineStr">
         <is>
@@ -18658,7 +18630,7 @@
       </c>
       <c r="V89" s="39" t="inlineStr">
         <is>
-          <t>CriticalEffect</t>
+          <t xml:space="preserve">CriticalRate</t>
         </is>
       </c>
       <c r="W89" s="39" t="inlineStr">
@@ -18666,10 +18638,8 @@
           <t>Add</t>
         </is>
       </c>
-      <c r="X89" s="39" t="inlineStr">
-        <is>
-          <t>0.1</t>
-        </is>
+      <c r="X89" s="39" t="n">
+        <v>0.05</v>
       </c>
       <c r="Y89" s="39" t="inlineStr">
         <is>
@@ -18701,7 +18671,7 @@
       <c r="K90" s="43" t="n"/>
       <c r="Q90" s="39" t="inlineStr">
         <is>
-          <t>G_4_4_ECHO</t>
+          <t xml:space="preserve">G_4_4_CRIT_EFFECT</t>
         </is>
       </c>
       <c r="R90" s="39" t="inlineStr">
@@ -18709,10 +18679,8 @@
           <t>G_4_4</t>
         </is>
       </c>
-      <c r="S90" s="39" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
+      <c r="S90" s="39" t="n">
+        <v>5</v>
       </c>
       <c r="T90" s="39" t="inlineStr">
         <is>
@@ -18726,7 +18694,7 @@
       </c>
       <c r="V90" s="39" t="inlineStr">
         <is>
-          <t>EchoEfficiency</t>
+          <t xml:space="preserve">CriticalEffect</t>
         </is>
       </c>
       <c r="W90" s="39" t="inlineStr">
@@ -18734,10 +18702,8 @@
           <t>Add</t>
         </is>
       </c>
-      <c r="X90" s="39" t="inlineStr">
-        <is>
-          <t>0.05</t>
-        </is>
+      <c r="X90" s="39" t="n">
+        <v>0.1</v>
       </c>
       <c r="Y90" s="39" t="inlineStr">
         <is>
@@ -18769,7 +18735,7 @@
       <c r="K91" s="43" t="n"/>
       <c r="Q91" s="39" t="inlineStr">
         <is>
-          <t>G_4_4_REACTION</t>
+          <t xml:space="preserve">G_4_4_ECHO</t>
         </is>
       </c>
       <c r="R91" s="39" t="inlineStr">
@@ -18777,10 +18743,8 @@
           <t>G_4_4</t>
         </is>
       </c>
-      <c r="S91" s="39" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
+      <c r="S91" s="39" t="n">
+        <v>6</v>
       </c>
       <c r="T91" s="39" t="inlineStr">
         <is>
@@ -18794,7 +18758,7 @@
       </c>
       <c r="V91" s="39" t="inlineStr">
         <is>
-          <t>ReactionEfficiency</t>
+          <t xml:space="preserve">EchoEfficiency</t>
         </is>
       </c>
       <c r="W91" s="39" t="inlineStr">
@@ -18837,22 +18801,20 @@
       <c r="K92" s="43" t="n"/>
       <c r="Q92" s="39" t="inlineStr">
         <is>
-          <t>G_4_5_STUN</t>
+          <t xml:space="preserve">G_4_4_REACTION</t>
         </is>
       </c>
       <c r="R92" s="39" t="inlineStr">
         <is>
-          <t>G_4_5</t>
-        </is>
-      </c>
-      <c r="S92" s="39" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+          <t xml:space="preserve">G_4_4</t>
+        </is>
+      </c>
+      <c r="S92" s="39" t="n">
+        <v>7</v>
       </c>
       <c r="T92" s="39" t="inlineStr">
         <is>
-          <t>OnEncounterTick</t>
+          <t xml:space="preserve">OnGrant</t>
         </is>
       </c>
       <c r="U92" s="39" t="inlineStr">
@@ -18862,33 +18824,29 @@
       </c>
       <c r="V92" s="39" t="inlineStr">
         <is>
-          <t>Stun</t>
+          <t xml:space="preserve">ReactionEfficiency</t>
         </is>
       </c>
       <c r="W92" s="39" t="inlineStr">
         <is>
-          <t>Override</t>
-        </is>
-      </c>
-      <c r="X92" s="39" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+          <t xml:space="preserve">Add</t>
+        </is>
+      </c>
+      <c r="X92" s="39" t="n">
+        <v>0.05</v>
       </c>
       <c r="Y92" s="39" t="inlineStr">
         <is>
-          <t>Card.EasterRandomStun</t>
+          <t xml:space="preserve">Card.EasterShardSacrifice</t>
         </is>
       </c>
       <c r="Z92" s="39" t="inlineStr">
         <is>
-          <t>PulseInterval</t>
-        </is>
-      </c>
-      <c r="AA92" s="39" t="inlineStr">
-        <is>
-          <t>0.5</t>
-        </is>
+          <t xml:space="preserve">ShardUnit</t>
+        </is>
+      </c>
+      <c r="AA92" s="39" t="n">
+        <v>15</v>
       </c>
     </row>
     <row r="93" ht="22" customHeight="1" s="41">
@@ -18905,7 +18863,7 @@
       <c r="K93" s="43" t="n"/>
       <c r="Q93" s="39" t="inlineStr">
         <is>
-          <t>G_4_5_RADIUS</t>
+          <t xml:space="preserve">G_4_5_STUN</t>
         </is>
       </c>
       <c r="R93" s="39" t="inlineStr">
@@ -18913,10 +18871,8 @@
           <t>G_4_5</t>
         </is>
       </c>
-      <c r="S93" s="39" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="S93" s="39" t="n">
+        <v>1</v>
       </c>
       <c r="T93" s="39" t="inlineStr">
         <is>
@@ -18930,7 +18886,7 @@
       </c>
       <c r="V93" s="39" t="inlineStr">
         <is>
-          <t>Damage</t>
+          <t xml:space="preserve">Stun</t>
         </is>
       </c>
       <c r="W93" s="39" t="inlineStr">
@@ -18938,10 +18894,8 @@
           <t>Override</t>
         </is>
       </c>
-      <c r="X93" s="39" t="inlineStr">
-        <is>
-          <t>400</t>
-        </is>
+      <c r="X93" s="39" t="n">
+        <v>1</v>
       </c>
       <c r="Y93" s="39" t="inlineStr">
         <is>
@@ -18950,13 +18904,11 @@
       </c>
       <c r="Z93" s="39" t="inlineStr">
         <is>
-          <t>RadiusCm</t>
-        </is>
-      </c>
-      <c r="AA93" s="39" t="inlineStr">
-        <is>
-          <t>400</t>
-        </is>
+          <t xml:space="preserve">PulseInterval</t>
+        </is>
+      </c>
+      <c r="AA93" s="39" t="n">
+        <v>0.5</v>
       </c>
     </row>
     <row r="94" ht="22" customHeight="1" s="41">
@@ -18973,22 +18925,20 @@
       <c r="K94" s="43" t="n"/>
       <c r="Q94" s="39" t="inlineStr">
         <is>
-          <t>G_4_6_THRESHOLD</t>
+          <t xml:space="preserve">G_4_5_RADIUS</t>
         </is>
       </c>
       <c r="R94" s="39" t="inlineStr">
         <is>
-          <t>G_4_6</t>
-        </is>
-      </c>
-      <c r="S94" s="39" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+          <t xml:space="preserve">G_4_5</t>
+        </is>
+      </c>
+      <c r="S94" s="39" t="n">
+        <v>2</v>
       </c>
       <c r="T94" s="39" t="inlineStr">
         <is>
-          <t>OnDamageResolved</t>
+          <t xml:space="preserve">OnEncounterTick</t>
         </is>
       </c>
       <c r="U94" s="39" t="inlineStr">
@@ -19003,28 +18953,24 @@
       </c>
       <c r="W94" s="39" t="inlineStr">
         <is>
-          <t>Add</t>
-        </is>
-      </c>
-      <c r="X94" s="39" t="inlineStr">
-        <is>
-          <t>55</t>
-        </is>
+          <t xml:space="preserve">Override</t>
+        </is>
+      </c>
+      <c r="X94" s="39" t="n">
+        <v>500</v>
       </c>
       <c r="Y94" s="39" t="inlineStr">
         <is>
-          <t>Card.EasterDamageCards</t>
+          <t xml:space="preserve">Card.EasterRandomStun</t>
         </is>
       </c>
       <c r="Z94" s="39" t="inlineStr">
         <is>
-          <t>GrantCount</t>
-        </is>
-      </c>
-      <c r="AA94" s="39" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
+          <t xml:space="preserve">RadiusCm</t>
+        </is>
+      </c>
+      <c r="AA94" s="39" t="n">
+        <v>500</v>
       </c>
     </row>
     <row r="95" ht="22" customHeight="1" s="41">
@@ -19041,22 +18987,20 @@
       <c r="K95" s="43" t="n"/>
       <c r="Q95" s="39" t="inlineStr">
         <is>
-          <t>G_4_7_ZERO</t>
+          <t xml:space="preserve">G_4_5_COUNT</t>
         </is>
       </c>
       <c r="R95" s="39" t="inlineStr">
         <is>
-          <t>G_4_7</t>
-        </is>
-      </c>
-      <c r="S95" s="39" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+          <t xml:space="preserve">G_4_5</t>
+        </is>
+      </c>
+      <c r="S95" s="39" t="n">
+        <v>3</v>
       </c>
       <c r="T95" s="39" t="inlineStr">
         <is>
-          <t>BeforeOutgoingHit</t>
+          <t xml:space="preserve">OnEncounterTick</t>
         </is>
       </c>
       <c r="U95" s="39" t="inlineStr">
@@ -19066,7 +19010,7 @@
       </c>
       <c r="V95" s="39" t="inlineStr">
         <is>
-          <t>Damage</t>
+          <t xml:space="preserve">Stun</t>
         </is>
       </c>
       <c r="W95" s="39" t="inlineStr">
@@ -19074,25 +19018,21 @@
           <t>Override</t>
         </is>
       </c>
-      <c r="X95" s="39" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="X95" s="39" t="n">
+        <v>5</v>
       </c>
       <c r="Y95" s="39" t="inlineStr">
         <is>
-          <t>Card.EasterPhysicalLottery</t>
+          <t xml:space="preserve">Card.EasterRandomStun</t>
         </is>
       </c>
       <c r="Z95" s="39" t="inlineStr">
         <is>
-          <t>Probability</t>
-        </is>
-      </c>
-      <c r="AA95" s="39" t="inlineStr">
-        <is>
-          <t>0.15</t>
-        </is>
+          <t xml:space="preserve">TargetCount</t>
+        </is>
+      </c>
+      <c r="AA95" s="39" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="96" ht="22" customHeight="1" s="41">
@@ -19109,22 +19049,20 @@
       <c r="K96" s="43" t="n"/>
       <c r="Q96" s="39" t="inlineStr">
         <is>
-          <t>G_4_7_TEN</t>
+          <t xml:space="preserve">G_4_6_REWARD</t>
         </is>
       </c>
       <c r="R96" s="39" t="inlineStr">
         <is>
-          <t>G_4_7</t>
-        </is>
-      </c>
-      <c r="S96" s="39" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+          <t xml:space="preserve">G_4_6</t>
+        </is>
+      </c>
+      <c r="S96" s="39" t="n">
+        <v>1</v>
       </c>
       <c r="T96" s="39" t="inlineStr">
         <is>
-          <t>BeforeOutgoingHit</t>
+          <t xml:space="preserve">OnEncounterEnd</t>
         </is>
       </c>
       <c r="U96" s="39" t="inlineStr">
@@ -19134,7 +19072,7 @@
       </c>
       <c r="V96" s="39" t="inlineStr">
         <is>
-          <t>Damage</t>
+          <t xml:space="preserve">MinimumGuaranteedTier</t>
         </is>
       </c>
       <c r="W96" s="39" t="inlineStr">
@@ -19142,25 +19080,21 @@
           <t>Override</t>
         </is>
       </c>
-      <c r="X96" s="39" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
+      <c r="X96" s="39" t="n">
+        <v>1</v>
       </c>
       <c r="Y96" s="39" t="inlineStr">
         <is>
-          <t>Card.EasterPhysicalLottery</t>
+          <t xml:space="preserve">Card.EasterDamageCards</t>
         </is>
       </c>
       <c r="Z96" s="39" t="inlineStr">
         <is>
-          <t>Probability</t>
-        </is>
-      </c>
-      <c r="AA96" s="39" t="inlineStr">
-        <is>
-          <t>0.35</t>
-        </is>
+          <t xml:space="preserve">GrantTier</t>
+        </is>
+      </c>
+      <c r="AA96" s="39" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="97" ht="22" customHeight="1" s="41">
@@ -19177,7 +19111,7 @@
       <c r="K97" s="43" t="n"/>
       <c r="Q97" s="39" t="inlineStr">
         <is>
-          <t>G_4_7_HUNDRED</t>
+          <t xml:space="preserve">G_4_7_ZERO</t>
         </is>
       </c>
       <c r="R97" s="39" t="inlineStr">
@@ -19185,10 +19119,8 @@
           <t>G_4_7</t>
         </is>
       </c>
-      <c r="S97" s="39" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="S97" s="39" t="n">
+        <v>1</v>
       </c>
       <c r="T97" s="39" t="inlineStr">
         <is>
@@ -19210,10 +19142,8 @@
           <t>Override</t>
         </is>
       </c>
-      <c r="X97" s="39" t="inlineStr">
-        <is>
-          <t>100</t>
-        </is>
+      <c r="X97" s="39" t="n">
+        <v>0</v>
       </c>
       <c r="Y97" s="39" t="inlineStr">
         <is>
@@ -19225,10 +19155,8 @@
           <t>Probability</t>
         </is>
       </c>
-      <c r="AA97" s="39" t="inlineStr">
-        <is>
-          <t>0.4</t>
-        </is>
+      <c r="AA97" s="39" t="n">
+        <v>0.15</v>
       </c>
     </row>
     <row r="98" ht="22" customHeight="1" s="41">
@@ -19245,7 +19173,7 @@
       <c r="K98" s="43" t="n"/>
       <c r="Q98" s="39" t="inlineStr">
         <is>
-          <t>G_4_7_THOUSAND</t>
+          <t xml:space="preserve">G_4_7_TEN</t>
         </is>
       </c>
       <c r="R98" s="39" t="inlineStr">
@@ -19253,10 +19181,8 @@
           <t>G_4_7</t>
         </is>
       </c>
-      <c r="S98" s="39" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
+      <c r="S98" s="39" t="n">
+        <v>2</v>
       </c>
       <c r="T98" s="39" t="inlineStr">
         <is>
@@ -19278,10 +19204,8 @@
           <t>Override</t>
         </is>
       </c>
-      <c r="X98" s="39" t="inlineStr">
-        <is>
-          <t>1000</t>
-        </is>
+      <c r="X98" s="39" t="n">
+        <v>10</v>
       </c>
       <c r="Y98" s="39" t="inlineStr">
         <is>
@@ -19293,10 +19217,8 @@
           <t>Probability</t>
         </is>
       </c>
-      <c r="AA98" s="39" t="inlineStr">
-        <is>
-          <t>0.08</t>
-        </is>
+      <c r="AA98" s="39" t="n">
+        <v>0.35</v>
       </c>
     </row>
     <row r="99" ht="22" customHeight="1" s="41">
@@ -19313,7 +19235,7 @@
       <c r="K99" s="43" t="n"/>
       <c r="Q99" s="39" t="inlineStr">
         <is>
-          <t>G_4_7_TEN_THOUSAND</t>
+          <t xml:space="preserve">G_4_7_HUNDRED</t>
         </is>
       </c>
       <c r="R99" s="39" t="inlineStr">
@@ -19321,10 +19243,8 @@
           <t>G_4_7</t>
         </is>
       </c>
-      <c r="S99" s="39" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
+      <c r="S99" s="39" t="n">
+        <v>3</v>
       </c>
       <c r="T99" s="39" t="inlineStr">
         <is>
@@ -19346,10 +19266,8 @@
           <t>Override</t>
         </is>
       </c>
-      <c r="X99" s="39" t="inlineStr">
-        <is>
-          <t>10000</t>
-        </is>
+      <c r="X99" s="39" t="n">
+        <v>100</v>
       </c>
       <c r="Y99" s="39" t="inlineStr">
         <is>
@@ -19361,10 +19279,8 @@
           <t>Probability</t>
         </is>
       </c>
-      <c r="AA99" s="39" t="inlineStr">
-        <is>
-          <t>0.02</t>
-        </is>
+      <c r="AA99" s="39" t="n">
+        <v>0.4</v>
       </c>
     </row>
     <row r="100" ht="22" customHeight="1" s="41">
@@ -19381,22 +19297,20 @@
       <c r="K100" s="43" t="n"/>
       <c r="Q100" s="39" t="inlineStr">
         <is>
-          <t>G_4_8_MORE</t>
+          <t xml:space="preserve">G_4_7_THOUSAND</t>
         </is>
       </c>
       <c r="R100" s="39" t="inlineStr">
         <is>
-          <t>G_4_8</t>
-        </is>
-      </c>
-      <c r="S100" s="39" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+          <t xml:space="preserve">G_4_7</t>
+        </is>
+      </c>
+      <c r="S100" s="39" t="n">
+        <v>4</v>
       </c>
       <c r="T100" s="39" t="inlineStr">
         <is>
-          <t>OnEncounterEnd</t>
+          <t xml:space="preserve">BeforeOutgoingHit</t>
         </is>
       </c>
       <c r="U100" s="39" t="inlineStr">
@@ -19406,33 +19320,29 @@
       </c>
       <c r="V100" s="39" t="inlineStr">
         <is>
-          <t>TimeShards</t>
+          <t xml:space="preserve">Damage</t>
         </is>
       </c>
       <c r="W100" s="39" t="inlineStr">
         <is>
-          <t>Multiply</t>
-        </is>
-      </c>
-      <c r="X100" s="39" t="inlineStr">
-        <is>
-          <t>-0.01</t>
-        </is>
+          <t xml:space="preserve">Override</t>
+        </is>
+      </c>
+      <c r="X100" s="39" t="n">
+        <v>1000</v>
       </c>
       <c r="Y100" s="39" t="inlineStr">
         <is>
-          <t>Card.EasterShardComparison</t>
+          <t xml:space="preserve">Card.EasterPhysicalLottery</t>
         </is>
       </c>
       <c r="Z100" s="39" t="inlineStr">
         <is>
-          <t>Step</t>
-        </is>
-      </c>
-      <c r="AA100" s="39" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
+          <t xml:space="preserve">Probability</t>
+        </is>
+      </c>
+      <c r="AA100" s="39" t="n">
+        <v>0.09</v>
       </c>
     </row>
     <row r="101" ht="22" customHeight="1" s="41">
@@ -19449,22 +19359,20 @@
       <c r="K101" s="43" t="n"/>
       <c r="Q101" s="39" t="inlineStr">
         <is>
-          <t>G_4_8_LESS</t>
+          <t xml:space="preserve">G_4_7_TEN_THOUSAND</t>
         </is>
       </c>
       <c r="R101" s="39" t="inlineStr">
         <is>
-          <t>G_4_8</t>
-        </is>
-      </c>
-      <c r="S101" s="39" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+          <t xml:space="preserve">G_4_7</t>
+        </is>
+      </c>
+      <c r="S101" s="39" t="n">
+        <v>5</v>
       </c>
       <c r="T101" s="39" t="inlineStr">
         <is>
-          <t>OnEncounterEnd</t>
+          <t xml:space="preserve">BeforeOutgoingHit</t>
         </is>
       </c>
       <c r="U101" s="39" t="inlineStr">
@@ -19474,33 +19382,29 @@
       </c>
       <c r="V101" s="39" t="inlineStr">
         <is>
-          <t>TimeShards</t>
+          <t xml:space="preserve">Damage</t>
         </is>
       </c>
       <c r="W101" s="39" t="inlineStr">
         <is>
-          <t>Multiply</t>
-        </is>
-      </c>
-      <c r="X101" s="39" t="inlineStr">
-        <is>
-          <t>0.05</t>
-        </is>
+          <t xml:space="preserve">Override</t>
+        </is>
+      </c>
+      <c r="X101" s="39" t="n">
+        <v>10000</v>
       </c>
       <c r="Y101" s="39" t="inlineStr">
         <is>
-          <t>Card.EasterShardComparison</t>
+          <t xml:space="preserve">Card.EasterPhysicalLottery</t>
         </is>
       </c>
       <c r="Z101" s="39" t="inlineStr">
         <is>
-          <t>Step</t>
-        </is>
-      </c>
-      <c r="AA101" s="39" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
+          <t xml:space="preserve">Probability</t>
+        </is>
+      </c>
+      <c r="AA101" s="39" t="n">
+        <v>0.01</v>
       </c>
     </row>
     <row r="102" ht="22" customHeight="1" s="41">
@@ -19517,12 +19421,12 @@
       <c r="K102" s="43" t="n"/>
       <c r="Q102" s="39" t="inlineStr">
         <is>
-          <t>G_4_9_HP</t>
+          <t xml:space="preserve">G_4_8_MORE</t>
         </is>
       </c>
       <c r="R102" s="39" t="inlineStr">
         <is>
-          <t>G_4_9</t>
+          <t xml:space="preserve">G_4_8</t>
         </is>
       </c>
       <c r="S102" s="39" t="inlineStr">
@@ -19542,33 +19446,29 @@
       </c>
       <c r="V102" s="39" t="inlineStr">
         <is>
-          <t>HpMaxAndPoint</t>
+          <t xml:space="preserve">TimeShards</t>
         </is>
       </c>
       <c r="W102" s="39" t="inlineStr">
         <is>
-          <t>Add</t>
-        </is>
-      </c>
-      <c r="X102" s="39" t="inlineStr">
-        <is>
-          <t>15</t>
-        </is>
+          <t xml:space="preserve">Multiply</t>
+        </is>
+      </c>
+      <c r="X102" s="39" t="n">
+        <v>-0.01</v>
       </c>
       <c r="Y102" s="39" t="inlineStr">
         <is>
-          <t>Card.EasterAttendance</t>
+          <t xml:space="preserve">Card.EasterShardComparison</t>
         </is>
       </c>
       <c r="Z102" s="39" t="inlineStr">
         <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="AA102" s="39" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+          <t xml:space="preserve">Step</t>
+        </is>
+      </c>
+      <c r="AA102" s="39" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="103" ht="26" customHeight="1" s="41">
@@ -19585,12 +19485,12 @@
       <c r="K103" s="43" t="n"/>
       <c r="Q103" s="39" t="inlineStr">
         <is>
-          <t>G_4_9_ELEMENTAL</t>
+          <t xml:space="preserve">G_4_8_LESS</t>
         </is>
       </c>
       <c r="R103" s="39" t="inlineStr">
         <is>
-          <t>G_4_9</t>
+          <t xml:space="preserve">G_4_8</t>
         </is>
       </c>
       <c r="S103" s="39" t="inlineStr">
@@ -19610,39 +19510,35 @@
       </c>
       <c r="V103" s="39" t="inlineStr">
         <is>
-          <t>ElementalAttack</t>
+          <t xml:space="preserve">TimeShards</t>
         </is>
       </c>
       <c r="W103" s="39" t="inlineStr">
         <is>
-          <t>Add</t>
-        </is>
-      </c>
-      <c r="X103" s="39" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+          <t xml:space="preserve">Multiply</t>
+        </is>
+      </c>
+      <c r="X103" s="39" t="n">
+        <v>0.05</v>
       </c>
       <c r="Y103" s="39" t="inlineStr">
         <is>
-          <t>Card.EasterAttendance</t>
+          <t xml:space="preserve">Card.EasterShardComparison</t>
         </is>
       </c>
       <c r="Z103" s="39" t="inlineStr">
         <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="AA103" s="39" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+          <t xml:space="preserve">Step</t>
+        </is>
+      </c>
+      <c r="AA103" s="39" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="104" ht="26" customHeight="1" s="41">
       <c r="Q104" s="39" t="inlineStr">
         <is>
-          <t>G_4_9_PHYSICAL</t>
+          <t xml:space="preserve">G_4_9_HP</t>
         </is>
       </c>
       <c r="R104" s="39" t="inlineStr">
@@ -19650,10 +19546,8 @@
           <t>G_4_9</t>
         </is>
       </c>
-      <c r="S104" s="39" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="S104" s="39" t="n">
+        <v>1</v>
       </c>
       <c r="T104" s="39" t="inlineStr">
         <is>
@@ -19667,7 +19561,7 @@
       </c>
       <c r="V104" s="39" t="inlineStr">
         <is>
-          <t>PhysicalAttack</t>
+          <t xml:space="preserve">HpMaxAndPoint</t>
         </is>
       </c>
       <c r="W104" s="39" t="inlineStr">
@@ -19675,10 +19569,8 @@
           <t>Add</t>
         </is>
       </c>
-      <c r="X104" s="39" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="X104" s="39" t="n">
+        <v>1</v>
       </c>
       <c r="Y104" s="39" t="inlineStr">
         <is>
@@ -19687,121 +19579,119 @@
       </c>
       <c r="Z104" s="39" t="inlineStr">
         <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="AA104" s="39" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+          <t xml:space="preserve">Max</t>
+        </is>
+      </c>
+      <c r="AA104" s="39" t="n">
+        <v>20</v>
       </c>
     </row>
     <row r="105" ht="26" customHeight="1" s="41">
-      <c r="Q105" s="46" t="inlineStr">
-        <is>
-          <t>G_4_7_HUNDRED</t>
-        </is>
-      </c>
-      <c r="R105" s="46" t="inlineStr">
-        <is>
-          <t>G_4_7</t>
-        </is>
-      </c>
-      <c r="S105" s="46" t="n">
+      <c r="Q105" s="39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">G_4_9_ELEMENTAL</t>
+        </is>
+      </c>
+      <c r="R105" s="39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">G_4_9</t>
+        </is>
+      </c>
+      <c r="S105" s="39" t="n">
+        <v>2</v>
+      </c>
+      <c r="T105" s="39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">OnEncounterEnd</t>
+        </is>
+      </c>
+      <c r="U105" s="39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CardBehavior</t>
+        </is>
+      </c>
+      <c r="V105" s="39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ElementalAttack</t>
+        </is>
+      </c>
+      <c r="W105" s="39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Add</t>
+        </is>
+      </c>
+      <c r="X105" s="39" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y105" s="39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Card.EasterAttendance</t>
+        </is>
+      </c>
+      <c r="Z105" s="39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Max</t>
+        </is>
+      </c>
+      <c r="AA105" s="39" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="106" ht="26" customHeight="1" s="41">
+      <c r="Q106" s="39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">G_4_9_PHYSICAL</t>
+        </is>
+      </c>
+      <c r="R106" s="39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">G_4_9</t>
+        </is>
+      </c>
+      <c r="S106" s="39" t="n">
         <v>3</v>
       </c>
-      <c r="T105" s="46" t="inlineStr">
-        <is>
-          <t>BeforeOutgoingHit</t>
-        </is>
-      </c>
-      <c r="U105" s="46" t="inlineStr">
-        <is>
-          <t>CardBehavior</t>
-        </is>
-      </c>
-      <c r="V105" s="46" t="inlineStr">
-        <is>
-          <t>Damage</t>
-        </is>
-      </c>
-      <c r="W105" s="46" t="inlineStr">
-        <is>
-          <t>Override</t>
-        </is>
-      </c>
-      <c r="X105" s="46" t="n">
-        <v>100</v>
-      </c>
-      <c r="Y105" s="46" t="inlineStr">
-        <is>
-          <t>Card.EasterPhysicalLottery</t>
-        </is>
-      </c>
-      <c r="Z105" s="46" t="inlineStr">
-        <is>
-          <t>Probability</t>
-        </is>
-      </c>
-      <c r="AA105" s="46" t="n">
-        <v>0.4</v>
-      </c>
-    </row>
-    <row r="106" ht="26" customHeight="1" s="41">
-      <c r="Q106" s="46" t="inlineStr">
-        <is>
-          <t>G_4_7_THOUSAND</t>
-        </is>
-      </c>
-      <c r="R106" s="46" t="inlineStr">
-        <is>
-          <t>G_4_7</t>
-        </is>
-      </c>
-      <c r="S106" s="46" t="n">
-        <v>4</v>
-      </c>
-      <c r="T106" s="46" t="inlineStr">
-        <is>
-          <t>BeforeOutgoingHit</t>
-        </is>
-      </c>
-      <c r="U106" s="46" t="inlineStr">
-        <is>
-          <t>CardBehavior</t>
-        </is>
-      </c>
-      <c r="V106" s="46" t="inlineStr">
-        <is>
-          <t>Damage</t>
-        </is>
-      </c>
-      <c r="W106" s="46" t="inlineStr">
-        <is>
-          <t>Override</t>
-        </is>
-      </c>
-      <c r="X106" s="46" t="n">
-        <v>1000</v>
-      </c>
-      <c r="Y106" s="46" t="inlineStr">
-        <is>
-          <t>Card.EasterPhysicalLottery</t>
-        </is>
-      </c>
-      <c r="Z106" s="46" t="inlineStr">
-        <is>
-          <t>Probability</t>
-        </is>
-      </c>
-      <c r="AA106" s="46" t="n">
-        <v>0.08</v>
+      <c r="T106" s="39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">OnEncounterEnd</t>
+        </is>
+      </c>
+      <c r="U106" s="39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CardBehavior</t>
+        </is>
+      </c>
+      <c r="V106" s="39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PhysicalAttack</t>
+        </is>
+      </c>
+      <c r="W106" s="39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Add</t>
+        </is>
+      </c>
+      <c r="X106" s="39" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y106" s="39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Card.EasterAttendance</t>
+        </is>
+      </c>
+      <c r="Z106" s="39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Max</t>
+        </is>
+      </c>
+      <c r="AA106" s="39" t="n">
+        <v>20</v>
       </c>
     </row>
     <row r="107" ht="26" customHeight="1" s="41">
       <c r="Q107" s="46" t="inlineStr">
         <is>
-          <t>G_4_7_TEN_THOUSAND</t>
+          <t>G_4_7_HUNDRED</t>
         </is>
       </c>
       <c r="R107" s="46" t="inlineStr">
@@ -19810,7 +19700,7 @@
         </is>
       </c>
       <c r="S107" s="46" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="T107" s="46" t="inlineStr">
         <is>
@@ -19833,7 +19723,7 @@
         </is>
       </c>
       <c r="X107" s="46" t="n">
-        <v>10000</v>
+        <v>100</v>
       </c>
       <c r="Y107" s="46" t="inlineStr">
         <is>
@@ -19846,26 +19736,26 @@
         </is>
       </c>
       <c r="AA107" s="46" t="n">
-        <v>0.02</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="108" ht="26" customHeight="1" s="41">
       <c r="Q108" s="46" t="inlineStr">
         <is>
-          <t>G_4_8_MORE</t>
+          <t>G_4_7_THOUSAND</t>
         </is>
       </c>
       <c r="R108" s="46" t="inlineStr">
         <is>
-          <t>G_4_8</t>
+          <t>G_4_7</t>
         </is>
       </c>
       <c r="S108" s="46" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="T108" s="46" t="inlineStr">
         <is>
-          <t>OnEncounterEnd</t>
+          <t>BeforeOutgoingHit</t>
         </is>
       </c>
       <c r="U108" s="46" t="inlineStr">
@@ -19875,48 +19765,48 @@
       </c>
       <c r="V108" s="46" t="inlineStr">
         <is>
-          <t>TimeShards</t>
+          <t>Damage</t>
         </is>
       </c>
       <c r="W108" s="46" t="inlineStr">
         <is>
-          <t>Multiply</t>
+          <t>Override</t>
         </is>
       </c>
       <c r="X108" s="46" t="n">
-        <v>-0.01</v>
+        <v>1000</v>
       </c>
       <c r="Y108" s="46" t="inlineStr">
         <is>
-          <t>Card.EasterShardComparison</t>
+          <t>Card.EasterPhysicalLottery</t>
         </is>
       </c>
       <c r="Z108" s="46" t="inlineStr">
         <is>
-          <t>Step</t>
+          <t>Probability</t>
         </is>
       </c>
       <c r="AA108" s="46" t="n">
-        <v>5</v>
+        <v>0.08</v>
       </c>
     </row>
     <row r="109" ht="26" customHeight="1" s="41">
       <c r="Q109" s="46" t="inlineStr">
         <is>
-          <t>G_4_8_LESS</t>
+          <t>G_4_7_TEN_THOUSAND</t>
         </is>
       </c>
       <c r="R109" s="46" t="inlineStr">
         <is>
-          <t>G_4_8</t>
+          <t>G_4_7</t>
         </is>
       </c>
       <c r="S109" s="46" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="T109" s="46" t="inlineStr">
         <is>
-          <t>OnEncounterEnd</t>
+          <t>BeforeOutgoingHit</t>
         </is>
       </c>
       <c r="U109" s="46" t="inlineStr">
@@ -19926,40 +19816,40 @@
       </c>
       <c r="V109" s="46" t="inlineStr">
         <is>
-          <t>TimeShards</t>
+          <t>Damage</t>
         </is>
       </c>
       <c r="W109" s="46" t="inlineStr">
         <is>
-          <t>Multiply</t>
+          <t>Override</t>
         </is>
       </c>
       <c r="X109" s="46" t="n">
-        <v>0.05</v>
+        <v>10000</v>
       </c>
       <c r="Y109" s="46" t="inlineStr">
         <is>
-          <t>Card.EasterShardComparison</t>
+          <t>Card.EasterPhysicalLottery</t>
         </is>
       </c>
       <c r="Z109" s="46" t="inlineStr">
         <is>
-          <t>Step</t>
+          <t>Probability</t>
         </is>
       </c>
       <c r="AA109" s="46" t="n">
-        <v>5</v>
+        <v>0.02</v>
       </c>
     </row>
     <row r="110" ht="26" customHeight="1" s="41">
       <c r="Q110" s="46" t="inlineStr">
         <is>
-          <t>G_4_9_HP</t>
+          <t>G_4_8_MORE</t>
         </is>
       </c>
       <c r="R110" s="46" t="inlineStr">
         <is>
-          <t>G_4_9</t>
+          <t>G_4_8</t>
         </is>
       </c>
       <c r="S110" s="46" t="n">
@@ -19977,40 +19867,40 @@
       </c>
       <c r="V110" s="46" t="inlineStr">
         <is>
-          <t>HpMaxAndPoint</t>
+          <t>TimeShards</t>
         </is>
       </c>
       <c r="W110" s="46" t="inlineStr">
         <is>
-          <t>Add</t>
+          <t>Multiply</t>
         </is>
       </c>
       <c r="X110" s="46" t="n">
-        <v>10</v>
+        <v>-0.01</v>
       </c>
       <c r="Y110" s="46" t="inlineStr">
         <is>
-          <t>Card.EasterAttendance</t>
+          <t>Card.EasterShardComparison</t>
         </is>
       </c>
       <c r="Z110" s="46" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Step</t>
         </is>
       </c>
       <c r="AA110" s="46" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="111" ht="26" customHeight="1" s="41">
       <c r="Q111" s="46" t="inlineStr">
         <is>
-          <t>G_4_9_ELEMENTAL</t>
+          <t>G_4_8_LESS</t>
         </is>
       </c>
       <c r="R111" s="46" t="inlineStr">
         <is>
-          <t>G_4_9</t>
+          <t>G_4_8</t>
         </is>
       </c>
       <c r="S111" s="46" t="n">
@@ -20028,79 +19918,181 @@
       </c>
       <c r="V111" s="46" t="inlineStr">
         <is>
-          <t>ElementalAttack</t>
+          <t>TimeShards</t>
         </is>
       </c>
       <c r="W111" s="46" t="inlineStr">
         <is>
-          <t>Add</t>
+          <t>Multiply</t>
         </is>
       </c>
       <c r="X111" s="46" t="n">
-        <v>1</v>
+        <v>0.05</v>
       </c>
       <c r="Y111" s="46" t="inlineStr">
         <is>
-          <t>Card.EasterAttendance</t>
+          <t>Card.EasterShardComparison</t>
         </is>
       </c>
       <c r="Z111" s="46" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Step</t>
         </is>
       </c>
       <c r="AA111" s="46" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="112" ht="26" customHeight="1" s="41">
       <c r="Q112" s="46" t="inlineStr">
         <is>
+          <t>G_4_9_HP</t>
+        </is>
+      </c>
+      <c r="R112" s="46" t="inlineStr">
+        <is>
+          <t>G_4_9</t>
+        </is>
+      </c>
+      <c r="S112" s="46" t="n">
+        <v>1</v>
+      </c>
+      <c r="T112" s="46" t="inlineStr">
+        <is>
+          <t>OnEncounterEnd</t>
+        </is>
+      </c>
+      <c r="U112" s="46" t="inlineStr">
+        <is>
+          <t>CardBehavior</t>
+        </is>
+      </c>
+      <c r="V112" s="46" t="inlineStr">
+        <is>
+          <t>HpMaxAndPoint</t>
+        </is>
+      </c>
+      <c r="W112" s="46" t="inlineStr">
+        <is>
+          <t>Add</t>
+        </is>
+      </c>
+      <c r="X112" s="46" t="n">
+        <v>10</v>
+      </c>
+      <c r="Y112" s="46" t="inlineStr">
+        <is>
+          <t>Card.EasterAttendance</t>
+        </is>
+      </c>
+      <c r="Z112" s="46" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="AA112" s="46" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="Q113" s="46" t="inlineStr">
+        <is>
+          <t>G_4_9_ELEMENTAL</t>
+        </is>
+      </c>
+      <c r="R113" s="46" t="inlineStr">
+        <is>
+          <t>G_4_9</t>
+        </is>
+      </c>
+      <c r="S113" s="46" t="n">
+        <v>2</v>
+      </c>
+      <c r="T113" s="46" t="inlineStr">
+        <is>
+          <t>OnEncounterEnd</t>
+        </is>
+      </c>
+      <c r="U113" s="46" t="inlineStr">
+        <is>
+          <t>CardBehavior</t>
+        </is>
+      </c>
+      <c r="V113" s="46" t="inlineStr">
+        <is>
+          <t>ElementalAttack</t>
+        </is>
+      </c>
+      <c r="W113" s="46" t="inlineStr">
+        <is>
+          <t>Add</t>
+        </is>
+      </c>
+      <c r="X113" s="46" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y113" s="46" t="inlineStr">
+        <is>
+          <t>Card.EasterAttendance</t>
+        </is>
+      </c>
+      <c r="Z113" s="46" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="AA113" s="46" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="Q114" s="46" t="inlineStr">
+        <is>
           <t>G_4_9_PHYSICAL</t>
         </is>
       </c>
-      <c r="R112" s="46" t="inlineStr">
+      <c r="R114" s="46" t="inlineStr">
         <is>
           <t>G_4_9</t>
         </is>
       </c>
-      <c r="S112" s="46" t="n">
+      <c r="S114" s="46" t="n">
         <v>3</v>
       </c>
-      <c r="T112" s="46" t="inlineStr">
+      <c r="T114" s="46" t="inlineStr">
         <is>
           <t>OnEncounterEnd</t>
         </is>
       </c>
-      <c r="U112" s="46" t="inlineStr">
+      <c r="U114" s="46" t="inlineStr">
         <is>
           <t>CardBehavior</t>
         </is>
       </c>
-      <c r="V112" s="46" t="inlineStr">
+      <c r="V114" s="46" t="inlineStr">
         <is>
           <t>PhysicalAttack</t>
         </is>
       </c>
-      <c r="W112" s="46" t="inlineStr">
+      <c r="W114" s="46" t="inlineStr">
         <is>
           <t>Add</t>
         </is>
       </c>
-      <c r="X112" s="46" t="n">
-        <v>1</v>
-      </c>
-      <c r="Y112" s="46" t="inlineStr">
+      <c r="X114" s="46" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y114" s="46" t="inlineStr">
         <is>
           <t>Card.EasterAttendance</t>
         </is>
       </c>
-      <c r="Z112" s="46" t="inlineStr">
+      <c r="Z114" s="46" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="AA112" s="46" t="n">
+      <c r="AA114" s="46" t="n">
         <v>0</v>
       </c>
     </row>
@@ -20138,32 +20130,32 @@
     <dataValidation sqref="H4:H77" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Trait,Disabled"</formula1>
     </dataValidation>
-    <dataValidation sqref="R4:R104" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" errorTitle="无效选项" error="只能从下拉列表中选择有效值。" promptTitle="请选择" prompt="请从下拉列表选择，不能输入列表外的值。" type="list">
+    <dataValidation sqref="R4:R106" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" errorTitle="无效选项" error="只能从下拉列表中选择有效值。" promptTitle="请选择" prompt="请从下拉列表选择，不能输入列表外的值。" type="list">
       <formula1>INDIRECT("tblCards[Id]")</formula1>
     </dataValidation>
-    <dataValidation sqref="T4:T104" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" errorTitle="无效选项" error="只能从下拉列表中选择有效值。" promptTitle="请选择" prompt="请从下拉列表选择，不能输入列表外的值。" type="list">
+    <dataValidation sqref="T4:T106" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" errorTitle="无效选项" error="只能从下拉列表中选择有效值。" promptTitle="请选择" prompt="请从下拉列表选择，不能输入列表外的值。" type="list">
       <formula1>DV_Logic_CardEffects_Trigger</formula1>
     </dataValidation>
-    <dataValidation sqref="U4:U104" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" errorTitle="无效选项" error="只能从下拉列表中选择有效值。" promptTitle="请选择" prompt="请从下拉列表选择，不能输入列表外的值。" type="list">
+    <dataValidation sqref="U4:U106" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" errorTitle="无效选项" error="只能从下拉列表中选择有效值。" promptTitle="请选择" prompt="请从下拉列表选择，不能输入列表外的值。" type="list">
       <formula1>DV_Logic_CardEffects_EffectKind</formula1>
     </dataValidation>
-    <dataValidation sqref="V4:V104" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" errorTitle="无效选项" error="只能从下拉列表中选择有效值。" promptTitle="请选择" prompt="请从下拉列表选择，不能输入列表外的值。" type="list">
+    <dataValidation sqref="V4:V106" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" errorTitle="无效选项" error="只能从下拉列表中选择有效值。" promptTitle="请选择" prompt="请从下拉列表选择，不能输入列表外的值。" type="list">
       <formula1>DV_Logic_CardEffects_Target</formula1>
     </dataValidation>
-    <dataValidation sqref="W4:W104" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" errorTitle="无效选项" error="只能从下拉列表中选择有效值。" promptTitle="请选择" prompt="请从下拉列表选择，不能输入列表外的值。" type="list">
+    <dataValidation sqref="W4:W106" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" errorTitle="无效选项" error="只能从下拉列表中选择有效值。" promptTitle="请选择" prompt="请从下拉列表选择，不能输入列表外的值。" type="list">
       <formula1>DV_Logic_CardEffects_ValueOp</formula1>
     </dataValidation>
-    <dataValidation sqref="Y4:Y104" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" errorTitle="无效选项" error="只能从下拉列表中选择有效值。" promptTitle="请选择" prompt="请从下拉列表选择，不能输入列表外的值。" type="list">
+    <dataValidation sqref="Y4:Y106" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" errorTitle="无效选项" error="只能从下拉列表中选择有效值。" promptTitle="请选择" prompt="请从下拉列表选择，不能输入列表外的值。" type="list">
       <formula1>DV_Logic_CardEffects_BehaviorId</formula1>
     </dataValidation>
-    <dataValidation sqref="Z4:Z104" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" errorTitle="无效选项" error="只能从下拉列表中选择有效值。" promptTitle="请选择" prompt="请从下拉列表选择，不能输入列表外的值。" type="list">
+    <dataValidation sqref="Z4:Z106" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" errorTitle="无效选项" error="只能从下拉列表中选择有效值。" promptTitle="请选择" prompt="请从下拉列表选择，不能输入列表外的值。" type="list">
       <formula1>DV_Logic_CardEffects_ParamName</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="2">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
[PROGRAMMER] fix easter level and sauce card
</commit_message>
<xml_diff>
--- a/Design/Data/ReEchoData.xlsx
+++ b/Design/Data/ReEchoData.xlsx
@@ -8879,7 +8879,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
@@ -9063,7 +9063,7 @@
       </c>
       <c r="E4" s="33" t="inlineStr">
         <is>
-          <t>移动速度+6%</t>
+          <t>绉诲姩閫熷害+1%</t>
         </is>
       </c>
       <c r="F4" s="29" t="inlineStr">
@@ -9140,7 +9140,7 @@
       </c>
       <c r="X4" s="29" t="inlineStr">
         <is>
-          <t>0.06</t>
+          <t>0.01</t>
         </is>
       </c>
       <c r="Y4" s="29" t="inlineStr">
@@ -12042,7 +12042,7 @@
       </c>
       <c r="E29" s="33" t="inlineStr">
         <is>
-          <t xml:space="preserve">你的回响每击杀15名敌人，物攻&amp;元攻永久+1
+          <t>你的回响每击杀15名敌人，物攻&amp;元攻永久+1
 你每击杀15名敌人，回响效能永久+2%</t>
         </is>
       </c>
@@ -13114,7 +13114,7 @@
       </c>
       <c r="E38" s="33" t="inlineStr">
         <is>
-          <t xml:space="preserve">你获得1000时间碎片，随机承受：
+          <t>你获得1000时间碎片，随机承受：
 你将不能再刷新商店/你将不能再购买额外卡牌组/敌人将不再掉落时间碎片</t>
         </is>
       </c>
@@ -14428,7 +14428,7 @@
       </c>
       <c r="E49" s="33" t="inlineStr">
         <is>
-          <t xml:space="preserve">完成任一任务后，获得666时间碎片：
+          <t>完成任一任务后，获得666时间碎片：
 击杀111个敌人/结束战斗时≥22生命值/结束战斗时≤3生命值</t>
         </is>
       </c>
@@ -15381,7 +15381,7 @@
       </c>
       <c r="E57" s="33" t="inlineStr">
         <is>
-          <t xml:space="preserve">你可以在商店赊账，欠款会收取10%利息/每关
+          <t>你可以在商店赊账，欠款会收取10%利息/每关
 第8关时，如果你还没有还清，会有很不好的事情发生！！</t>
         </is>
       </c>
@@ -16810,7 +16810,7 @@
       </c>
       <c r="E69" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">每关结束后，赌一把大的！攒够了家底以后，商店刷新永远为你开放！
+          <t>每关结束后，赌一把大的！攒够了家底以后，商店刷新永远为你开放！
 ——策划 爆培嘉 敬上</t>
         </is>
       </c>
@@ -16930,7 +16930,7 @@
       </c>
       <c r="E70" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">选择后，你可能拥有至高无上的暴击数值，也可能从此一蹶不振！
+          <t>选择后，你可能拥有至高无上的暴击数值，也可能从此一蹶不振！
 ——策划 斑 敬上</t>
         </is>
       </c>
@@ -17050,7 +17050,7 @@
       </c>
       <c r="E71" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">回响触碰到敌人，造成20物理伤害；如果是你，你回复10生命值。数值每关翻倍！
+          <t>回响触碰到敌人，造成20物理伤害；如果是你，你回复10生命值。数值每关翻倍！
 ——策划 麦麦熊 敬上</t>
         </is>
       </c>
@@ -17170,7 +17170,7 @@
       </c>
       <c r="E72" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">失去所有时间碎片。每失去15时间碎片，随机获得一些属性！
+          <t>失去所有时间碎片。每失去15时间碎片，随机获得一些属性！
 ——策划 呕乐兮 敬上</t>
         </is>
       </c>
@@ -17290,7 +17290,7 @@
       </c>
       <c r="E73" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">身边的敌人都被你迷倒了！
+          <t>身边的敌人都被你迷倒了！
 ——特别鸣谢 程序 T爷</t>
         </is>
       </c>
@@ -17410,7 +17410,7 @@
       </c>
       <c r="E74" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">你努力奔跑。下一关，1滴血换1张1级卡牌
+          <t>你努力奔跑。下一关，1滴血换1张1级卡牌
 ——特别鸣谢 程序 Jo爷</t>
         </is>
       </c>
@@ -17530,7 +17530,7 @@
       </c>
       <c r="E75" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">神秘人往你的物理伤害后面加随机个0
+          <t>神秘人往你的物理伤害后面加随机个0
 ——特别鸣谢 美术 00</t>
         </is>
       </c>
@@ -17650,7 +17650,7 @@
       </c>
       <c r="E76" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">经济系统被赋予“ELO”机制
+          <t>经济系统被赋予“ELO”机制
 ——特别鸣谢 美术 子涵</t>
         </is>
       </c>
@@ -17770,7 +17770,7 @@
       </c>
       <c r="E77" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">每一关卡结束后，随机获得巨额生命值/元攻/物攻
+          <t>每一关卡结束后，随机获得巨额生命值/元攻/物攻
 ——特别鸣谢 美术 雯雯</t>
         </is>
       </c>
@@ -17888,8 +17888,8 @@
       </c>
       <c r="E78" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">选择后，攻击力永久增加5。
-策划：为什么表现是这样的？
+          <t>选择后，攻击力永久增加5。
+策划：为什么表现是这样的？
 程序：单子上是这么写的，符合预期</t>
         </is>
       </c>
@@ -18068,7 +18068,7 @@
       <c r="K80" s="43" t="n"/>
       <c r="Q80" s="29" t="inlineStr">
         <is>
-          <t xml:space="preserve">G_4_1_REFRESH</t>
+          <t>G_4_1_REFRESH</t>
         </is>
       </c>
       <c r="R80" s="29" t="inlineStr">
@@ -18093,12 +18093,12 @@
       </c>
       <c r="V80" s="29" t="inlineStr">
         <is>
-          <t xml:space="preserve">FreeShopRefresh</t>
+          <t>FreeShopRefresh</t>
         </is>
       </c>
       <c r="W80" s="29" t="inlineStr">
         <is>
-          <t xml:space="preserve">Override</t>
+          <t>Override</t>
         </is>
       </c>
       <c r="X80" s="29" t="n">
@@ -18106,12 +18106,12 @@
       </c>
       <c r="Y80" s="29" t="inlineStr">
         <is>
-          <t xml:space="preserve">Card.EasterShardThreshold</t>
+          <t>Card.EasterShardThreshold</t>
         </is>
       </c>
       <c r="Z80" s="29" t="inlineStr">
         <is>
-          <t xml:space="preserve">Threshold</t>
+          <t>Threshold</t>
         </is>
       </c>
       <c r="AA80" s="29" t="n">
@@ -18198,7 +18198,7 @@
       <c r="K82" s="43" t="n"/>
       <c r="Q82" s="29" t="inlineStr">
         <is>
-          <t xml:space="preserve">G_4_2_CRIT_EFFECT</t>
+          <t>G_4_2_CRIT_EFFECT</t>
         </is>
       </c>
       <c r="R82" s="29" t="inlineStr">
@@ -18223,7 +18223,7 @@
       </c>
       <c r="V82" s="29" t="inlineStr">
         <is>
-          <t xml:space="preserve">CriticalEffect</t>
+          <t>CriticalEffect</t>
         </is>
       </c>
       <c r="W82" s="29" t="inlineStr">
@@ -18336,12 +18336,12 @@
       <c r="K84" s="43" t="n"/>
       <c r="Q84" s="29" t="inlineStr">
         <is>
-          <t xml:space="preserve">G_4_2_CRIT_PENALTY</t>
+          <t>G_4_2_CRIT_PENALTY</t>
         </is>
       </c>
       <c r="R84" s="29" t="inlineStr">
         <is>
-          <t xml:space="preserve">G_4_2</t>
+          <t>G_4_2</t>
         </is>
       </c>
       <c r="S84" s="29" t="n">
@@ -18349,7 +18349,7 @@
       </c>
       <c r="T84" s="29" t="inlineStr">
         <is>
-          <t xml:space="preserve">OnGrant</t>
+          <t>OnGrant</t>
         </is>
       </c>
       <c r="U84" s="29" t="inlineStr">
@@ -18359,12 +18359,12 @@
       </c>
       <c r="V84" s="29" t="inlineStr">
         <is>
-          <t xml:space="preserve">CritNegateAmplification</t>
+          <t>CritNegateAmplification</t>
         </is>
       </c>
       <c r="W84" s="29" t="inlineStr">
         <is>
-          <t xml:space="preserve">Override</t>
+          <t>Override</t>
         </is>
       </c>
       <c r="X84" s="29" t="n">
@@ -18372,12 +18372,12 @@
       </c>
       <c r="Y84" s="29" t="inlineStr">
         <is>
-          <t xml:space="preserve">Card.EasterIndependentGrant</t>
+          <t>Card.EasterIndependentGrant</t>
         </is>
       </c>
       <c r="Z84" s="29" t="inlineStr">
         <is>
-          <t xml:space="preserve">Chance</t>
+          <t>Chance</t>
         </is>
       </c>
       <c r="AA84" s="29" t="n">
@@ -18398,12 +18398,12 @@
       <c r="K85" s="43" t="n"/>
       <c r="Q85" s="29" t="inlineStr">
         <is>
-          <t xml:space="preserve">G_4_3_CONTACT_DAMAGE</t>
+          <t>G_4_3_CONTACT_DAMAGE</t>
         </is>
       </c>
       <c r="R85" s="29" t="inlineStr">
         <is>
-          <t xml:space="preserve">G_4_3</t>
+          <t>G_4_3</t>
         </is>
       </c>
       <c r="S85" s="29" t="inlineStr">
@@ -18413,7 +18413,7 @@
       </c>
       <c r="T85" s="29" t="inlineStr">
         <is>
-          <t xml:space="preserve">OnCompileRules</t>
+          <t>OnCompileRules</t>
         </is>
       </c>
       <c r="U85" s="29" t="inlineStr">
@@ -18423,7 +18423,7 @@
       </c>
       <c r="V85" s="29" t="inlineStr">
         <is>
-          <t xml:space="preserve">Damage</t>
+          <t>Damage</t>
         </is>
       </c>
       <c r="W85" s="29" t="inlineStr">
@@ -18436,12 +18436,12 @@
       </c>
       <c r="Y85" s="29" t="inlineStr">
         <is>
-          <t xml:space="preserve">Card.EasterEchoContact</t>
+          <t>Card.EasterEchoContact</t>
         </is>
       </c>
       <c r="Z85" s="29" t="inlineStr">
         <is>
-          <t xml:space="preserve">PlayerHealing</t>
+          <t>PlayerHealing</t>
         </is>
       </c>
       <c r="AA85" s="29" t="n">
@@ -18462,7 +18462,7 @@
       <c r="K86" s="43" t="n"/>
       <c r="Q86" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">G_4_4_HP</t>
+          <t>G_4_4_HP</t>
         </is>
       </c>
       <c r="R86" s="39" t="inlineStr">
@@ -18485,7 +18485,7 @@
       </c>
       <c r="V86" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">HpMaxAndPoint</t>
+          <t>HpMaxAndPoint</t>
         </is>
       </c>
       <c r="W86" s="39" t="inlineStr">
@@ -18528,7 +18528,7 @@
       <c r="K87" s="43" t="n"/>
       <c r="Q87" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">G_4_4_PHYSICAL</t>
+          <t>G_4_4_PHYSICAL</t>
         </is>
       </c>
       <c r="R87" s="39" t="inlineStr">
@@ -18551,7 +18551,7 @@
       </c>
       <c r="V87" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">PhysicalAttack</t>
+          <t>PhysicalAttack</t>
         </is>
       </c>
       <c r="W87" s="39" t="inlineStr">
@@ -18594,7 +18594,7 @@
       <c r="K88" s="43" t="n"/>
       <c r="Q88" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">G_4_4_ELEMENTAL</t>
+          <t>G_4_4_ELEMENTAL</t>
         </is>
       </c>
       <c r="R88" s="39" t="inlineStr">
@@ -18617,7 +18617,7 @@
       </c>
       <c r="V88" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">ElementalAttack</t>
+          <t>ElementalAttack</t>
         </is>
       </c>
       <c r="W88" s="39" t="inlineStr">
@@ -18658,7 +18658,7 @@
       <c r="K89" s="43" t="n"/>
       <c r="Q89" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">G_4_4_CRIT_RATE</t>
+          <t>G_4_4_CRIT_RATE</t>
         </is>
       </c>
       <c r="R89" s="39" t="inlineStr">
@@ -18681,7 +18681,7 @@
       </c>
       <c r="V89" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">CriticalRate</t>
+          <t>CriticalRate</t>
         </is>
       </c>
       <c r="W89" s="39" t="inlineStr">
@@ -18722,7 +18722,7 @@
       <c r="K90" s="43" t="n"/>
       <c r="Q90" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">G_4_4_CRIT_EFFECT</t>
+          <t>G_4_4_CRIT_EFFECT</t>
         </is>
       </c>
       <c r="R90" s="39" t="inlineStr">
@@ -18745,7 +18745,7 @@
       </c>
       <c r="V90" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">CriticalEffect</t>
+          <t>CriticalEffect</t>
         </is>
       </c>
       <c r="W90" s="39" t="inlineStr">
@@ -18786,7 +18786,7 @@
       <c r="K91" s="43" t="n"/>
       <c r="Q91" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">G_4_4_ECHO</t>
+          <t>G_4_4_ECHO</t>
         </is>
       </c>
       <c r="R91" s="39" t="inlineStr">
@@ -18809,7 +18809,7 @@
       </c>
       <c r="V91" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">EchoEfficiency</t>
+          <t>EchoEfficiency</t>
         </is>
       </c>
       <c r="W91" s="39" t="inlineStr">
@@ -18852,12 +18852,12 @@
       <c r="K92" s="43" t="n"/>
       <c r="Q92" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">G_4_4_REACTION</t>
+          <t>G_4_4_REACTION</t>
         </is>
       </c>
       <c r="R92" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">G_4_4</t>
+          <t>G_4_4</t>
         </is>
       </c>
       <c r="S92" s="39" t="n">
@@ -18865,7 +18865,7 @@
       </c>
       <c r="T92" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">OnGrant</t>
+          <t>OnGrant</t>
         </is>
       </c>
       <c r="U92" s="39" t="inlineStr">
@@ -18875,12 +18875,12 @@
       </c>
       <c r="V92" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">ReactionEfficiency</t>
+          <t>ReactionEfficiency</t>
         </is>
       </c>
       <c r="W92" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Add</t>
+          <t>Add</t>
         </is>
       </c>
       <c r="X92" s="39" t="n">
@@ -18888,12 +18888,12 @@
       </c>
       <c r="Y92" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Card.EasterShardSacrifice</t>
+          <t>Card.EasterShardSacrifice</t>
         </is>
       </c>
       <c r="Z92" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">ShardUnit</t>
+          <t>ShardUnit</t>
         </is>
       </c>
       <c r="AA92" s="39" t="n">
@@ -18914,7 +18914,7 @@
       <c r="K93" s="43" t="n"/>
       <c r="Q93" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">G_4_5_STUN</t>
+          <t>G_4_5_STUN</t>
         </is>
       </c>
       <c r="R93" s="39" t="inlineStr">
@@ -18937,7 +18937,7 @@
       </c>
       <c r="V93" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Stun</t>
+          <t>Stun</t>
         </is>
       </c>
       <c r="W93" s="39" t="inlineStr">
@@ -18955,7 +18955,7 @@
       </c>
       <c r="Z93" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">PulseInterval</t>
+          <t>PulseInterval</t>
         </is>
       </c>
       <c r="AA93" s="39" t="n">
@@ -18976,12 +18976,12 @@
       <c r="K94" s="43" t="n"/>
       <c r="Q94" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">G_4_5_RADIUS</t>
+          <t>G_4_5_RADIUS</t>
         </is>
       </c>
       <c r="R94" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">G_4_5</t>
+          <t>G_4_5</t>
         </is>
       </c>
       <c r="S94" s="39" t="n">
@@ -18989,7 +18989,7 @@
       </c>
       <c r="T94" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">OnEncounterTick</t>
+          <t>OnEncounterTick</t>
         </is>
       </c>
       <c r="U94" s="39" t="inlineStr">
@@ -19004,7 +19004,7 @@
       </c>
       <c r="W94" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Override</t>
+          <t>Override</t>
         </is>
       </c>
       <c r="X94" s="39" t="n">
@@ -19012,12 +19012,12 @@
       </c>
       <c r="Y94" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Card.EasterRandomStun</t>
+          <t>Card.EasterRandomStun</t>
         </is>
       </c>
       <c r="Z94" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">RadiusCm</t>
+          <t>RadiusCm</t>
         </is>
       </c>
       <c r="AA94" s="39" t="n">
@@ -19038,12 +19038,12 @@
       <c r="K95" s="43" t="n"/>
       <c r="Q95" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">G_4_5_COUNT</t>
+          <t>G_4_5_COUNT</t>
         </is>
       </c>
       <c r="R95" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">G_4_5</t>
+          <t>G_4_5</t>
         </is>
       </c>
       <c r="S95" s="39" t="n">
@@ -19051,7 +19051,7 @@
       </c>
       <c r="T95" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">OnEncounterTick</t>
+          <t>OnEncounterTick</t>
         </is>
       </c>
       <c r="U95" s="39" t="inlineStr">
@@ -19061,7 +19061,7 @@
       </c>
       <c r="V95" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Stun</t>
+          <t>Stun</t>
         </is>
       </c>
       <c r="W95" s="39" t="inlineStr">
@@ -19074,12 +19074,12 @@
       </c>
       <c r="Y95" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Card.EasterRandomStun</t>
+          <t>Card.EasterRandomStun</t>
         </is>
       </c>
       <c r="Z95" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">TargetCount</t>
+          <t>TargetCount</t>
         </is>
       </c>
       <c r="AA95" s="39" t="n">
@@ -19100,12 +19100,12 @@
       <c r="K96" s="43" t="n"/>
       <c r="Q96" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">G_4_6_REWARD</t>
+          <t>G_4_6_REWARD</t>
         </is>
       </c>
       <c r="R96" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">G_4_6</t>
+          <t>G_4_6</t>
         </is>
       </c>
       <c r="S96" s="39" t="n">
@@ -19113,7 +19113,7 @@
       </c>
       <c r="T96" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">OnEncounterEnd</t>
+          <t>OnEncounterEnd</t>
         </is>
       </c>
       <c r="U96" s="39" t="inlineStr">
@@ -19123,7 +19123,7 @@
       </c>
       <c r="V96" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">MinimumGuaranteedTier</t>
+          <t>MinimumGuaranteedTier</t>
         </is>
       </c>
       <c r="W96" s="39" t="inlineStr">
@@ -19136,12 +19136,12 @@
       </c>
       <c r="Y96" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Card.EasterDamageCards</t>
+          <t>Card.EasterDamageCards</t>
         </is>
       </c>
       <c r="Z96" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">GrantTier</t>
+          <t>GrantTier</t>
         </is>
       </c>
       <c r="AA96" s="39" t="n">
@@ -19162,7 +19162,7 @@
       <c r="K97" s="43" t="n"/>
       <c r="Q97" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">G_4_7_ZERO</t>
+          <t>G_4_7_ZERO</t>
         </is>
       </c>
       <c r="R97" s="39" t="inlineStr">
@@ -19224,7 +19224,7 @@
       <c r="K98" s="43" t="n"/>
       <c r="Q98" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">G_4_7_TEN</t>
+          <t>G_4_7_TEN</t>
         </is>
       </c>
       <c r="R98" s="39" t="inlineStr">
@@ -19286,7 +19286,7 @@
       <c r="K99" s="43" t="n"/>
       <c r="Q99" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">G_4_7_HUNDRED</t>
+          <t>G_4_7_HUNDRED</t>
         </is>
       </c>
       <c r="R99" s="39" t="inlineStr">
@@ -19348,12 +19348,12 @@
       <c r="K100" s="43" t="n"/>
       <c r="Q100" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">G_4_7_THOUSAND</t>
+          <t>G_4_7_THOUSAND</t>
         </is>
       </c>
       <c r="R100" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">G_4_7</t>
+          <t>G_4_7</t>
         </is>
       </c>
       <c r="S100" s="39" t="n">
@@ -19361,7 +19361,7 @@
       </c>
       <c r="T100" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">BeforeOutgoingHit</t>
+          <t>BeforeOutgoingHit</t>
         </is>
       </c>
       <c r="U100" s="39" t="inlineStr">
@@ -19371,12 +19371,12 @@
       </c>
       <c r="V100" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Damage</t>
+          <t>Damage</t>
         </is>
       </c>
       <c r="W100" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Override</t>
+          <t>Override</t>
         </is>
       </c>
       <c r="X100" s="39" t="n">
@@ -19384,12 +19384,12 @@
       </c>
       <c r="Y100" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Card.EasterPhysicalLottery</t>
+          <t>Card.EasterPhysicalLottery</t>
         </is>
       </c>
       <c r="Z100" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Probability</t>
+          <t>Probability</t>
         </is>
       </c>
       <c r="AA100" s="39" t="n">
@@ -19410,12 +19410,12 @@
       <c r="K101" s="43" t="n"/>
       <c r="Q101" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">G_4_7_TEN_THOUSAND</t>
+          <t>G_4_7_TEN_THOUSAND</t>
         </is>
       </c>
       <c r="R101" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">G_4_7</t>
+          <t>G_4_7</t>
         </is>
       </c>
       <c r="S101" s="39" t="n">
@@ -19423,7 +19423,7 @@
       </c>
       <c r="T101" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">BeforeOutgoingHit</t>
+          <t>BeforeOutgoingHit</t>
         </is>
       </c>
       <c r="U101" s="39" t="inlineStr">
@@ -19433,12 +19433,12 @@
       </c>
       <c r="V101" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Damage</t>
+          <t>Damage</t>
         </is>
       </c>
       <c r="W101" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Override</t>
+          <t>Override</t>
         </is>
       </c>
       <c r="X101" s="39" t="n">
@@ -19446,12 +19446,12 @@
       </c>
       <c r="Y101" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Card.EasterPhysicalLottery</t>
+          <t>Card.EasterPhysicalLottery</t>
         </is>
       </c>
       <c r="Z101" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Probability</t>
+          <t>Probability</t>
         </is>
       </c>
       <c r="AA101" s="39" t="n">
@@ -19472,12 +19472,12 @@
       <c r="K102" s="43" t="n"/>
       <c r="Q102" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">G_4_8_MORE</t>
+          <t>G_4_8_MORE</t>
         </is>
       </c>
       <c r="R102" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">G_4_8</t>
+          <t>G_4_8</t>
         </is>
       </c>
       <c r="S102" s="39" t="inlineStr">
@@ -19497,12 +19497,12 @@
       </c>
       <c r="V102" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">TimeShards</t>
+          <t>TimeShards</t>
         </is>
       </c>
       <c r="W102" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Multiply</t>
+          <t>Multiply</t>
         </is>
       </c>
       <c r="X102" s="39" t="n">
@@ -19510,12 +19510,12 @@
       </c>
       <c r="Y102" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Card.EasterShardComparison</t>
+          <t>Card.EasterShardComparison</t>
         </is>
       </c>
       <c r="Z102" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Step</t>
+          <t>Step</t>
         </is>
       </c>
       <c r="AA102" s="39" t="n">
@@ -19536,12 +19536,12 @@
       <c r="K103" s="43" t="n"/>
       <c r="Q103" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">G_4_8_LESS</t>
+          <t>G_4_8_LESS</t>
         </is>
       </c>
       <c r="R103" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">G_4_8</t>
+          <t>G_4_8</t>
         </is>
       </c>
       <c r="S103" s="39" t="inlineStr">
@@ -19561,12 +19561,12 @@
       </c>
       <c r="V103" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">TimeShards</t>
+          <t>TimeShards</t>
         </is>
       </c>
       <c r="W103" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Multiply</t>
+          <t>Multiply</t>
         </is>
       </c>
       <c r="X103" s="39" t="n">
@@ -19574,12 +19574,12 @@
       </c>
       <c r="Y103" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Card.EasterShardComparison</t>
+          <t>Card.EasterShardComparison</t>
         </is>
       </c>
       <c r="Z103" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Step</t>
+          <t>Step</t>
         </is>
       </c>
       <c r="AA103" s="39" t="n">
@@ -19589,7 +19589,7 @@
     <row r="104" ht="26" customHeight="1" s="41">
       <c r="Q104" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">G_4_9_HP</t>
+          <t>G_4_9_HP</t>
         </is>
       </c>
       <c r="R104" s="39" t="inlineStr">
@@ -19612,7 +19612,7 @@
       </c>
       <c r="V104" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">HpMaxAndPoint</t>
+          <t>HpMaxAndPoint</t>
         </is>
       </c>
       <c r="W104" s="39" t="inlineStr">
@@ -19630,7 +19630,7 @@
       </c>
       <c r="Z104" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Max</t>
+          <t>Max</t>
         </is>
       </c>
       <c r="AA104" s="39" t="n">
@@ -19640,12 +19640,12 @@
     <row r="105" ht="26" customHeight="1" s="41">
       <c r="Q105" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">G_4_9_ELEMENTAL</t>
+          <t>G_4_9_ELEMENTAL</t>
         </is>
       </c>
       <c r="R105" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">G_4_9</t>
+          <t>G_4_9</t>
         </is>
       </c>
       <c r="S105" s="39" t="n">
@@ -19653,22 +19653,22 @@
       </c>
       <c r="T105" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">OnEncounterEnd</t>
+          <t>OnEncounterEnd</t>
         </is>
       </c>
       <c r="U105" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">CardBehavior</t>
+          <t>CardBehavior</t>
         </is>
       </c>
       <c r="V105" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">ElementalAttack</t>
+          <t>ElementalAttack</t>
         </is>
       </c>
       <c r="W105" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Add</t>
+          <t>Add</t>
         </is>
       </c>
       <c r="X105" s="39" t="n">
@@ -19676,12 +19676,12 @@
       </c>
       <c r="Y105" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Card.EasterAttendance</t>
+          <t>Card.EasterAttendance</t>
         </is>
       </c>
       <c r="Z105" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Max</t>
+          <t>Max</t>
         </is>
       </c>
       <c r="AA105" s="39" t="n">
@@ -19691,12 +19691,12 @@
     <row r="106" ht="26" customHeight="1" s="41">
       <c r="Q106" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">G_4_9_PHYSICAL</t>
+          <t>G_4_9_PHYSICAL</t>
         </is>
       </c>
       <c r="R106" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">G_4_9</t>
+          <t>G_4_9</t>
         </is>
       </c>
       <c r="S106" s="39" t="n">
@@ -19704,22 +19704,22 @@
       </c>
       <c r="T106" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">OnEncounterEnd</t>
+          <t>OnEncounterEnd</t>
         </is>
       </c>
       <c r="U106" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">CardBehavior</t>
+          <t>CardBehavior</t>
         </is>
       </c>
       <c r="V106" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">PhysicalAttack</t>
+          <t>PhysicalAttack</t>
         </is>
       </c>
       <c r="W106" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Add</t>
+          <t>Add</t>
         </is>
       </c>
       <c r="X106" s="39" t="n">
@@ -19727,12 +19727,12 @@
       </c>
       <c r="Y106" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Card.EasterAttendance</t>
+          <t>Card.EasterAttendance</t>
         </is>
       </c>
       <c r="Z106" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Max</t>
+          <t>Max</t>
         </is>
       </c>
       <c r="AA106" s="39" t="n">
@@ -20205,8 +20205,8 @@
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="2">
-    <tablePart r:id="rId1"/>
-    <tablePart r:id="rId2"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
   </tableParts>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
[PROGRAMMER] fix easter card reward chains
</commit_message>
<xml_diff>
--- a/Design/Data/ReEchoData.xlsx
+++ b/Design/Data/ReEchoData.xlsx
@@ -17410,7 +17410,7 @@
       </c>
       <c r="E74" s="39" t="inlineStr">
         <is>
-          <t>你努力奔跑。下一关，1滴血换1张1级卡牌
+          <t>下一关卡结束后，你获得X张随机1级卡牌。X=你下一关卡受到的伤害
 ——特别鸣谢 程序 Jo爷</t>
         </is>
       </c>
@@ -19141,11 +19141,13 @@
       </c>
       <c r="Z96" s="39" t="inlineStr">
         <is>
-          <t>GrantTier</t>
-        </is>
-      </c>
-      <c r="AA96" s="39" t="n">
-        <v>1</v>
+          <t>DamageToCards</t>
+        </is>
+      </c>
+      <c r="AA96" s="39" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
     </row>
     <row r="97" ht="22" customHeight="1" s="41">

</xml_diff>

<commit_message>
[PROGRAMMER] fix easter text and inspiration crash
</commit_message>
<xml_diff>
--- a/Design/Data/ReEchoData.xlsx
+++ b/Design/Data/ReEchoData.xlsx
@@ -16810,7 +16810,7 @@
       </c>
       <c r="E69" s="39" t="inlineStr">
         <is>
-          <t>每关结束后，赌一把大的！攒够了家底以后，商店刷新永远为你开放！
+          <t>每关结束后，赌一把大的！攒够了家底以后，获得来自程序邱孙红的宝库。
 ——策划 爆培嘉 敬上</t>
         </is>
       </c>
@@ -17050,7 +17050,7 @@
       </c>
       <c r="E71" s="39" t="inlineStr">
         <is>
-          <t>回响触碰到敌人，造成20物理伤害；如果是你，你回复10生命值。数值每关翻倍！
+          <t>回响触碰到敌人，造成1000物理伤害；如果是你，你回复1000生命值。数值每关翻倍！
 ——策划 麦麦熊 敬上</t>
         </is>
       </c>
@@ -17170,7 +17170,7 @@
       </c>
       <c r="E72" s="39" t="inlineStr">
         <is>
-          <t>失去所有时间碎片。每失去15时间碎片，随机获得一些属性！
+          <t>用更高的效率把所有的时间碎片转化为随机属性。你觉得这个怎么样？
 ——策划 呕乐兮 敬上</t>
         </is>
       </c>
@@ -17290,7 +17290,7 @@
       </c>
       <c r="E73" s="39" t="inlineStr">
         <is>
-          <t>身边的敌人都被你迷倒了！
+          <t>身边的所有敌人都被你彻彻底底迷晕了，迷倒了！
 ——特别鸣谢 程序 T爷</t>
         </is>
       </c>
@@ -17410,7 +17410,7 @@
       </c>
       <c r="E74" s="39" t="inlineStr">
         <is>
-          <t>下一关卡结束后，你获得X张随机1级卡牌。X=你下一关卡受到的伤害
+          <t>“野狗不需要墓碑”，你快要飞升成神了。下一关，1滴血换10张1级卡牌
 ——特别鸣谢 程序 Jo爷</t>
         </is>
       </c>
@@ -17530,7 +17530,7 @@
       </c>
       <c r="E75" s="39" t="inlineStr">
         <is>
-          <t>神秘人往你的物理伤害后面加随机个0
+          <t>往你的物理伤害后面加随机个、很多个、真的很多0！
 ——特别鸣谢 美术 00</t>
         </is>
       </c>
@@ -17650,7 +17650,7 @@
       </c>
       <c r="E76" s="39" t="inlineStr">
         <is>
-          <t>经济系统被赋予“ELO”机制
+          <t>经济系统被赋予被彻底魔改的“ELO”机制
 ——特别鸣谢 美术 子涵</t>
         </is>
       </c>
@@ -17770,7 +17770,7 @@
       </c>
       <c r="E77" s="39" t="inlineStr">
         <is>
-          <t>每一关卡结束后，随机获得巨额生命值/元攻/物攻
+          <t>每一关卡结束后，随机获得巨额生命值/元攻/物攻（真的是巨额！）
 ——特别鸣谢 美术 雯雯</t>
         </is>
       </c>

</xml_diff>